<commit_message>
📊 Weekly RSI Screener Report – 2026-05-02
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1048.35</v>
+        <v>299.55</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>68.18000000000001</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>69.01000000000001</v>
+        <v>73.06</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>71.98</v>
+        <v>69.3</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>26.68</v>
+        <v>25.73</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>879.58</v>
+        <v>258.23</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>850.54</v>
+        <v>253.83</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>6768928</v>
+        <v>21860914</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>234427</v>
+        <v>375899</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,31 +585,31 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>401.85</v>
+        <v>481.45</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>65.70999999999999</v>
+        <v>68.81</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>68.56999999999999</v>
+        <v>67.89</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>68.65000000000001</v>
+        <v>71.64</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>37.43</v>
+        <v>28.06</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>355.97</v>
+        <v>417.39</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>351.69</v>
+        <v>410.04</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>13965303</v>
+        <v>13716832</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>389661</v>
+        <v>296797</v>
       </c>
     </row>
     <row r="4">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>316.4</v>
+        <v>318.35</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>65.33</v>
+        <v>63.44</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>67.02</v>
+        <v>68</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>62.65</v>
+        <v>63</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>32.46</v>
+        <v>25.22</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>286.09</v>
+        <v>287.86</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>284.71</v>
+        <v>286.23</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>15917825</v>
+        <v>14990049</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>294271</v>
+        <v>296689</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>210.07</v>
+        <v>1038</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>60.01</v>
+        <v>60.05</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>62.9</v>
+        <v>67.11</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>65.88</v>
+        <v>71.59</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>56.11</v>
+        <v>25.44</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>186.76</v>
+        <v>888.97</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>181.88</v>
+        <v>858.8</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>31612445</v>
+        <v>6630097</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>261996</v>
+        <v>231889</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>456</v>
+        <v>1264.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>57.77</v>
+        <v>59.13</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>62.34</v>
+        <v>60.52</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>68.7</v>
+        <v>65.34</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>29.79</v>
+        <v>37.66</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>414.47</v>
+        <v>1170.1</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>407.52</v>
+        <v>1149.55</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>13707759</v>
+        <v>2251234</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>281020</v>
+        <v>308228</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,37 +741,37 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>284.8</v>
+        <v>399.15</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>57.07</v>
+        <v>58.37</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>67.69</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>66.56</v>
+        <v>68.26000000000001</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>30.92</v>
+        <v>30.65</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>256.09</v>
+        <v>358.5</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>252.05</v>
+        <v>353.87</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>20869156</v>
+        <v>12917354</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>358286</v>
+        <v>387770</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -780,31 +780,31 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1101.1</v>
+        <v>211.36</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>56.02</v>
+        <v>57.74</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>60.01</v>
+        <v>63.51</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>65.04000000000001</v>
+        <v>66.14</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>72.3</v>
+        <v>41.45</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1014.15</v>
+        <v>188.18</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>984.42</v>
+        <v>183.15</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>18057938</v>
+        <v>31566640</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1016383</v>
+        <v>263655</v>
       </c>
     </row>
     <row r="9">
@@ -819,31 +819,31 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>4410</v>
+        <v>4385.2</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>55.53</v>
+        <v>52.64</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>62.41</v>
+        <v>61.42</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>63.39</v>
+        <v>63.12</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>44.59</v>
+        <v>51.89</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>4015.88</v>
+        <v>4036.85</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>3932.88</v>
+        <v>3951.72</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>1206041</v>
+        <v>1194655</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>391187</v>
+        <v>389235</v>
       </c>
     </row>
   </sheetData>
@@ -922,16 +922,16 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1421.3</v>
+        <v>1458.6</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>79.25</v>
+        <v>79.62</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>71.52</v>
+        <v>74.33</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>62.84</v>
+        <v>64.25</v>
       </c>
     </row>
     <row r="3">
@@ -946,22 +946,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>2287.6</v>
+        <v>2408.4</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>69.89</v>
+        <v>74.44</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>55.39</v>
+        <v>59.63</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>48.33</v>
+        <v>50.29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -970,22 +970,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1174</v>
+        <v>1657.3</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>69.23999999999999</v>
+        <v>71.88</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>57.78</v>
+        <v>66</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>57.41</v>
+        <v>63.08</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -994,22 +994,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1048.35</v>
+        <v>299.55</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>68.18000000000001</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>69.01000000000001</v>
+        <v>73.06</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>71.98</v>
+        <v>69.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1018,22 +1018,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>401.85</v>
+        <v>481.45</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>65.70999999999999</v>
+        <v>68.81</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>68.56999999999999</v>
+        <v>67.89</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>68.65000000000001</v>
+        <v>71.64</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1042,22 +1042,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1585.1</v>
+        <v>318.35</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>65.67</v>
+        <v>63.44</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>61.01</v>
+        <v>68</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>61.1</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1066,22 +1066,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>316.4</v>
+        <v>916.05</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>65.33</v>
+        <v>63.2</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>67.02</v>
+        <v>58.19</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>62.65</v>
+        <v>47.41</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1090,22 +1090,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>4297.3</v>
+        <v>1808.3</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>64.8</v>
+        <v>63.06</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>53.57</v>
+        <v>58.29</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>48.81</v>
+        <v>59.06</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1114,22 +1114,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>2327.3</v>
+        <v>9994</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>63.76</v>
+        <v>62.93</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>52.51</v>
+        <v>61.14</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>49</v>
+        <v>62.12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1138,22 +1138,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1317.1</v>
+        <v>1430.8</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>61.94</v>
+        <v>61.66</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>57.85</v>
+        <v>52.63</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>57.55</v>
+        <v>53.44</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1162,22 +1162,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1365.9</v>
+        <v>314.9</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>61.51</v>
+        <v>60.95</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>61.48</v>
+        <v>41.31</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>60.31</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1186,22 +1186,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>2485.1</v>
+        <v>1309.6</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>60.98</v>
+        <v>60.91</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>51.8</v>
+        <v>42.23</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>48.36</v>
+        <v>45.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1210,22 +1210,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1295</v>
+        <v>1038</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>60.59</v>
+        <v>60.05</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>40.61</v>
+        <v>67.11</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>44.29</v>
+        <v>71.59</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1234,22 +1234,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1255.7</v>
+        <v>1322.9</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>60.13</v>
+        <v>59.53</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>59.85</v>
+        <v>58.72</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>64.95999999999999</v>
+        <v>57.88</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1258,22 +1258,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>210.07</v>
+        <v>1264.5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>60.01</v>
+        <v>59.13</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>62.9</v>
+        <v>60.52</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>65.88</v>
+        <v>65.34</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1282,22 +1282,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>7732.5</v>
+        <v>399.15</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>57.93</v>
+        <v>58.37</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>57.03</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>60.5</v>
+        <v>68.26000000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1306,22 +1306,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>456</v>
+        <v>2794.5</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>57.77</v>
+        <v>58.21</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>62.34</v>
+        <v>53.69</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>68.7</v>
+        <v>57.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1330,22 +1330,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>11998</v>
+        <v>1886.8</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>57.3</v>
+        <v>57.89</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>52.09</v>
+        <v>47.68</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>55.74</v>
+        <v>60.39</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1354,22 +1354,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>284.8</v>
+        <v>937</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>57.07</v>
+        <v>57.75</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>67.69</v>
+        <v>50.31</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>66.56</v>
+        <v>55.21</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1378,22 +1378,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1101.1</v>
+        <v>211.36</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>56.02</v>
+        <v>57.74</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>60.01</v>
+        <v>63.51</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>65.04000000000001</v>
+        <v>66.14</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1402,22 +1402,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>4014.3</v>
+        <v>1144.6</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>55.99</v>
+        <v>56.58</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>53.88</v>
+        <v>53.74</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>58.1</v>
+        <v>55.81</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1426,22 +1426,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>350.5</v>
+        <v>4144.6</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>55.79</v>
+        <v>56.21</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>48.41</v>
+        <v>50.35</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v/>
+        <v>47.58</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1450,22 +1450,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>4410</v>
+        <v>2444.5</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>55.53</v>
+        <v>55.91</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>62.41</v>
+        <v>49.97</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>63.39</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1474,22 +1474,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>921.55</v>
+        <v>1473.5</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>54.14</v>
+        <v>55.19</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>48.15</v>
+        <v>49.84</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>54.41</v>
+        <v>52.03</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1498,22 +1498,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>9576</v>
+        <v>383.3</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>53.22</v>
+        <v>54.24</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>55.16</v>
+        <v>44.28</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>59.77</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1522,22 +1522,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>2739.3</v>
+        <v>4014</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>53.07</v>
+        <v>54.22</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>50.35</v>
+        <v>54.06</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>56.01</v>
+        <v>58.09</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1546,22 +1546,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>444.45</v>
+        <v>4385.2</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>52.63</v>
+        <v>52.64</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>56.61</v>
+        <v>61.42</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>66.34999999999999</v>
+        <v>63.12</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1570,22 +1570,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>5730.5</v>
+        <v>2250.9</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>52.16</v>
+        <v>52.2</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>48.16</v>
+        <v>47.76</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>55.04</v>
+        <v>46.74</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1594,22 +1594,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1011.3</v>
+        <v>5726</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>52.03</v>
+        <v>52.01</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>59.95</v>
+        <v>48.11</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>66.51000000000001</v>
+        <v>54.98</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1618,22 +1618,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1326.2</v>
+        <v>7636.5</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>51.74</v>
+        <v>51.57</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>48.48</v>
+        <v>54.9</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>55.26</v>
+        <v>59.68</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1642,16 +1642,16 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>847.95</v>
+        <v>13314</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>51.61</v>
+        <v>50.71</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>49.5</v>
+        <v>42.37</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>44.11</v>
+        <v>51.85</v>
       </c>
     </row>
     <row r="33">
@@ -1666,22 +1666,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>7111.5</v>
+        <v>7109</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>49.87</v>
+        <v>49.61</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>50.91</v>
+        <v>50.89</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>63.12</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1690,22 +1690,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>308.1</v>
+        <v>341.55</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>49.55</v>
+        <v>48.87</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>44.51</v>
+        <v>45.91</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>52.95</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1714,22 +1714,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>301.6</v>
+        <v>200.65</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>47.35</v>
+        <v>48.03</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>33.15</v>
+        <v>38.06</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>35.51</v>
+        <v>41.83</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1738,22 +1738,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>199.36</v>
+        <v>11586</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>46.21</v>
+        <v>47.45</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>36.57</v>
+        <v>47.61</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>41.43</v>
+        <v>53.43</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1762,22 +1762,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1770.7</v>
+        <v>1068.45</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>46.1</v>
+        <v>46.64</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>41.07</v>
+        <v>55.63</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>47.97</v>
+        <v>63.68</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1786,22 +1786,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>370.85</v>
+        <v>3097.5</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>45.07</v>
+        <v>46.45</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>38.25</v>
+        <v>42.53</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>46.49</v>
+        <v>55.34</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1810,22 +1810,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>13048</v>
+        <v>2473.9</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>44.48</v>
+        <v>46.11</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>39.7</v>
+        <v>35.47</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>50.74</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1834,22 +1834,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>784.85</v>
+        <v>5099</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>44.45</v>
+        <v>45.49</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>32.33</v>
+        <v>46.44</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>42.09</v>
+        <v>56.35</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1858,22 +1858,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1327.8</v>
+        <v>431.3</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>42.69</v>
+        <v>44.43</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>39.43</v>
+        <v>52.75</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>47.61</v>
+        <v>65.06999999999999</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1882,22 +1882,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1814.5</v>
+        <v>300.45</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>42.45</v>
+        <v>44.12</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>40.21</v>
+        <v>42.89</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>57.5</v>
+        <v>51.83</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1906,22 +1906,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>3038.4</v>
+        <v>1747.2</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>42</v>
+        <v>42.87</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>40.36</v>
+        <v>39.49</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>54.15</v>
+        <v>47.11</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1930,22 +1930,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>4961.5</v>
+        <v>1268.3</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>39.42</v>
+        <v>42.22</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>43.36</v>
+        <v>50.64</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>54.62</v>
+        <v>56.31</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1954,22 +1954,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>588.2</v>
+        <v>1819</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>38.75</v>
+        <v>41.48</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>32.01</v>
+        <v>43.8</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>40.04</v>
+        <v>55.11</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1978,22 +1978,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>2396.9</v>
+        <v>771.7</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>37.83</v>
+        <v>41.2</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>30.3</v>
+        <v>31.16</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>33.42</v>
+        <v>40.76</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -2002,22 +2002,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1358.5</v>
+        <v>937.35</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>36.9</v>
+        <v>40.7</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>40.79</v>
+        <v>51.33</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>47.81</v>
+        <v>63.88</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -2026,22 +2026,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1768.9</v>
+        <v>1263.4</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>33.67</v>
+        <v>40.28</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>39.99</v>
+        <v>42.08</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>52.98</v>
+        <v>51.04</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2050,16 +2050,16 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>1620.4</v>
+        <v>586.9</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>33.33</v>
+        <v>39.94</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>40.83</v>
+        <v>32.22</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>51.27</v>
+        <v>39.94</v>
       </c>
     </row>
     <row r="50">
@@ -2074,16 +2074,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1154.6</v>
+        <v>1181.8</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>27.38</v>
+        <v>35.91</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>29.09</v>
+        <v>32.22</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>36.23</v>
+        <v>37.03</v>
       </c>
     </row>
     <row r="51">
@@ -2098,16 +2098,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1203.2</v>
+        <v>1199.1</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>27.18</v>
+        <v>30.08</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>30.88</v>
+        <v>32.06</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>41.39</v>
+        <v>40.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-05-09
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>299.55</v>
+        <v>1760.4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>69.45999999999999</v>
+        <v>75.03</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>73.06</v>
+        <v>69.95</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>69.3</v>
+        <v>65.75</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>25.73</v>
+        <v>26.31</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>258.23</v>
+        <v>1478.23</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>253.83</v>
+        <v>1457.9</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>21860914</v>
+        <v>3658101</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>375899</v>
+        <v>405589</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>481.45</v>
+        <v>10711.5</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>68.81</v>
+        <v>73.83</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>67.89</v>
+        <v>67.87</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>71.64</v>
+        <v>65.81999999999999</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>28.06</v>
+        <v>26.73</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>417.39</v>
+        <v>9340.35</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>410.04</v>
+        <v>9238.02</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>13716832</v>
+        <v>432598</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>296797</v>
+        <v>299142</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>318.35</v>
+        <v>8097</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>63.44</v>
+        <v>69.34</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>68</v>
+        <v>62.86</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>63</v>
+        <v>63.57</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>25.22</v>
+        <v>40.31</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>287.86</v>
+        <v>7447.16</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>286.23</v>
+        <v>7391.61</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>14990049</v>
+        <v>415748</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>296689</v>
+        <v>116422</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,31 +663,31 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1038</v>
+        <v>4509</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>60.05</v>
+        <v>60.36</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>67.11</v>
+        <v>64.69</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>71.59</v>
+        <v>64.56</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>25.44</v>
+        <v>43.03</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>888.97</v>
+        <v>4063.11</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>858.8</v>
+        <v>3974.77</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>6630097</v>
+        <v>1300090</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>231889</v>
+        <v>399969</v>
       </c>
     </row>
     <row r="6">
@@ -702,31 +702,31 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1264.5</v>
+        <v>1277.8</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>59.13</v>
+        <v>60.11</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>60.52</v>
+        <v>61.93</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>65.34</v>
+        <v>65.95</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>37.66</v>
+        <v>26.99</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1170.1</v>
+        <v>1177.73</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1149.55</v>
+        <v>1156.38</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2251234</v>
+        <v>2005817</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>308228</v>
+        <v>311864</v>
       </c>
     </row>
     <row r="7">
@@ -741,31 +741,31 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>399.15</v>
+        <v>402.15</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>58.37</v>
+        <v>59.54</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>67.40000000000001</v>
+        <v>67.86</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>68.26000000000001</v>
+        <v>68.73</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>30.65</v>
+        <v>35.53</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>358.5</v>
+        <v>361.62</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>353.87</v>
+        <v>356.42</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>12917354</v>
+        <v>11478817</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>387770</v>
+        <v>389951</v>
       </c>
     </row>
     <row r="8">
@@ -780,70 +780,31 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>211.36</v>
+        <v>214.49</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>57.74</v>
+        <v>59.36</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>63.51</v>
+        <v>64.95</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>66.14</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>41.45</v>
+        <v>25.73</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>188.18</v>
+        <v>190.14</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>183.15</v>
+        <v>184.92</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>31566640</v>
+        <v>27390784</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>263655</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TITAN</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>4385.2</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>52.64</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>61.42</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>63.12</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>51.89</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>4036.85</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>3951.72</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>1194655</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>389235</v>
+        <v>267509</v>
       </c>
     </row>
   </sheetData>
@@ -855,7 +816,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -922,22 +882,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1458.6</v>
+        <v>1482.4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>79.62</v>
+        <v>78.51000000000001</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>74.33</v>
+        <v>75.5</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>64.25</v>
+        <v>65.16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -946,22 +906,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>2408.4</v>
+        <v>1760.4</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>74.44</v>
+        <v>75.03</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>59.63</v>
+        <v>69.95</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>50.29</v>
+        <v>65.75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -970,22 +930,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1657.3</v>
+        <v>10711.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>71.88</v>
+        <v>73.83</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>66</v>
+        <v>67.87</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>63.08</v>
+        <v>65.81999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -994,22 +954,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>299.55</v>
+        <v>2968.6</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>69.45999999999999</v>
+        <v>73.28</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>73.06</v>
+        <v>62.38</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>69.3</v>
+        <v>61.53</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1018,22 +978,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>481.45</v>
+        <v>2505.9</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>68.81</v>
+        <v>73.18000000000001</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>67.89</v>
+        <v>62.61</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>71.64</v>
+        <v>51.87</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1042,22 +1002,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>318.35</v>
+        <v>2599.9</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>63.44</v>
+        <v>69.59</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>68</v>
+        <v>56.92</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>63</v>
+        <v>50.86</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1066,22 +1026,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>916.05</v>
+        <v>8097</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>63.2</v>
+        <v>69.34</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>58.19</v>
+        <v>62.86</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>47.41</v>
+        <v>63.57</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1090,22 +1050,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1808.3</v>
+        <v>950.75</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>63.06</v>
+        <v>68.56999999999999</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>58.29</v>
+        <v>61.28</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>59.06</v>
+        <v>49.06</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1114,22 +1074,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>9994</v>
+        <v>1847.9</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>62.93</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>61.14</v>
+        <v>60.79</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>62.12</v>
+        <v>60.44</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1138,22 +1098,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1430.8</v>
+        <v>1347</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>61.66</v>
+        <v>64.37</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>52.63</v>
+        <v>48.52</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>53.44</v>
+        <v>47.56</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1162,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>314.9</v>
+        <v>1176.2</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>60.95</v>
+        <v>63.37</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>41.31</v>
+        <v>57.14</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>38.8</v>
+        <v>57.65</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1186,22 +1146,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1309.6</v>
+        <v>4509</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>60.91</v>
+        <v>60.36</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>42.23</v>
+        <v>64.69</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>45.2</v>
+        <v>64.56</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1210,22 +1170,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1038</v>
+        <v>1277.8</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>60.05</v>
+        <v>60.11</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>67.11</v>
+        <v>61.93</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>71.59</v>
+        <v>65.95</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1234,22 +1194,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1322.9</v>
+        <v>3330.4</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>59.53</v>
+        <v>59.81</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>58.72</v>
+        <v>50.68</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>57.88</v>
+        <v>59.79</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1258,22 +1218,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1264.5</v>
+        <v>402.15</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>59.13</v>
+        <v>59.54</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>60.52</v>
+        <v>67.86</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>65.34</v>
+        <v>68.73</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1282,22 +1242,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>399.15</v>
+        <v>214.49</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>58.37</v>
+        <v>59.36</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>67.40000000000001</v>
+        <v>64.95</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>68.26000000000001</v>
+        <v>66.81999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1306,22 +1266,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2794.5</v>
+        <v>1435.2</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>58.21</v>
+        <v>59.02</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>53.69</v>
+        <v>52.58</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>57.4</v>
+        <v>53.68</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1330,22 +1290,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1886.8</v>
+        <v>4242.3</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>57.89</v>
+        <v>58.97</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>47.68</v>
+        <v>52.3</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>60.39</v>
+        <v>48.44</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1354,22 +1314,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>937</v>
+        <v>1044.4</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>57.75</v>
+        <v>58.66</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>50.31</v>
+        <v>67.81</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>55.21</v>
+        <v>71.84999999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1378,22 +1338,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>211.36</v>
+        <v>955.35</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>57.74</v>
+        <v>58.15</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>63.51</v>
+        <v>52.19</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>66.14</v>
+        <v>56.19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1402,22 +1362,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1144.6</v>
+        <v>13726</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>56.58</v>
+        <v>57.34</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>53.74</v>
+        <v>46.21</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>55.81</v>
+        <v>53.58</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1426,22 +1386,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>4144.6</v>
+        <v>355.45</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>56.21</v>
+        <v>56.28</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>50.35</v>
+        <v>50.37</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>47.58</v>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1450,22 +1410,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>2444.5</v>
+        <v>5322</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>55.91</v>
+        <v>56.27</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>49.97</v>
+        <v>50.59</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>47.5</v>
+        <v>58.74</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1474,22 +1434,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1473.5</v>
+        <v>621.7</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>55.19</v>
+        <v>55.32</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>49.84</v>
+        <v>40.49</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>52.03</v>
+        <v>44.03</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1498,22 +1458,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>383.3</v>
+        <v>7302.5</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>54.24</v>
+        <v>55.15</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>44.28</v>
+        <v>53.77</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>48.8</v>
+        <v>64.44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1522,22 +1482,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>4014</v>
+        <v>1818.3</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>54.22</v>
+        <v>54.42</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>54.06</v>
+        <v>45.36</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>58.09</v>
+        <v>49.82</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1546,16 +1506,16 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>4385.2</v>
+        <v>11950</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>52.64</v>
+        <v>54.29</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>61.42</v>
+        <v>51.56</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>63.12</v>
+        <v>55.63</v>
       </c>
     </row>
     <row r="29">
@@ -1570,22 +1530,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>2250.9</v>
+        <v>2287.7</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>52.2</v>
+        <v>54.28</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>47.76</v>
+        <v>50.01</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>46.74</v>
+        <v>47.93</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1594,22 +1554,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>5726</v>
+        <v>1007.75</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>52.01</v>
+        <v>54.24</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>48.11</v>
+        <v>57.55</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>54.98</v>
+        <v>66.58</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1618,22 +1578,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>7636.5</v>
+        <v>313.95</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>51.57</v>
+        <v>53.88</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>54.9</v>
+        <v>64.26000000000001</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>59.68</v>
+        <v>61.6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1642,22 +1602,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>13314</v>
+        <v>1463</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>50.71</v>
+        <v>52.89</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>42.37</v>
+        <v>49.08</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>51.85</v>
+        <v>51.61</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1666,22 +1626,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>7109</v>
+        <v>380.8</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>49.61</v>
+        <v>52.67</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>50.89</v>
+        <v>43.21</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>63.1</v>
+        <v>48.35</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1690,22 +1650,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>341.55</v>
+        <v>1293.9</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>48.87</v>
+        <v>52.21</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>45.91</v>
+        <v>54.03</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v/>
+        <v>55.55</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1714,22 +1674,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>200.65</v>
+        <v>439.7</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>48.03</v>
+        <v>51.56</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>38.06</v>
+        <v>54.81</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>41.83</v>
+        <v>65.95999999999999</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1738,22 +1698,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>11586</v>
+        <v>1872.1</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>47.45</v>
+        <v>50.93</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>47.61</v>
+        <v>47.46</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>53.43</v>
+        <v>57.29</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1762,22 +1722,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1068.45</v>
+        <v>307.45</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>46.64</v>
+        <v>50.48</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>55.63</v>
+        <v>38.38</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>63.68</v>
+        <v>37.64</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1786,22 +1746,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>3097.5</v>
+        <v>3974.5</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>46.45</v>
+        <v>50.09</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>42.53</v>
+        <v>52.63</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>55.34</v>
+        <v>57.28</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1810,22 +1770,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>2473.9</v>
+        <v>456.4</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>46.11</v>
+        <v>48.61</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>35.47</v>
+        <v>58.73</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>35.5</v>
+        <v>65.15000000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1834,22 +1794,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>5099</v>
+        <v>1834.5</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>45.49</v>
+        <v>47.74</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>46.44</v>
+        <v>43.31</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>56.35</v>
+        <v>57.35</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1858,22 +1818,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>431.3</v>
+        <v>302.75</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>44.43</v>
+        <v>47.04</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>52.75</v>
+        <v>43.38</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>65.06999999999999</v>
+        <v>52.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1882,22 +1842,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>300.45</v>
+        <v>780.85</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>44.12</v>
+        <v>45.71</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>42.89</v>
+        <v>33.16</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>51.83</v>
+        <v>41.77</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1906,16 +1866,16 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1747.2</v>
+        <v>197.91</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>42.87</v>
+        <v>43.94</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>39.49</v>
+        <v>36.25</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>47.11</v>
+        <v>41.19</v>
       </c>
     </row>
     <row r="44">
@@ -1933,10 +1893,10 @@
         <v>1268.3</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>42.22</v>
+        <v>43.82</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>50.64</v>
+        <v>49.94</v>
       </c>
       <c r="F44" s="4" t="n">
         <v>56.31</v>
@@ -1945,7 +1905,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1954,22 +1914,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1819</v>
+        <v>279.2</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>41.48</v>
+        <v>43.03</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>43.8</v>
+        <v>58.27</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>55.11</v>
+        <v>61.79</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1978,22 +1938,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>771.7</v>
+        <v>1264.8</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>41.2</v>
+        <v>42.79</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>31.16</v>
+        <v>42.06</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>40.76</v>
+        <v>51.15</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -2002,22 +1962,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>937.35</v>
+        <v>5520</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>40.7</v>
+        <v>40.15</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>51.33</v>
+        <v>41.51</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>63.88</v>
+        <v>51.81</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -2026,22 +1986,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1263.4</v>
+        <v>1179.2</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>40.28</v>
+        <v>38.87</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>42.08</v>
+        <v>31.99</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>51.04</v>
+        <v>36.95</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2050,22 +2010,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>586.9</v>
+        <v>2394.4</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>39.94</v>
+        <v>38.59</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>32.22</v>
+        <v>32.74</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>39.94</v>
+        <v>34.31</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2074,16 +2034,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1181.8</v>
+        <v>1019.3</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>35.91</v>
+        <v>37.49</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>32.22</v>
+        <v>48.74</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>37.03</v>
+        <v>59.92</v>
       </c>
     </row>
     <row r="51">
@@ -2098,16 +2058,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1199.1</v>
+        <v>1198.4</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>30.08</v>
+        <v>32.83</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>32.06</v>
+        <v>31.79</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>40.57</v>
+        <v>41.59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-05-16
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1760.4</v>
+        <v>1795.1</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.03</v>
+        <v>69.59</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>69.95</v>
+        <v>71.39</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>65.75</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>26.31</v>
+        <v>26.81</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1478.23</v>
+        <v>1496.01</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1457.9</v>
+        <v>1472.69</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>3658101</v>
+        <v>3826358</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>405589</v>
+        <v>413584</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>10711.5</v>
+        <v>8082.5</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>73.83</v>
+        <v>64.97</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>67.87</v>
+        <v>62.47</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>65.81999999999999</v>
+        <v>63.46</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>26.73</v>
+        <v>22.9</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>9340.35</v>
+        <v>7486.84</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>9238.02</v>
+        <v>7424.34</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>432598</v>
+        <v>378971</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>299142</v>
+        <v>116214</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>8097</v>
+        <v>299.35</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>69.34</v>
+        <v>60.94</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>62.86</v>
+        <v>65.76000000000001</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>63.57</v>
+        <v>69.22</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>40.31</v>
+        <v>28.54</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>7447.16</v>
+        <v>262.68</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7391.61</v>
+        <v>257.64</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>415748</v>
+        <v>18759890</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>116422</v>
+        <v>376591</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>4509</v>
+        <v>216.84</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>60.36</v>
+        <v>58.21</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>64.69</v>
+        <v>66.04000000000001</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>64.56</v>
+        <v>67.31999999999999</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>43.03</v>
+        <v>23.45</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>4063.11</v>
+        <v>191.83</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>3974.77</v>
+        <v>186.45</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>1300090</v>
+        <v>26436259</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>399969</v>
+        <v>270440</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1277.8</v>
+        <v>1430.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>60.11</v>
+        <v>58.05</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>61.93</v>
+        <v>66.61</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>65.95</v>
+        <v>62.33</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>26.99</v>
+        <v>34.05</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1177.73</v>
+        <v>1286.58</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1156.38</v>
+        <v>1269.13</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2005817</v>
+        <v>2302030</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>311864</v>
+        <v>275845</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,37 +741,37 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>402.15</v>
+        <v>1278.8</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>59.54</v>
+        <v>56.83</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>67.86</v>
+        <v>62.03</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>68.73</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>35.53</v>
+        <v>29.53</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>361.62</v>
+        <v>1183.9</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>356.42</v>
+        <v>1162.13</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>11478817</v>
+        <v>2070783</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>389951</v>
+        <v>312108</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -780,31 +780,70 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>214.49</v>
+        <v>462.2</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>59.36</v>
+        <v>52.11</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>64.95</v>
+        <v>60.07</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>66.81999999999999</v>
+        <v>66.54000000000001</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>25.73</v>
+        <v>32.74</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>190.14</v>
+        <v>424.09</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>184.92</v>
+        <v>416</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>27390784</v>
+        <v>12114342</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>267509</v>
+        <v>284841</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>395.25</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>52.04</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>63.57</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>66.95</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>50.79</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>363.68</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>358.27</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>10640064</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>383261</v>
       </c>
     </row>
   </sheetData>
@@ -816,6 +855,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -873,7 +913,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -882,22 +922,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1482.4</v>
+        <v>2716</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>78.51000000000001</v>
+        <v>75.56999999999999</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>75.5</v>
+        <v>68.17</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>65.16</v>
+        <v>54.97</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -906,22 +946,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1760.4</v>
+        <v>1432.1</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>75.03</v>
+        <v>69.97</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>69.95</v>
+        <v>58.46</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>65.75</v>
+        <v>52.25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -930,22 +970,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>10711.5</v>
+        <v>1795.1</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>73.83</v>
+        <v>69.59</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>67.87</v>
+        <v>71.39</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>65.81999999999999</v>
+        <v>66.56999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -954,22 +994,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2968.6</v>
+        <v>1234</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>73.28</v>
+        <v>65.53</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>62.38</v>
+        <v>63.13</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>61.53</v>
+        <v>60.64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -978,22 +1018,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>2505.9</v>
+        <v>8082.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>73.18000000000001</v>
+        <v>64.97</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>62.61</v>
+        <v>62.47</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>51.87</v>
+        <v>63.46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1002,22 +1042,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>2599.9</v>
+        <v>1878.2</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>69.59</v>
+        <v>64.95999999999999</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>56.92</v>
+        <v>62.7</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>50.86</v>
+        <v>61.44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1026,22 +1066,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>8097</v>
+        <v>2605.6</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>69.34</v>
+        <v>63.23</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>62.86</v>
+        <v>57.17</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>63.57</v>
+        <v>50.98</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1050,22 +1090,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>950.75</v>
+        <v>2933.8</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>68.56999999999999</v>
+        <v>62.64</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>61.28</v>
+        <v>59.96</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>49.06</v>
+        <v>60.77</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1074,22 +1114,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1847.9</v>
+        <v>299.35</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>65.70999999999999</v>
+        <v>60.94</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>60.79</v>
+        <v>65.76000000000001</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>60.44</v>
+        <v>69.22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1098,22 +1138,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1347</v>
+        <v>10377.5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>64.37</v>
+        <v>60.09</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>48.52</v>
+        <v>62.14</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>47.56</v>
+        <v>64.19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1122,22 +1162,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1176.2</v>
+        <v>1336.7</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>63.37</v>
+        <v>59.87</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>57.14</v>
+        <v>59</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>57.65</v>
+        <v>58.71</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1146,22 +1186,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4509</v>
+        <v>1905.4</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>60.36</v>
+        <v>59.62</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>64.69</v>
+        <v>49.55</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>64.56</v>
+        <v>61.13</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,22 +1210,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1277.8</v>
+        <v>216.84</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>60.11</v>
+        <v>58.21</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>61.93</v>
+        <v>66.04000000000001</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>65.95</v>
+        <v>67.31999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1194,22 +1234,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>3330.4</v>
+        <v>1067.5</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>59.81</v>
+        <v>58.13</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>50.68</v>
+        <v>69.75</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>59.79</v>
+        <v>72.73999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1218,22 +1258,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>402.15</v>
+        <v>1430.5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>59.54</v>
+        <v>58.05</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>67.86</v>
+        <v>66.61</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>68.73</v>
+        <v>62.33</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1242,22 +1282,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>214.49</v>
+        <v>387.05</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>59.36</v>
+        <v>57.89</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>64.95</v>
+        <v>46.12</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>66.81999999999999</v>
+        <v>49.51</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1266,22 +1306,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1435.2</v>
+        <v>1278.8</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>59.02</v>
+        <v>56.83</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>52.58</v>
+        <v>62.03</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>53.68</v>
+        <v>65.98999999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1290,22 +1330,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>4242.3</v>
+        <v>356.55</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>58.97</v>
+        <v>56.81</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>52.3</v>
+        <v>50.73</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>48.44</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1314,22 +1354,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1044.4</v>
+        <v>309.45</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>58.66</v>
+        <v>53.83</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>67.81</v>
+        <v>39.55</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>71.84999999999999</v>
+        <v>37.94</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1338,22 +1378,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>955.35</v>
+        <v>462.2</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>58.15</v>
+        <v>52.11</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>52.19</v>
+        <v>60.07</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>56.19</v>
+        <v>66.54000000000001</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1362,22 +1402,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>13726</v>
+        <v>395.25</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>57.34</v>
+        <v>52.04</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>46.21</v>
+        <v>63.57</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>53.58</v>
+        <v>66.95</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1386,22 +1426,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>355.45</v>
+        <v>2272.2</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>56.28</v>
+        <v>51.8</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>50.37</v>
+        <v>48.98</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v/>
+        <v>47.44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1410,22 +1450,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>5322</v>
+        <v>4101.3</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>56.27</v>
+        <v>50.29</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>50.59</v>
+        <v>49.2</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>58.74</v>
+        <v>47.23</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1434,22 +1474,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>621.7</v>
+        <v>1864.5</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>55.32</v>
+        <v>50.07</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>40.49</v>
+        <v>46.98</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>44.03</v>
+        <v>56.99</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1458,22 +1498,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>7302.5</v>
+        <v>608.7</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>55.15</v>
+        <v>49.62</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>53.77</v>
+        <v>38.53</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>64.44</v>
+        <v>42.57</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1482,22 +1522,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1818.3</v>
+        <v>886.4</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>54.42</v>
+        <v>49.26</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>45.36</v>
+        <v>52.6</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>49.82</v>
+        <v>46.13</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1506,22 +1546,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>11950</v>
+        <v>13221</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>54.29</v>
+        <v>47.34</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>51.56</v>
+        <v>42.43</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>55.63</v>
+        <v>51.41</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1530,22 +1570,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>2287.7</v>
+        <v>3909</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>54.28</v>
+        <v>46.68</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>50.01</v>
+        <v>50.55</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>47.93</v>
+        <v>55.98</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1554,22 +1594,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1007.75</v>
+        <v>910.45</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>54.24</v>
+        <v>46.44</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>57.55</v>
+        <v>46.8</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>66.58</v>
+        <v>53.47</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1578,22 +1618,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>313.95</v>
+        <v>3123.1</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>53.88</v>
+        <v>46.39</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>64.26000000000001</v>
+        <v>44.68</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>61.6</v>
+        <v>55.88</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1602,22 +1642,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1463</v>
+        <v>5064.5</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>52.89</v>
+        <v>45.08</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>49.08</v>
+        <v>45.95</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>51.61</v>
+        <v>55.85</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1626,22 +1666,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>380.8</v>
+        <v>767.5</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>52.67</v>
+        <v>44.45</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>43.21</v>
+        <v>31.49</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>48.35</v>
+        <v>40.44</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1650,22 +1690,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1293.9</v>
+        <v>7014.5</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>52.21</v>
+        <v>44.35</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>54.03</v>
+        <v>49.13</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>55.55</v>
+        <v>61.97</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1674,22 +1714,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>439.7</v>
+        <v>305.85</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>51.56</v>
+        <v>43.99</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>54.81</v>
+        <v>58.28</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>65.95999999999999</v>
+        <v>59.18</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1698,22 +1738,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1872.1</v>
+        <v>11487</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>50.93</v>
+        <v>43.96</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>47.46</v>
+        <v>46.62</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>57.29</v>
+        <v>52.72</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1722,22 +1762,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>307.45</v>
+        <v>4169.1</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>50.48</v>
+        <v>43.31</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>38.38</v>
+        <v>51.38</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>37.64</v>
+        <v>58.92</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1746,22 +1786,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>3974.5</v>
+        <v>937.9</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>50.09</v>
+        <v>43.05</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>52.63</v>
+        <v>50.54</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>57.28</v>
+        <v>63.9</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1770,22 +1810,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>456.4</v>
+        <v>423.65</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>48.61</v>
+        <v>42.1</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>58.73</v>
+        <v>50.03</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>65.15000000000001</v>
+        <v>63.55</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1794,22 +1834,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1834.5</v>
+        <v>1728.1</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>47.74</v>
+        <v>40.79</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>43.31</v>
+        <v>40.27</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>57.35</v>
+        <v>46.43</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1818,22 +1858,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>302.75</v>
+        <v>1370.5</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>47.04</v>
+        <v>40.49</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>43.38</v>
+        <v>43.05</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>52.2</v>
+        <v>48.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1842,22 +1882,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>780.85</v>
+        <v>1244.5</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>45.71</v>
+        <v>40.12</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>33.16</v>
+        <v>40.02</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>41.77</v>
+        <v>49.53</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1866,22 +1906,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>197.91</v>
+        <v>1244.8</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>43.94</v>
+        <v>39.34</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>36.25</v>
+        <v>47.45</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>41.19</v>
+        <v>54.88</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1890,22 +1930,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1268.3</v>
+        <v>1336.4</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>43.82</v>
+        <v>38.85</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>49.94</v>
+        <v>42.72</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>56.31</v>
+        <v>48.08</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1914,22 +1954,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>279.2</v>
+        <v>5406</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>43.03</v>
+        <v>38.43</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>58.27</v>
+        <v>38.41</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>61.79</v>
+        <v>50.21</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1938,22 +1978,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>1264.8</v>
+        <v>284.45</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>42.79</v>
+        <v>38.4</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>42.06</v>
+        <v>38.78</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>51.15</v>
+        <v>49.18</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1962,22 +2002,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>5520</v>
+        <v>190</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>40.15</v>
+        <v>35.8</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>41.51</v>
+        <v>32.55</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>51.81</v>
+        <v>39.46</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1986,22 +2026,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1179.2</v>
+        <v>963.2</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>38.87</v>
+        <v>33.97</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>31.99</v>
+        <v>44.36</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>36.95</v>
+        <v>57.25</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2010,22 +2050,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>2394.4</v>
+        <v>1119</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>38.59</v>
+        <v>33.79</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>32.74</v>
+        <v>28.83</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>34.31</v>
+        <v>35.09</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2034,16 +2074,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1019.3</v>
+        <v>2264</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>37.49</v>
+        <v>29.8</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>48.74</v>
+        <v>28.89</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>59.92</v>
+        <v>32.52</v>
       </c>
     </row>
     <row r="51">
@@ -2058,16 +2098,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1198.4</v>
+        <v>1132.6</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>32.83</v>
+        <v>26.71</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>31.79</v>
+        <v>28.52</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>41.59</v>
+        <v>39.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-05-22
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1795.1</v>
+        <v>3155.3</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>69.59</v>
+        <v>77.56999999999999</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>71.39</v>
+        <v>68.36</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>66.56999999999999</v>
+        <v>65.16</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>26.81</v>
+        <v>25.99</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1496.01</v>
+        <v>2793.52</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1472.69</v>
+        <v>2777.8</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>3826358</v>
+        <v>992560</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>413584</v>
+        <v>213984</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>8082.5</v>
+        <v>1786.9</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>64.97</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>62.47</v>
+        <v>70.53</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>63.46</v>
+        <v>66.38</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>22.9</v>
+        <v>33.84</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>7486.84</v>
+        <v>1514.43</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>7424.34</v>
+        <v>1487.98</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>378971</v>
+        <v>3522950</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>116214</v>
+        <v>411694</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>299.35</v>
+        <v>1109.2</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>60.94</v>
+        <v>64.2</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>65.76000000000001</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>69.22</v>
+        <v>74.22</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>28.54</v>
+        <v>21.08</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>262.68</v>
+        <v>922.39</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>257.64</v>
+        <v>889.1900000000001</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>18759890</v>
+        <v>5066951</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>376591</v>
+        <v>248034</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>216.84</v>
+        <v>10549.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>58.21</v>
+        <v>60.86</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>66.04000000000001</v>
+        <v>63.84</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>67.31999999999999</v>
+        <v>65.05</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>23.45</v>
+        <v>20.25</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>191.83</v>
+        <v>9474.879999999999</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>186.45</v>
+        <v>9350.549999999999</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>26436259</v>
+        <v>410631</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>270440</v>
+        <v>294618</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1430.5</v>
+        <v>1285.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>58.05</v>
+        <v>57.35</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>66.61</v>
+        <v>62.72</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>62.33</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>34.05</v>
+        <v>44.72</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1286.58</v>
+        <v>1190.52</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1269.13</v>
+        <v>1168.44</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2302030</v>
+        <v>1988829</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>275845</v>
+        <v>313743</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,37 +741,37 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1278.8</v>
+        <v>1423.1</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>56.83</v>
+        <v>54.63</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>62.03</v>
+        <v>65.43000000000001</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>65.98999999999999</v>
+        <v>61.85</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>29.53</v>
+        <v>43.95</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1183.9</v>
+        <v>1295.35</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1162.13</v>
+        <v>1276.63</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>2070783</v>
+        <v>2350840</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>312108</v>
+        <v>274418</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -780,70 +780,31 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>462.2</v>
+        <v>290</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>52.11</v>
+        <v>49.29</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>60.07</v>
+        <v>60.34</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>66.54000000000001</v>
+        <v>65.56</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>32.74</v>
+        <v>24.49</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>424.09</v>
+        <v>264.8</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>416</v>
+        <v>259.52</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>12114342</v>
+        <v>16561833</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>284841</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>NTPC</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>395.25</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>52.04</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>63.57</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>66.95</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>50.79</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>363.68</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>358.27</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>10640064</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>383261</v>
+        <v>364828</v>
       </c>
     </row>
   </sheetData>
@@ -855,7 +816,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -913,7 +873,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -922,22 +882,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>2716</v>
+        <v>3155.3</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.56999999999999</v>
+        <v>77.56999999999999</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.17</v>
+        <v>68.36</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>54.97</v>
+        <v>65.16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -946,22 +906,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1432.1</v>
+        <v>8362.5</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>69.97</v>
+        <v>72.61</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>58.46</v>
+        <v>66.72</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>52.25</v>
+        <v>65.48999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -970,22 +930,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1795.1</v>
+        <v>2717.3</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>69.59</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>71.39</v>
+        <v>68.2</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>66.56999999999999</v>
+        <v>54.98</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -994,22 +954,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1234</v>
+        <v>2639.8</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>65.53</v>
+        <v>65.56999999999999</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>63.13</v>
+        <v>58.67</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>60.64</v>
+        <v>51.66</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1018,22 +978,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>8082.5</v>
+        <v>1786.9</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>64.97</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>62.47</v>
+        <v>70.53</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>63.46</v>
+        <v>66.38</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1042,22 +1002,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1878.2</v>
+        <v>1109.2</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>64.95999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>62.7</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>61.44</v>
+        <v>74.22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1066,22 +1026,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>2605.6</v>
+        <v>1399.2</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>63.23</v>
+        <v>61.93</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>57.17</v>
+        <v>54.11</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>50.98</v>
+        <v>50.54</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1090,22 +1050,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2933.8</v>
+        <v>4296.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>62.64</v>
+        <v>61.01</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>59.96</v>
+        <v>53.33</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>60.77</v>
+        <v>48.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1114,22 +1074,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>299.35</v>
+        <v>10549.5</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>60.94</v>
+        <v>60.86</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>65.76000000000001</v>
+        <v>63.84</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>69.22</v>
+        <v>65.05</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1138,22 +1098,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>10377.5</v>
+        <v>363.35</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>60.09</v>
+        <v>59.9</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>62.14</v>
+        <v>53.02</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>64.19</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1162,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1336.7</v>
+        <v>203.11</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>59.87</v>
+        <v>59.22</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>59</v>
+        <v>42.94</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>58.71</v>
+        <v>42.62</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1186,22 +1146,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1905.4</v>
+        <v>1285.5</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>59.62</v>
+        <v>57.35</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>49.55</v>
+        <v>62.72</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>61.13</v>
+        <v>66.29000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1210,22 +1170,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>216.84</v>
+        <v>910.15</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>58.21</v>
+        <v>55.65</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>66.04000000000001</v>
+        <v>55.12</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>67.31999999999999</v>
+        <v>47.15</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1234,22 +1194,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1067.5</v>
+        <v>1423.1</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>58.13</v>
+        <v>54.63</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>69.75</v>
+        <v>65.43000000000001</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>72.73999999999999</v>
+        <v>61.85</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1258,22 +1218,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1430.5</v>
+        <v>1844.6</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>58.05</v>
+        <v>54.53</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>66.61</v>
+        <v>59.25</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>62.33</v>
+        <v>60.33</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1282,22 +1242,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>387.05</v>
+        <v>616.6</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>57.89</v>
+        <v>53.52</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>46.12</v>
+        <v>40.42</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>49.51</v>
+        <v>43.47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1306,22 +1266,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1278.8</v>
+        <v>384.15</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>56.83</v>
+        <v>53.45</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>62.03</v>
+        <v>44.97</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>65.98999999999999</v>
+        <v>48.96</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1330,22 +1290,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>356.55</v>
+        <v>1191.8</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>56.81</v>
+        <v>53.44</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>50.73</v>
+        <v>56.88</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v/>
+        <v>58.5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1354,22 +1314,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>309.45</v>
+        <v>1285.4</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>53.83</v>
+        <v>52.85</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>39.55</v>
+        <v>51.91</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>37.94</v>
+        <v>57.13</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1378,22 +1338,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>462.2</v>
+        <v>1307.2</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>52.11</v>
+        <v>52.41</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>60.07</v>
+        <v>54.62</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>66.54000000000001</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1402,22 +1362,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>395.25</v>
+        <v>1871.4</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>52.04</v>
+        <v>52.13</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>63.57</v>
+        <v>46.89</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>66.95</v>
+        <v>59.47</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1426,22 +1386,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>2272.2</v>
+        <v>3926.6</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>51.8</v>
+        <v>51.68</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>48.98</v>
+        <v>52.29</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>47.44</v>
+        <v>57.09</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1450,22 +1410,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>4101.3</v>
+        <v>1870.7</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>50.29</v>
+        <v>51.24</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>49.2</v>
+        <v>47.45</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>47.23</v>
+        <v>57.23</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1474,22 +1434,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1864.5</v>
+        <v>290</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>50.07</v>
+        <v>49.29</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>46.98</v>
+        <v>60.34</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>56.99</v>
+        <v>65.56</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1498,22 +1458,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>608.7</v>
+        <v>1422.2</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>49.62</v>
+        <v>48.76</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>38.53</v>
+        <v>46.97</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>42.57</v>
+        <v>50.05</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1522,22 +1482,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>886.4</v>
+        <v>1766</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>49.26</v>
+        <v>48.68</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>52.6</v>
+        <v>43.15</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>46.13</v>
+        <v>47.85</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1546,22 +1506,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>13221</v>
+        <v>916.55</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>47.34</v>
+        <v>48.41</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>42.43</v>
+        <v>47.59</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>51.41</v>
+        <v>53.86</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1570,22 +1530,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>3909</v>
+        <v>1264.3</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>46.68</v>
+        <v>48.31</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>50.55</v>
+        <v>42.92</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>55.98</v>
+        <v>51.11</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1594,22 +1554,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>910.45</v>
+        <v>456.55</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>46.44</v>
+        <v>47.87</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>46.8</v>
+        <v>58.09</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>53.47</v>
+        <v>65.18000000000001</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1618,22 +1578,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>3123.1</v>
+        <v>295.6</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>46.39</v>
+        <v>47.75</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>44.68</v>
+        <v>42.76</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>55.88</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1642,22 +1602,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>5064.5</v>
+        <v>209.19</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>45.08</v>
+        <v>47.74</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>45.95</v>
+        <v>59.52</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>55.85</v>
+        <v>65.22</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1666,22 +1626,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>767.5</v>
+        <v>11569</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>44.45</v>
+        <v>47.63</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>31.49</v>
+        <v>47.58</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>40.44</v>
+        <v>53.31</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1690,22 +1650,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>7014.5</v>
+        <v>1174.5</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>44.35</v>
+        <v>46.46</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>49.13</v>
+        <v>35.19</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>61.97</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1714,22 +1674,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>305.85</v>
+        <v>388.65</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>43.99</v>
+        <v>45.97</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>58.28</v>
+        <v>59.69</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>59.18</v>
+        <v>64.86</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1738,22 +1698,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>11487</v>
+        <v>941</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>43.96</v>
+        <v>45.88</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>46.62</v>
+        <v>50.82</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>52.72</v>
+        <v>64.03</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1762,22 +1722,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>4169.1</v>
+        <v>6981.5</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>43.31</v>
+        <v>45.69</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>51.38</v>
+        <v>48.61</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>58.92</v>
+        <v>61.58</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1786,22 +1746,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>937.9</v>
+        <v>766.8</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>43.05</v>
+        <v>45.48</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>50.54</v>
+        <v>31.4</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>63.9</v>
+        <v>40.39</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1810,22 +1770,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>423.65</v>
+        <v>1354.5</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>42.1</v>
+        <v>45.39</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>50.03</v>
+        <v>44.76</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>63.55</v>
+        <v>49.02</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1834,22 +1794,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1728.1</v>
+        <v>3081.3</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>40.79</v>
+        <v>44.27</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>40.27</v>
+        <v>43.56</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>46.43</v>
+        <v>54.92</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1858,22 +1818,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1370.5</v>
+        <v>2203.6</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>40.49</v>
+        <v>43.94</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>43.05</v>
+        <v>44.6</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>48.2</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1882,22 +1842,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1244.5</v>
+        <v>12987</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>40.12</v>
+        <v>43.03</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>40.02</v>
+        <v>40.76</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>49.53</v>
+        <v>50.35</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1906,22 +1866,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1244.8</v>
+        <v>301.7</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>39.34</v>
+        <v>42.39</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>47.45</v>
+        <v>36.64</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>54.88</v>
+        <v>36.79</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1930,22 +1890,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1336.4</v>
+        <v>4966</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>38.85</v>
+        <v>41.77</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>42.72</v>
+        <v>44.28</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>48.08</v>
+        <v>54.47</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1954,22 +1914,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>5406</v>
+        <v>416.55</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>38.43</v>
+        <v>40.38</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>38.41</v>
+        <v>48.04</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>50.21</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1978,22 +1938,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>284.45</v>
+        <v>4079.8</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>38.4</v>
+        <v>39.11</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>38.78</v>
+        <v>48.55</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>49.18</v>
+        <v>57.34</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -2002,22 +1962,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>190</v>
+        <v>2317.3</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>35.8</v>
+        <v>38.95</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>32.55</v>
+        <v>32.39</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>39.46</v>
+        <v>33.22</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -2026,22 +1986,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>963.2</v>
+        <v>1164</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>33.97</v>
+        <v>37.47</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>44.36</v>
+        <v>32.11</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>57.25</v>
+        <v>40.17</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2050,22 +2010,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>1119</v>
+        <v>5331.5</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>33.79</v>
+        <v>36.05</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>28.83</v>
+        <v>36.5</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>35.09</v>
+        <v>49.22</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2074,22 +2034,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>2264</v>
+        <v>294.3</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>29.8</v>
+        <v>33.94</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>28.89</v>
+        <v>51.01</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>32.52</v>
+        <v>56.05</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2098,16 +2058,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1132.6</v>
+        <v>949.2</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>26.71</v>
+        <v>33.73</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>28.52</v>
+        <v>43.07</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>39.2</v>
+        <v>56.33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-05-30
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -546,31 +546,31 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>3155.3</v>
+        <v>3122.4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>77.56999999999999</v>
+        <v>69.06</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.36</v>
+        <v>66.14</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>65.16</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>25.99</v>
+        <v>25.21</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>2793.52</v>
+        <v>2812.36</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>2777.8</v>
+        <v>2792.43</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>992560</v>
+        <v>999786</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>213984</v>
+        <v>211753</v>
       </c>
     </row>
     <row r="3">
@@ -585,31 +585,31 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1786.9</v>
+        <v>1804.6</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>65.51000000000001</v>
+        <v>64.89</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>70.53</v>
+        <v>71.33</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>66.38</v>
+        <v>66.78</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>33.84</v>
+        <v>35.22</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1514.43</v>
+        <v>1529.86</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>1487.98</v>
+        <v>1500.85</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>3522950</v>
+        <v>3180591</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>411694</v>
+        <v>415772</v>
       </c>
     </row>
     <row r="4">
@@ -624,31 +624,31 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1109.2</v>
+        <v>1126.7</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>64.2</v>
+        <v>62.53</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>72.93000000000001</v>
+        <v>74.15000000000001</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>74.22</v>
+        <v>74.79000000000001</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>21.08</v>
+        <v>24.64</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>922.39</v>
+        <v>935.5599999999999</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>889.1900000000001</v>
+        <v>900.89</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>5066973</v>
+        <v>4934238</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>248034</v>
+        <v>251947</v>
       </c>
     </row>
     <row r="5">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>10549.5</v>
+        <v>10460</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>60.86</v>
+        <v>58.56</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>63.84</v>
+        <v>64.41</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>65.05</v>
+        <v>65.33</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>20.25</v>
+        <v>27.84</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>9474.879999999999</v>
+        <v>9419.26</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>9350.549999999999</v>
+        <v>9285.57</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>410632</v>
+        <v>394851</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>294618</v>
+        <v>292118</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,31 +702,31 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1285.5</v>
+        <v>8176.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>57.35</v>
+        <v>58.2</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>62.72</v>
+        <v>61.72</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>66.29000000000001</v>
+        <v>64.17</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>44.72</v>
+        <v>32.96</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1190.52</v>
+        <v>7578.49</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1168.44</v>
+        <v>7500.39</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1988829</v>
+        <v>427070</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>313743</v>
+        <v>117566</v>
       </c>
     </row>
     <row r="7">
@@ -741,37 +741,37 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1423.1</v>
+        <v>1421.5</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>54.63</v>
+        <v>53.08</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>65.43000000000001</v>
+        <v>65.16</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>61.85</v>
+        <v>61.74</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>43.95</v>
+        <v>45.51</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1295.35</v>
+        <v>1303.63</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1276.63</v>
+        <v>1283.83</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>2350842</v>
+        <v>2664198</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>274418</v>
+        <v>274110</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -780,31 +780,31 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>290</v>
+        <v>1278</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>49.29</v>
+        <v>51.6</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>60.34</v>
+        <v>61.37</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>65.56</v>
+        <v>65.95999999999999</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>24.49</v>
+        <v>39.82</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>264.8</v>
+        <v>1197.3</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>259.52</v>
+        <v>1174.57</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>16561907</v>
+        <v>1958090</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>364828</v>
+        <v>311913</v>
       </c>
     </row>
   </sheetData>
@@ -873,7 +873,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -882,22 +882,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>3155.3</v>
+        <v>2937.4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>77.56999999999999</v>
+        <v>76.61</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.36</v>
+        <v>73.06</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>65.16</v>
+        <v>57.82</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -906,22 +906,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>8362.5</v>
+        <v>393.9</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>72.61</v>
+        <v>69.28</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>66.72</v>
+        <v>52.53</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>65.48999999999999</v>
+        <v>39.11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -930,16 +930,16 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>2717.3</v>
+        <v>3122.4</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>71.93000000000001</v>
+        <v>69.06</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>68.2</v>
+        <v>66.14</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>54.98</v>
+        <v>64.56999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -954,16 +954,16 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2639.8</v>
+        <v>2671.6</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>65.56999999999999</v>
+        <v>67.45</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>58.67</v>
+        <v>60.08</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>51.66</v>
+        <v>52.28</v>
       </c>
     </row>
     <row r="6">
@@ -978,22 +978,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1786.9</v>
+        <v>1804.6</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>65.51000000000001</v>
+        <v>64.89</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>70.53</v>
+        <v>71.33</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>66.38</v>
+        <v>66.78</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1002,22 +1002,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1109.2</v>
+        <v>4076.5</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>64.2</v>
+        <v>62.93</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>72.93000000000001</v>
+        <v>56.79</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>74.22</v>
+        <v>59.58</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1399.2</v>
+        <v>1126.7</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>61.93</v>
+        <v>62.53</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>54.11</v>
+        <v>74.15000000000001</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>50.54</v>
+        <v>74.79000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1050,16 +1050,16 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>4296.5</v>
+        <v>1401</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>61.01</v>
+        <v>59.36</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>53.33</v>
+        <v>54.31</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>48.9</v>
+        <v>50.64</v>
       </c>
     </row>
     <row r="10">
@@ -1074,22 +1074,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>10549.5</v>
+        <v>10460</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>60.86</v>
+        <v>58.56</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>63.84</v>
+        <v>64.41</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>65.05</v>
+        <v>65.33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1098,16 +1098,16 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>363.35</v>
+        <v>8176.5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>59.9</v>
+        <v>58.2</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>53.02</v>
+        <v>61.72</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v/>
+        <v>64.17</v>
       </c>
     </row>
     <row r="12">
@@ -1122,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>203.11</v>
+        <v>204.25</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>59.22</v>
+        <v>58.1</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>42.94</v>
+        <v>43.76</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>42.62</v>
+        <v>42.98</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1146,22 +1146,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1285.5</v>
+        <v>1483.9</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>57.35</v>
+        <v>57.85</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>62.72</v>
+        <v>51.29</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>66.29000000000001</v>
+        <v>52.41</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,22 +1170,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>910.15</v>
+        <v>4224</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>55.65</v>
+        <v>55.44</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>55.12</v>
+        <v>51.65</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>47.15</v>
+        <v>48.28</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1194,22 +1194,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1423.1</v>
+        <v>914.35</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>54.63</v>
+        <v>53.98</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>65.43000000000001</v>
+        <v>55.57</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>61.85</v>
+        <v>47.33</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1218,22 +1218,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1844.6</v>
+        <v>1421.5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>54.53</v>
+        <v>53.08</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>59.25</v>
+        <v>65.16</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>60.33</v>
+        <v>61.74</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1242,22 +1242,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>616.6</v>
+        <v>1278</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>53.52</v>
+        <v>51.6</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>40.42</v>
+        <v>61.37</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>43.47</v>
+        <v>65.95999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1266,22 +1266,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>384.15</v>
+        <v>1286.6</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>53.45</v>
+        <v>51.39</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>44.97</v>
+        <v>52.04</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>48.96</v>
+        <v>57.18</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1290,22 +1290,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1191.8</v>
+        <v>7177</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>53.44</v>
+        <v>51.36</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>56.88</v>
+        <v>51.85</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>58.5</v>
+        <v>63.58</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1314,22 +1314,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1285.4</v>
+        <v>384.2</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>52.85</v>
+        <v>51.24</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>51.91</v>
+        <v>44.99</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>57.13</v>
+        <v>48.97</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1338,22 +1338,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1307.2</v>
+        <v>1178.4</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>52.41</v>
+        <v>50.57</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>54.62</v>
+        <v>56.4</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>56.6</v>
+        <v>58.32</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1362,22 +1362,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1871.4</v>
+        <v>1783.6</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>52.13</v>
+        <v>50.4</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>46.89</v>
+        <v>44.5</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>59.47</v>
+        <v>48.53</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>3926.6</v>
+        <v>1303.5</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>51.68</v>
+        <v>50.14</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>52.29</v>
+        <v>54.07</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>57.09</v>
+        <v>56.3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1410,22 +1410,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1870.7</v>
+        <v>457.9</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>51.24</v>
+        <v>48.53</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>47.45</v>
+        <v>58.44</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>57.23</v>
+        <v>65.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1434,22 +1434,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>290</v>
+        <v>298.1</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>49.29</v>
+        <v>48.22</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>60.34</v>
+        <v>43.65</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>65.56</v>
+        <v>51.42</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1458,22 +1458,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1422.2</v>
+        <v>947.15</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>48.76</v>
+        <v>47.41</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>46.97</v>
+        <v>51.43</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>50.05</v>
+        <v>64.28</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1482,22 +1482,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1766</v>
+        <v>13127</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>48.68</v>
+        <v>47.25</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>43.15</v>
+        <v>42.22</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>47.85</v>
+        <v>50.98</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1506,16 +1506,16 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>916.55</v>
+        <v>1799.2</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>48.41</v>
+        <v>45.87</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>47.59</v>
+        <v>54.84</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>53.86</v>
+        <v>58.59</v>
       </c>
     </row>
     <row r="29">
@@ -1530,22 +1530,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1264.3</v>
+        <v>1256.4</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>48.31</v>
+        <v>45.8</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>42.92</v>
+        <v>42.05</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>51.11</v>
+        <v>50.47</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1554,22 +1554,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>456.55</v>
+        <v>208.02</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>47.87</v>
+        <v>45.51</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>58.09</v>
+        <v>58.57</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>65.18000000000001</v>
+        <v>64.73</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1578,22 +1578,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>295.6</v>
+        <v>11482</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>47.75</v>
+        <v>45.37</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>42.76</v>
+        <v>46.62</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>51</v>
+        <v>52.69</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1602,22 +1602,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>209.19</v>
+        <v>908.25</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>47.74</v>
+        <v>45.08</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>59.52</v>
+        <v>46.57</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>65.22</v>
+        <v>53.34</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1626,22 +1626,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>11569</v>
+        <v>1829</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>47.63</v>
+        <v>45.05</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>47.58</v>
+        <v>43.73</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>53.31</v>
+        <v>57.05</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1650,16 +1650,16 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1174.5</v>
+        <v>1183.8</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>46.46</v>
+        <v>44.97</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>35.19</v>
+        <v>34.35</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>36.8</v>
+        <v>40.91</v>
       </c>
     </row>
     <row r="35">
@@ -1674,22 +1674,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>388.65</v>
+        <v>386.9</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>45.97</v>
+        <v>44.44</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>59.69</v>
+        <v>58.66</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>64.86</v>
+        <v>64.31999999999999</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1698,22 +1698,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>941</v>
+        <v>1160.9</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>45.88</v>
+        <v>43.91</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>50.82</v>
+        <v>34.38</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>64.03</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1722,22 +1722,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>6981.5</v>
+        <v>1830.1</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>45.69</v>
+        <v>42.98</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>48.61</v>
+        <v>44.67</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>61.58</v>
+        <v>55.58</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1746,22 +1746,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>766.8</v>
+        <v>594.8</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>45.48</v>
+        <v>42.13</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>31.4</v>
+        <v>37.03</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>40.39</v>
+        <v>40.92</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1770,22 +1770,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1354.5</v>
+        <v>3045.6</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>45.39</v>
+        <v>42</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>44.76</v>
+        <v>42.58</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>49.02</v>
+        <v>54.01</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1794,22 +1794,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>3081.3</v>
+        <v>4074.9</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>44.27</v>
+        <v>40.96</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>43.56</v>
+        <v>48.39</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>54.92</v>
+        <v>57.26</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1818,22 +1818,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>2203.6</v>
+        <v>4903</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>43.94</v>
+        <v>40.29</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>44.6</v>
+        <v>43.2</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>45.4</v>
+        <v>53.62</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1842,22 +1842,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>12987</v>
+        <v>964.4</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>43.03</v>
+        <v>39.76</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>40.76</v>
+        <v>45.24</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>50.35</v>
+        <v>57.33</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1866,22 +1866,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>301.7</v>
+        <v>744.55</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>42.39</v>
+        <v>38.75</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>36.64</v>
+        <v>28.63</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>36.79</v>
+        <v>38.77</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1890,22 +1890,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>4966</v>
+        <v>1321.2</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>41.77</v>
+        <v>38.42</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>44.28</v>
+        <v>41.81</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>54.47</v>
+        <v>47.32</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1914,22 +1914,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>416.55</v>
+        <v>2153.5</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>40.38</v>
+        <v>37.66</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>48.04</v>
+        <v>41.67</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>62.2</v>
+        <v>44.06</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1938,16 +1938,16 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>4079.8</v>
+        <v>410.75</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>39.11</v>
+        <v>37.43</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>48.55</v>
+        <v>46.41</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>57.34</v>
+        <v>61.14</v>
       </c>
     </row>
     <row r="47">
@@ -1962,22 +1962,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>2317.3</v>
+        <v>2258.9</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>38.95</v>
+        <v>37.13</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>32.39</v>
+        <v>31.52</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>33.22</v>
+        <v>32.85</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1986,22 +1986,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1164</v>
+        <v>290.55</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>37.47</v>
+        <v>35.72</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>32.11</v>
+        <v>48.87</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>40.17</v>
+        <v>55.1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2010,22 +2010,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>5331.5</v>
+        <v>286.9</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>36.05</v>
+        <v>34.9</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>36.5</v>
+        <v>34.19</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>49.22</v>
+        <v>35.82</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2034,22 +2034,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>294.3</v>
+        <v>265.4</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>33.94</v>
+        <v>31.18</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>51.01</v>
+        <v>48.94</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>56.05</v>
+        <v>57.56</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>949.2</v>
+        <v>5204.5</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>33.73</v>
+        <v>29.96</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>43.07</v>
+        <v>33.44</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>56.33</v>
+        <v>47.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-06-06
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>3122.4</v>
+        <v>1824.2</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>69.06</v>
+        <v>63.45</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>66.14</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>64.56999999999999</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>25.21</v>
+        <v>51.12</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>2812.36</v>
+        <v>1551.09</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>2792.43</v>
+        <v>1518.29</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>999786</v>
+        <v>2832055</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>211753</v>
+        <v>420288</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1804.6</v>
+        <v>3087.7</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>64.89</v>
+        <v>61.69</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>71.33</v>
+        <v>63.79</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>66.78</v>
+        <v>63.35</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>35.22</v>
+        <v>37.18</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1529.86</v>
+        <v>2835.12</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>1500.85</v>
+        <v>2810.29</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>3180591</v>
+        <v>950140</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>415772</v>
+        <v>209399</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1126.7</v>
+        <v>8304.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>62.53</v>
+        <v>61.64</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>74.15000000000001</v>
+        <v>63.73</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>74.79000000000001</v>
+        <v>65.16</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>24.64</v>
+        <v>54.46</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>935.5599999999999</v>
+        <v>7619.26</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>900.89</v>
+        <v>7535.21</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>4934238</v>
+        <v>428894</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>251947</v>
+        <v>119406</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>10460</v>
+        <v>472.3</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>58.56</v>
+        <v>56.65</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>64.41</v>
+        <v>62.1</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>65.33</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>27.84</v>
+        <v>39.95</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>9419.26</v>
+        <v>431.44</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>9285.57</v>
+        <v>422.72</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>394851</v>
+        <v>18851772</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>292118</v>
+        <v>291066</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>8176.5</v>
+        <v>10342</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>58.2</v>
+        <v>54.51</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>61.72</v>
+        <v>62.58</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>64.17</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>32.96</v>
+        <v>40.64</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>7578.49</v>
+        <v>9478.27</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7500.39</v>
+        <v>9339.68</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>427070</v>
+        <v>407985</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>117566</v>
+        <v>288823</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,31 +741,31 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1421.5</v>
+        <v>1092.6</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>53.08</v>
+        <v>50.92</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>65.16</v>
+        <v>67.72</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>61.74</v>
+        <v>71.45999999999999</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>45.51</v>
+        <v>31.79</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1303.63</v>
+        <v>948</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1283.83</v>
+        <v>911.9400000000001</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>2664198</v>
+        <v>5096988</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>274110</v>
+        <v>244322</v>
       </c>
     </row>
     <row r="8">
@@ -780,31 +780,31 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1278</v>
+        <v>1284</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>51.6</v>
+        <v>50.72</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>61.37</v>
+        <v>62.07</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>65.95999999999999</v>
+        <v>66.23999999999999</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>39.82</v>
+        <v>42.09</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1197.3</v>
+        <v>1203.99</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1174.57</v>
+        <v>1180.61</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1958090</v>
+        <v>1727162</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>311913</v>
+        <v>313377</v>
       </c>
     </row>
   </sheetData>
@@ -882,16 +882,16 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>2937.4</v>
+        <v>3048.2</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>76.61</v>
+        <v>75.83</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>73.06</v>
+        <v>75.12</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>57.82</v>
+        <v>59.22</v>
       </c>
     </row>
     <row r="3">
@@ -906,22 +906,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>393.9</v>
+        <v>397.8</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>69.28</v>
+        <v>66.69</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>52.53</v>
+        <v>53.41</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>39.11</v>
+        <v>39.43</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -930,22 +930,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>3122.4</v>
+        <v>2686.7</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>69.06</v>
+        <v>66.09</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>66.14</v>
+        <v>60.77</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>64.56999999999999</v>
+        <v>52.58</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -954,22 +954,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2671.6</v>
+        <v>1824.2</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>67.45</v>
+        <v>63.45</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>60.08</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>52.28</v>
+        <v>67.26000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -978,22 +978,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1804.6</v>
+        <v>3087.7</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>64.89</v>
+        <v>61.69</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>71.33</v>
+        <v>63.79</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>66.78</v>
+        <v>63.35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1002,22 +1002,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>4076.5</v>
+        <v>8304.5</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>62.93</v>
+        <v>61.64</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>56.79</v>
+        <v>63.73</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>59.58</v>
+        <v>65.16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1126.7</v>
+        <v>1401.3</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>62.53</v>
+        <v>61</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>74.15000000000001</v>
+        <v>55.86</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>74.79000000000001</v>
+        <v>51.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1050,22 +1050,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1401</v>
+        <v>472.3</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>59.36</v>
+        <v>56.65</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>54.31</v>
+        <v>62.1</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>50.64</v>
+        <v>67.34999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1074,22 +1074,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>10460</v>
+        <v>4260.2</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>58.56</v>
+        <v>55.63</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>64.41</v>
+        <v>54.41</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>65.33</v>
+        <v>59.66</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>8176.5</v>
+        <v>10342</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>58.2</v>
+        <v>54.51</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>61.72</v>
+        <v>62.58</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>64.17</v>
+        <v>64.76000000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1122,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>204.25</v>
+        <v>1483.5</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>58.1</v>
+        <v>53.29</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>43.76</v>
+        <v>51.26</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>42.98</v>
+        <v>52.39</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1146,22 +1146,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1483.9</v>
+        <v>1092.6</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>57.85</v>
+        <v>50.92</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>51.29</v>
+        <v>67.72</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>52.41</v>
+        <v>71.45999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,22 +1170,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>4224</v>
+        <v>1197.5</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>55.44</v>
+        <v>50.73</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>51.65</v>
+        <v>38.48</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>48.28</v>
+        <v>38.46</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1194,22 +1194,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>914.35</v>
+        <v>1284</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>53.98</v>
+        <v>50.72</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>55.57</v>
+        <v>62.07</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>47.33</v>
+        <v>66.23999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1218,22 +1218,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1421.5</v>
+        <v>904.8</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>53.08</v>
+        <v>50.49</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>65.16</v>
+        <v>54.24</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>61.74</v>
+        <v>46.88</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1242,22 +1242,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1278</v>
+        <v>1262.1</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>51.6</v>
+        <v>49.71</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>61.37</v>
+        <v>42.95</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>65.95999999999999</v>
+        <v>50.95</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1286.6</v>
+        <v>3953.2</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>51.39</v>
+        <v>49.48</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>52.04</v>
+        <v>52.48</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>57.18</v>
@@ -1281,7 +1281,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1290,22 +1290,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>7177</v>
+        <v>2774.2</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>51.36</v>
+        <v>49.2</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>51.85</v>
+        <v>41.68</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>63.58</v>
+        <v>39.65</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1314,22 +1314,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>384.2</v>
+        <v>1272.3</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>51.24</v>
+        <v>48.75</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>44.99</v>
+        <v>50.3</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>48.97</v>
+        <v>56.24</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1338,22 +1338,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1178.4</v>
+        <v>977.7</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>50.57</v>
+        <v>47.22</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>56.4</v>
+        <v>47.14</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>58.32</v>
+        <v>57.79</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1362,22 +1362,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1783.6</v>
+        <v>295</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>50.4</v>
+        <v>46.59</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>44.5</v>
+        <v>42.76</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>48.53</v>
+        <v>50.86</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1303.5</v>
+        <v>7070</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>50.14</v>
+        <v>46.5</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>54.07</v>
+        <v>49.99</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>56.3</v>
+        <v>62.21</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1410,22 +1410,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>457.9</v>
+        <v>198.37</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>48.53</v>
+        <v>46.22</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>58.44</v>
+        <v>40.55</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>65.5</v>
+        <v>41.53</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1434,22 +1434,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>298.1</v>
+        <v>13050</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>48.22</v>
+        <v>45.68</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>43.65</v>
+        <v>41.62</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>51.42</v>
+        <v>50.61</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1458,22 +1458,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>947.15</v>
+        <v>377.45</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>47.41</v>
+        <v>45.21</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>51.43</v>
+        <v>42.15</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>64.28</v>
+        <v>47.68</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1482,22 +1482,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>13127</v>
+        <v>1278.2</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>47.25</v>
+        <v>45.13</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>42.22</v>
+        <v>50.39</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>50.98</v>
+        <v>54.22</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1506,22 +1506,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1799.2</v>
+        <v>3040.5</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>45.87</v>
+        <v>44.33</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>54.84</v>
+        <v>42.44</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>58.59</v>
+        <v>53.87</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1530,22 +1530,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1256.4</v>
+        <v>206.77</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>45.8</v>
+        <v>43.53</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>42.05</v>
+        <v>57.51</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>50.47</v>
+        <v>64.18000000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1554,22 +1554,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>208.02</v>
+        <v>923.3</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>45.51</v>
+        <v>43.45</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>58.57</v>
+        <v>48.93</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>64.73</v>
+        <v>62.46</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1578,22 +1578,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>11482</v>
+        <v>889.4</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>45.37</v>
+        <v>42.66</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>46.62</v>
+        <v>44.26</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>52.69</v>
+        <v>52.09</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1602,22 +1602,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>908.25</v>
+        <v>1386.2</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>45.08</v>
+        <v>42.56</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>46.57</v>
+        <v>59.35</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>53.34</v>
+        <v>59.37</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1626,16 +1626,16 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1829</v>
+        <v>1782.2</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>45.05</v>
+        <v>42.26</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>43.73</v>
+        <v>53.25</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>57.05</v>
+        <v>57.67</v>
       </c>
     </row>
     <row r="34">
@@ -1650,22 +1650,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1183.8</v>
+        <v>1154.7</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>44.97</v>
+        <v>41.06</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>34.35</v>
+        <v>32.64</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>40.91</v>
+        <v>39.92</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1674,22 +1674,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>386.9</v>
+        <v>747.05</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>44.44</v>
+        <v>41.06</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>58.66</v>
+        <v>29.38</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>64.31999999999999</v>
+        <v>39.07</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1698,22 +1698,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1160.9</v>
+        <v>1798.2</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>43.91</v>
+        <v>40.47</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>34.38</v>
+        <v>41.54</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>36.36</v>
+        <v>55.29</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1722,22 +1722,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1830.1</v>
+        <v>1130.9</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>42.98</v>
+        <v>40.01</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>44.67</v>
+        <v>50.03</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>55.58</v>
+        <v>54.83</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1746,22 +1746,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>594.8</v>
+        <v>2121.5</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>42.13</v>
+        <v>39.62</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>37.03</v>
+        <v>39.87</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>40.92</v>
+        <v>43.18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1770,22 +1770,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>3045.6</v>
+        <v>2198.9</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>42</v>
+        <v>39.13</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>42.58</v>
+        <v>29.71</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>54.01</v>
+        <v>32.03</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1794,22 +1794,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>4074.9</v>
+        <v>4835</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>40.96</v>
+        <v>39.1</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>48.39</v>
+        <v>42</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>57.26</v>
+        <v>52.67</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1818,22 +1818,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>4903</v>
+        <v>408.2</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>40.29</v>
+        <v>37.83</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>43.2</v>
+        <v>45.68</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>53.62</v>
+        <v>60.65</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1842,22 +1842,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>964.4</v>
+        <v>1782.8</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>39.76</v>
+        <v>37.36</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>45.24</v>
+        <v>41.61</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>57.33</v>
+        <v>53.02</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1866,22 +1866,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>744.55</v>
+        <v>1703.2</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>38.75</v>
+        <v>36.61</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>28.63</v>
+        <v>39.87</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>38.77</v>
+        <v>45.61</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1890,22 +1890,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1321.2</v>
+        <v>280.7</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>38.42</v>
+        <v>35.81</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>41.81</v>
+        <v>32.74</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>47.32</v>
+        <v>35.16</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1914,22 +1914,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>2153.5</v>
+        <v>285.65</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>37.66</v>
+        <v>35.3</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>41.67</v>
+        <v>46.15</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>44.06</v>
+        <v>53.82</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1938,22 +1938,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>410.75</v>
+        <v>575.3</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>37.43</v>
+        <v>34.53</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>46.41</v>
+        <v>34.26</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>61.14</v>
+        <v>39.22</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1962,22 +1962,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>2258.9</v>
+        <v>1291</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>37.13</v>
+        <v>33.29</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>31.52</v>
+        <v>39.75</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>32.85</v>
+        <v>46.06</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1986,22 +1986,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>290.55</v>
+        <v>264.75</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>35.72</v>
+        <v>32.91</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>48.87</v>
+        <v>48.67</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>55.1</v>
+        <v>57.36</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2010,22 +2010,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>286.9</v>
+        <v>10912</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>34.9</v>
+        <v>32.4</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>34.19</v>
+        <v>40.83</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>35.82</v>
+        <v>48.67</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2034,22 +2034,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>265.4</v>
+        <v>5120.5</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>31.18</v>
+        <v>30.35</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>48.94</v>
+        <v>31.55</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>57.56</v>
+        <v>46.53</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>5204.5</v>
+        <v>361.65</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>29.96</v>
+        <v>28.2</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>33.44</v>
+        <v>46.32</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>47.62</v>
+        <v>57.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-06-13
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,31 +546,31 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1824.2</v>
+        <v>8498</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>63.45</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>72.23999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>67.26000000000001</v>
+        <v>66.56</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>51.12</v>
+        <v>56.19</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1551.09</v>
+        <v>7674.62</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1518.29</v>
+        <v>7582.51</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>2832055</v>
+        <v>464871</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>420288</v>
+        <v>122188</v>
       </c>
     </row>
     <row r="3">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>3087.7</v>
+        <v>3105.5</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>61.69</v>
+        <v>60.64</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>63.79</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>63.35</v>
+        <v>63.97</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>37.18</v>
+        <v>47.06</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2835.12</v>
+        <v>2851.26</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>2810.29</v>
+        <v>2824.54</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>950140</v>
+        <v>913440</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>209399</v>
+        <v>210607</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>8304.5</v>
+        <v>1812.9</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>61.64</v>
+        <v>58.97</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>63.73</v>
+        <v>71.78</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>65.16</v>
+        <v>67.17</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>54.46</v>
+        <v>52.62</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>7619.26</v>
+        <v>1561.38</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7535.21</v>
+        <v>1526.45</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>428894</v>
+        <v>2728423</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>119406</v>
+        <v>417685</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,148 +663,31 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>472.3</v>
+        <v>1297.6</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>56.65</v>
+        <v>55.65</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>62.1</v>
+        <v>63.7</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>67.34999999999999</v>
+        <v>66.88</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>39.95</v>
+        <v>44.55</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>431.44</v>
+        <v>1208.6</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>422.72</v>
+        <v>1185.45</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>18851772</v>
+        <v>1739195</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>291066</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>BAJAJ-AUTO</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>10342</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>54.51</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>62.58</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>64.76000000000001</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>40.64</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>9478.27</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>9339.68</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>407985</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>288823</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>HINDALCO</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>1092.6</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>50.92</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>67.72</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>71.45999999999999</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>31.79</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>948</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>911.9400000000001</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>5096988</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>244322</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>JSWSTEEL</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>1284</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>50.72</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>62.07</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>66.23999999999999</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>42.09</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>1203.99</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>1180.61</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>1727162</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>313377</v>
+        <v>316722</v>
       </c>
     </row>
   </sheetData>
@@ -813,9 +696,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -873,7 +753,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -882,22 +762,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>3048.2</v>
+        <v>1356.3</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.83</v>
+        <v>67.98</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>75.12</v>
+        <v>58.97</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>59.22</v>
+        <v>60.42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -906,22 +786,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>397.8</v>
+        <v>2747.4</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>66.69</v>
+        <v>67.81999999999999</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>53.41</v>
+        <v>63.47</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>39.43</v>
+        <v>53.79</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -930,22 +810,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>2686.7</v>
+        <v>403.3</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>66.09</v>
+        <v>67.58</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>60.77</v>
+        <v>54.09</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>52.58</v>
+        <v>52.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -954,22 +834,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1824.2</v>
+        <v>8498</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>63.45</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>72.23999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>67.26000000000001</v>
+        <v>66.56</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -978,22 +858,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3087.7</v>
+        <v>1340.8</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>61.69</v>
+        <v>67.01000000000001</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>63.79</v>
+        <v>53.7</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>63.35</v>
+        <v>56.76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1002,22 +882,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>8304.5</v>
+        <v>4709.7</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>61.64</v>
+        <v>62.38</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>63.73</v>
+        <v>50.98</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>65.16</v>
+        <v>52.22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1026,22 +906,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1401.3</v>
+        <v>1017.15</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>61</v>
+        <v>61.49</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>55.86</v>
+        <v>52.42</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>51.4</v>
+        <v>59.69</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1050,22 +930,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>472.3</v>
+        <v>2921.6</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>56.65</v>
+        <v>61.44</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>62.1</v>
+        <v>68.72</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>67.34999999999999</v>
+        <v>57.56</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1074,22 +954,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>4260.2</v>
+        <v>3105.5</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>55.63</v>
+        <v>60.64</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>54.41</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>59.66</v>
+        <v>63.97</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1098,22 +978,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>10342</v>
+        <v>1812.9</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>54.51</v>
+        <v>58.97</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>62.58</v>
+        <v>71.78</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>64.76000000000001</v>
+        <v>67.17</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1122,22 +1002,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1483.5</v>
+        <v>390</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>53.29</v>
+        <v>58.33</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>51.26</v>
+        <v>51.35</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>52.39</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1146,22 +1026,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1092.6</v>
+        <v>4049.3</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>50.92</v>
+        <v>58.28</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>67.72</v>
+        <v>55.33</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>71.45999999999999</v>
+        <v>59.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,22 +1050,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1197.5</v>
+        <v>7312</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>50.73</v>
+        <v>57.44</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>38.48</v>
+        <v>54.01</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>38.46</v>
+        <v>64.56999999999999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1194,22 +1074,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1284</v>
+        <v>1389.4</v>
       </c>
       <c r="D15" s="4" t="n">
+        <v>56.89</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>54.49</v>
+      </c>
+      <c r="F15" s="4" t="n">
         <v>50.72</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>62.07</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>66.23999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1218,22 +1098,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>904.8</v>
+        <v>13366</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>50.49</v>
+        <v>56.81</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>54.24</v>
+        <v>45.11</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>46.88</v>
+        <v>52.08</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1242,22 +1122,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1262.1</v>
+        <v>1297.6</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>49.71</v>
+        <v>55.65</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>42.95</v>
+        <v>63.7</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>50.95</v>
+        <v>66.88</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1266,22 +1146,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>3953.2</v>
+        <v>772.45</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>49.48</v>
+        <v>55.31</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>52.48</v>
+        <v>36.7</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>57.18</v>
+        <v>41.91</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1290,22 +1170,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>2774.2</v>
+        <v>954.95</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>49.2</v>
+        <v>54.4</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>41.68</v>
+        <v>52.24</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>39.65</v>
+        <v>64.62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1314,22 +1194,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1272.3</v>
+        <v>918.3</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>48.75</v>
+        <v>54.09</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>50.3</v>
+        <v>48.48</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>56.24</v>
+        <v>53.92</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1338,22 +1218,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>977.7</v>
+        <v>1012.45</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>47.22</v>
+        <v>53.58</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>47.14</v>
+        <v>48.01</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>57.79</v>
+        <v>52.03</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1362,22 +1242,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>295</v>
+        <v>4184</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>46.59</v>
+        <v>51.53</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>42.76</v>
+        <v>51.74</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>50.86</v>
+        <v>58.71</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1386,22 +1266,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>7070</v>
+        <v>1807.7</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>46.5</v>
+        <v>50.66</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>49.99</v>
+        <v>55.35</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>62.21</v>
+        <v>58.92</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1410,22 +1290,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>198.37</v>
+        <v>2168.8</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>46.22</v>
+        <v>49.17</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>40.55</v>
+        <v>43.74</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>41.53</v>
+        <v>44.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1434,22 +1314,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>13050</v>
+        <v>235.89</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>45.68</v>
+        <v>49.08</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>41.62</v>
+        <v>38.31</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>50.61</v>
+        <v>42.13</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1458,22 +1338,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>377.45</v>
+        <v>2755.3</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>45.21</v>
+        <v>48.9</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>42.15</v>
+        <v>41.32</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>47.68</v>
+        <v>39.55</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1482,16 +1362,16 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1278.2</v>
+        <v>1822.5</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>45.13</v>
+        <v>48.72</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>50.39</v>
+        <v>43.92</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>54.22</v>
+        <v>56.67</v>
       </c>
     </row>
     <row r="28">
@@ -1506,22 +1386,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>3040.5</v>
+        <v>3042.9</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>44.33</v>
+        <v>47.86</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>42.44</v>
+        <v>42.54</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>53.87</v>
+        <v>53.94</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1530,22 +1410,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>206.77</v>
+        <v>243.8</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>43.53</v>
+        <v>47.2</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>57.51</v>
+        <v>44.26</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>64.18000000000001</v>
+        <v>51.19</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1554,22 +1434,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>923.3</v>
+        <v>1275.4</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>43.45</v>
+        <v>45.13</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>48.93</v>
+        <v>49.98</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>62.46</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1578,22 +1458,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>889.4</v>
+        <v>10063</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>42.66</v>
+        <v>44.92</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>44.26</v>
+        <v>57.47</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>52.09</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1602,22 +1482,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1386.2</v>
+        <v>285.1</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>42.56</v>
+        <v>44.78</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>59.35</v>
+        <v>35.7</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>59.37</v>
+        <v>36.29</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1626,22 +1506,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1782.2</v>
+        <v>1429.2</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>42.26</v>
+        <v>44.61</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>53.25</v>
+        <v>47.33</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>57.67</v>
+        <v>50.15</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1650,22 +1530,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1154.7</v>
+        <v>11117</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>41.06</v>
+        <v>44.37</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>32.64</v>
+        <v>43.54</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>39.92</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1674,22 +1554,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>747.05</v>
+        <v>1293</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>41.06</v>
+        <v>42.08</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>29.38</v>
+        <v>40.3</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>39.07</v>
+        <v>46.16</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1698,22 +1578,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1798.2</v>
+        <v>1375.7</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>40.47</v>
+        <v>41.76</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>41.54</v>
+        <v>57.7</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>55.29</v>
+        <v>58.69</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1722,22 +1602,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1130.9</v>
+        <v>1689.1</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>40.01</v>
+        <v>41.33</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>50.03</v>
+        <v>39.1</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>54.83</v>
+        <v>45.13</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1746,22 +1626,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>2121.5</v>
+        <v>197.86</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>39.62</v>
+        <v>41.03</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>39.87</v>
+        <v>53.48</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>43.18</v>
+        <v>62.12</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1770,22 +1650,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>2198.9</v>
+        <v>1116.4</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>39.13</v>
+        <v>40.7</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>29.71</v>
+        <v>34.83</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>32.03</v>
+        <v>35.69</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1794,22 +1674,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>4835</v>
+        <v>406.5</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>39.1</v>
+        <v>40.02</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>42</v>
+        <v>45.17</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>52.67</v>
+        <v>60.32</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1818,22 +1698,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>408.2</v>
+        <v>2161.4</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>37.83</v>
+        <v>38.44</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>45.68</v>
+        <v>28.56</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>60.65</v>
+        <v>31.53</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1842,22 +1722,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1782.8</v>
+        <v>1021.6</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>37.36</v>
+        <v>38.24</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>41.61</v>
+        <v>56.7</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>53.02</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1866,22 +1746,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1703.2</v>
+        <v>284.8</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>36.61</v>
+        <v>37.65</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>39.87</v>
+        <v>45.68</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>45.61</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1890,22 +1770,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>280.7</v>
+        <v>443.5</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>35.81</v>
+        <v>37.48</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>32.74</v>
+        <v>52.2</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>35.16</v>
+        <v>62.01</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1914,22 +1794,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>285.65</v>
+        <v>1100.7</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>35.3</v>
+        <v>34.19</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>46.15</v>
+        <v>46.39</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>53.82</v>
+        <v>52.68</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1938,22 +1818,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>575.3</v>
+        <v>1109.6</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>34.53</v>
+        <v>33.29</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>34.26</v>
+        <v>30.15</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>39.22</v>
+        <v>38.47</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1962,22 +1842,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1291</v>
+        <v>180.14</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>33.29</v>
+        <v>32.77</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>39.75</v>
+        <v>32.58</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>46.06</v>
+        <v>37.6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1986,22 +1866,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>264.75</v>
+        <v>555.35</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>32.91</v>
+        <v>32.5</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>48.67</v>
+        <v>31.65</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>57.36</v>
+        <v>37.62</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2010,22 +1890,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>10912</v>
+        <v>1706</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>32.4</v>
+        <v>27.63</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>40.83</v>
+        <v>37.16</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>48.67</v>
+        <v>49.32</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2034,22 +1914,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>5120.5</v>
+        <v>353.9</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>30.35</v>
+        <v>27.23</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>31.55</v>
+        <v>43.3</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>46.53</v>
+        <v>55.1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2058,16 +1938,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>361.65</v>
+        <v>246.2</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>28.2</v>
+        <v>22.68</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>46.32</v>
+        <v>41.8</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>57.02</v>
+        <v>52.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-06-20
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>8498</v>
+        <v>3038.4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>67.20999999999999</v>
+        <v>69.28</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>71.15000000000001</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>66.56</v>
+        <v>59.11</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>56.19</v>
+        <v>21.49</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>7674.62</v>
+        <v>2440.12</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>7582.51</v>
+        <v>2422.81</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>464871</v>
+        <v>2592381</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>122188</v>
+        <v>416865</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>3105.5</v>
+        <v>8489.5</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>60.64</v>
+        <v>63.56</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>64.48999999999999</v>
+        <v>66.34999999999999</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>63.97</v>
+        <v>66.5</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>47.06</v>
+        <v>56.13</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2851.26</v>
+        <v>7723.84</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>2824.54</v>
+        <v>7624.24</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>913440</v>
+        <v>434741</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>210607</v>
+        <v>122066</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,70 +624,148 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1812.9</v>
+        <v>3149.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>58.97</v>
+        <v>63.06</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>71.78</v>
+        <v>66.22</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>67.17</v>
+        <v>65.09</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>52.62</v>
+        <v>57.29</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1561.38</v>
+        <v>2870.52</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1526.45</v>
+        <v>2840.38</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>2728423</v>
+        <v>898160</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>417685</v>
+        <v>213591</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1835.3</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>61.18</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>72.37</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>35.72</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>1578.58</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>1541.49</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>2380638</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>422846</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1414.8</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>52.96</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>61.94</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>61.28</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>1321</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1300.06</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>1964791</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>272818</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>JSWSTEEL</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>1297.6</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>55.65</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>63.7</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>66.88</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>44.55</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>1208.6</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>1185.45</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>1739195</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>316722</v>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>1287.7</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>61.63</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>66.42</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>46.75</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>1213.71</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>1190.43</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>1695975</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>314305</v>
       </c>
     </row>
   </sheetData>
@@ -696,6 +774,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -753,7 +833,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -762,22 +842,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1356.3</v>
+        <v>3205.8</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>67.98</v>
+        <v>75.26000000000001</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>58.97</v>
+        <v>54.21</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>60.42</v>
+        <v>43.66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -786,22 +866,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>2747.4</v>
+        <v>1094.75</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>67.81999999999999</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>63.47</v>
+        <v>57.23</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>53.79</v>
+        <v>56.03</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -810,22 +890,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>403.3</v>
+        <v>5021.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>67.58</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>54.09</v>
+        <v>57.57</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>52.6</v>
+        <v>55.45</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -834,16 +914,16 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>8498</v>
+        <v>3038.4</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>67.20999999999999</v>
+        <v>69.28</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>71.15000000000001</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>66.56</v>
+        <v>59.11</v>
       </c>
     </row>
     <row r="6">
@@ -858,22 +938,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1340.8</v>
+        <v>1346.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>67.01000000000001</v>
+        <v>66.42</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>53.7</v>
+        <v>54.37</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>56.76</v>
+        <v>57.13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -882,22 +962,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>4709.7</v>
+        <v>4209.4</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>62.38</v>
+        <v>66.3</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>50.98</v>
+        <v>59.66</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>52.22</v>
+        <v>61.54</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -906,22 +986,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1017.15</v>
+        <v>7611</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>61.49</v>
+        <v>64.61</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>52.42</v>
+        <v>58.44</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>59.69</v>
+        <v>66.56999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -930,22 +1010,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2921.6</v>
+        <v>1357.9</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>61.44</v>
+        <v>64.58</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>68.72</v>
+        <v>59.11</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>57.56</v>
+        <v>60.49</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -954,22 +1034,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3105.5</v>
+        <v>1910.8</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>60.64</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>64.48999999999999</v>
+        <v>51.65</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>63.97</v>
+        <v>60.39</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -978,22 +1058,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1812.9</v>
+        <v>1035.1</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>58.97</v>
+        <v>63.97</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>71.78</v>
+        <v>54.64</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>67.17</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1002,22 +1082,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>390</v>
+        <v>8489.5</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>58.33</v>
+        <v>63.56</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>51.35</v>
+        <v>66.34999999999999</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>38.9</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,22 +1106,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4049.3</v>
+        <v>4419.9</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>58.28</v>
+        <v>63.39</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>55.33</v>
+        <v>58.53</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>59.2</v>
+        <v>61.53</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1050,22 +1130,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>7312</v>
+        <v>961.8</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>57.44</v>
+        <v>63.14</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>54.01</v>
+        <v>54.12</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>64.56999999999999</v>
+        <v>56.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1074,22 +1154,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1389.4</v>
+        <v>3149.5</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>56.89</v>
+        <v>63.06</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>54.49</v>
+        <v>66.22</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>50.72</v>
+        <v>65.09</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1098,22 +1178,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>13366</v>
+        <v>264.3</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>56.81</v>
+        <v>62.24</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>45.11</v>
+        <v>52.27</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>52.08</v>
+        <v>55.59</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1122,22 +1202,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1297.6</v>
+        <v>2732.9</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>55.65</v>
+        <v>62.03</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>63.7</v>
+        <v>62.37</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>66.88</v>
+        <v>53.51</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1146,22 +1226,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>772.45</v>
+        <v>1001.9</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>55.31</v>
+        <v>61.42</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>36.7</v>
+        <v>56.73</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>41.91</v>
+        <v>66.52</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1170,22 +1250,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>954.95</v>
+        <v>779.8</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>54.4</v>
+        <v>61.21</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>52.24</v>
+        <v>41.88</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>64.62</v>
+        <v>43.99</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1194,22 +1274,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>918.3</v>
+        <v>1835.3</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>54.09</v>
+        <v>61.18</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>48.48</v>
+        <v>72.37</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>53.92</v>
+        <v>67.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1218,22 +1298,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1012.45</v>
+        <v>1838.3</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>53.58</v>
+        <v>59.31</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>48.01</v>
+        <v>57.79</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>52.03</v>
+        <v>60.06</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1242,22 +1322,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>4184</v>
+        <v>399.25</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>51.53</v>
+        <v>59.3</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>51.74</v>
+        <v>52.27</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>58.71</v>
+        <v>51.88</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1266,22 +1346,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1807.7</v>
+        <v>426.9</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>50.66</v>
+        <v>58.18</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>55.35</v>
+        <v>52.1</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>58.92</v>
+        <v>63.03</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1290,22 +1370,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>2168.8</v>
+        <v>244.45</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>49.17</v>
+        <v>57.68</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>43.74</v>
+        <v>44.44</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>44.6</v>
+        <v>43.94</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1314,22 +1394,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>235.89</v>
+        <v>292.5</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>49.08</v>
+        <v>55.15</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>38.31</v>
+        <v>40.45</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>42.13</v>
+        <v>38.12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1338,22 +1418,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>2755.3</v>
+        <v>591.85</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>48.9</v>
+        <v>54.19</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>41.32</v>
+        <v>41.01</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>39.55</v>
+        <v>40.84</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1362,22 +1442,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1822.5</v>
+        <v>1769.4</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>48.72</v>
+        <v>54.03</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>43.92</v>
+        <v>45.54</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>56.67</v>
+        <v>47.99</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1386,22 +1466,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>3042.9</v>
+        <v>13395</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>47.86</v>
+        <v>53.08</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>42.54</v>
+        <v>45.43</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>53.94</v>
+        <v>52.21</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1410,22 +1490,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>243.8</v>
+        <v>1414.8</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>47.2</v>
+        <v>52.96</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>44.26</v>
+        <v>61.94</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>51.19</v>
+        <v>61.28</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1434,22 +1514,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1275.4</v>
+        <v>2194.6</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>45.13</v>
+        <v>52.3</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>49.98</v>
+        <v>45.79</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>54</v>
+        <v>45.48</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1458,22 +1538,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>10063</v>
+        <v>1287.7</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>44.92</v>
+        <v>51.8</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>57.47</v>
+        <v>61.63</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>62.2</v>
+        <v>66.42</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1482,22 +1562,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>285.1</v>
+        <v>11367</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>44.78</v>
+        <v>51.24</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>35.7</v>
+        <v>46.75</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>36.29</v>
+        <v>51.82</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1506,22 +1586,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1429.2</v>
+        <v>292.25</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>44.61</v>
+        <v>50.23</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>47.33</v>
+        <v>50.48</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>50.15</v>
+        <v>55.47</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1530,22 +1610,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>11117</v>
+        <v>1800.2</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>44.37</v>
+        <v>49.63</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>43.54</v>
+        <v>44.94</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>50.04</v>
+        <v>53.93</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1554,22 +1634,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1293</v>
+        <v>3074.8</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>42.08</v>
+        <v>49.18</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>40.3</v>
+        <v>43.94</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>46.16</v>
+        <v>54.67</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1578,22 +1658,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1375.7</v>
+        <v>1309.5</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>41.76</v>
+        <v>46.8</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>57.7</v>
+        <v>42.48</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>58.69</v>
+        <v>47.02</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1602,22 +1682,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1689.1</v>
+        <v>10066</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>41.33</v>
+        <v>46.71</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>39.1</v>
+        <v>57.51</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>45.13</v>
+        <v>62.23</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1626,22 +1706,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>197.86</v>
+        <v>365.8</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>41.03</v>
+        <v>45.87</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>53.48</v>
+        <v>48.81</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>62.12</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1650,22 +1730,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1116.4</v>
+        <v>1351.8</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>40.7</v>
+        <v>45.01</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>34.83</v>
+        <v>48.89</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>35.69</v>
+        <v>48.56</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1674,22 +1754,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>406.5</v>
+        <v>198.96</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>40.02</v>
+        <v>44.75</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>45.17</v>
+        <v>54.02</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>60.32</v>
+        <v>62.59</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1698,22 +1778,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>2161.4</v>
+        <v>1272.1</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>38.44</v>
+        <v>44.74</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>28.56</v>
+        <v>49.47</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>31.53</v>
+        <v>53.74</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1722,22 +1802,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1021.6</v>
+        <v>451.3</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>38.24</v>
+        <v>44.7</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>56.7</v>
+        <v>54.32</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>65.40000000000001</v>
+        <v>63.85</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1746,22 +1826,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>284.8</v>
+        <v>359.5</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>37.65</v>
+        <v>43</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>45.68</v>
+        <v>44.77</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>53.6</v>
+        <v>37.51</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1770,22 +1850,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>443.5</v>
+        <v>1409.6</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>37.48</v>
+        <v>42.3</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>52.2</v>
+        <v>45.96</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>62.01</v>
+        <v>49.39</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1794,22 +1874,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1100.7</v>
+        <v>1131.7</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>34.19</v>
+        <v>41.69</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>46.39</v>
+        <v>32.86</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>52.68</v>
+        <v>39.17</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1818,22 +1898,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>1109.6</v>
+        <v>1111.5</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>33.29</v>
+        <v>40.74</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>30.15</v>
+        <v>47.85</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>38.47</v>
+        <v>53.43</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1842,22 +1922,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>180.14</v>
+        <v>1010</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>32.77</v>
+        <v>39.6</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>32.58</v>
+        <v>55.12</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>37.6</v>
+        <v>64.51000000000001</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1866,22 +1946,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>555.35</v>
+        <v>2125</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>32.5</v>
+        <v>37.21</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>31.65</v>
+        <v>27.45</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>37.62</v>
+        <v>31.05</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1890,22 +1970,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>1706</v>
+        <v>180.8</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>27.63</v>
+        <v>35.92</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>37.16</v>
+        <v>33.09</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>49.32</v>
+        <v>37.73</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1914,16 +1994,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>353.9</v>
+        <v>1051.4</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>27.23</v>
+        <v>33.21</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>43.3</v>
+        <v>31.21</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>55.1</v>
+        <v>33.65</v>
       </c>
     </row>
     <row r="51">
@@ -1938,16 +2018,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>246.2</v>
+        <v>246.25</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>22.68</v>
+        <v>28.76</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>41.8</v>
+        <v>41.82</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>52.2</v>
+        <v>52.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-06-27
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>3038.4</v>
+        <v>8592</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>69.28</v>
+        <v>67.69</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>71.15000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>59.11</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>21.49</v>
+        <v>46.06</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>2440.12</v>
+        <v>7765.72</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>2422.81</v>
+        <v>7659.53</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>2592381</v>
+        <v>422049</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>416865</v>
+        <v>123439</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,31 +585,31 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>8489.5</v>
+        <v>3038</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>63.56</v>
+        <v>62.15</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>66.34999999999999</v>
+        <v>71.19</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>66.5</v>
+        <v>59.14</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>56.13</v>
+        <v>28.73</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>7723.84</v>
+        <v>2470.78</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>7624.24</v>
+        <v>2446.11</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>434741</v>
+        <v>2368400</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>122066</v>
+        <v>417125</v>
       </c>
     </row>
     <row r="4">
@@ -624,31 +624,31 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>3149.5</v>
+        <v>3126.6</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>63.06</v>
+        <v>56.51</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>66.22</v>
+        <v>64.7</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>65.09</v>
+        <v>64.72</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>57.29</v>
+        <v>58.1</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>2870.52</v>
+        <v>2884.81</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>2840.38</v>
+        <v>2852.96</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>898160</v>
+        <v>849696</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>213591</v>
+        <v>212261</v>
       </c>
     </row>
     <row r="5">
@@ -663,31 +663,31 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1835.3</v>
+        <v>1796</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>61.18</v>
+        <v>51.46</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>72.37</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>67.7</v>
+        <v>66.69</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>35.72</v>
+        <v>41.46</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1578.58</v>
+        <v>1590.36</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>1541.49</v>
+        <v>1551.95</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>2380638</v>
+        <v>2220783</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>422846</v>
+        <v>413561</v>
       </c>
     </row>
     <row r="6">
@@ -702,70 +702,31 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1414.8</v>
+        <v>1402.6</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>52.96</v>
+        <v>50.19</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>61.94</v>
+        <v>61.1</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>61.28</v>
+        <v>60.93</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>47</v>
+        <v>40.58</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1321</v>
+        <v>1324.83</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1300.06</v>
+        <v>1303.8</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1964791</v>
+        <v>1989179</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>272818</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>JSWSTEEL</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>1287.7</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>61.63</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>66.42</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>46.75</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>1213.71</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>1190.43</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>1695975</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>314305</v>
+        <v>271854</v>
       </c>
     </row>
   </sheetData>
@@ -775,7 +736,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -833,7 +793,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -842,16 +802,16 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>3205.8</v>
+        <v>5450</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.26000000000001</v>
+        <v>78.63</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>54.21</v>
+        <v>64.78</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>43.66</v>
+        <v>59.34</v>
       </c>
     </row>
     <row r="3">
@@ -866,22 +826,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1094.75</v>
+        <v>1123.35</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>71.01000000000001</v>
+        <v>72.33</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>57.23</v>
+        <v>59.85</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>56.03</v>
+        <v>57.25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -890,22 +850,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>5021.5</v>
+        <v>1387.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>70.95999999999999</v>
+        <v>71.20999999999999</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>57.57</v>
+        <v>58.92</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>55.45</v>
+        <v>59.57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -914,22 +874,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>3038.4</v>
+        <v>3216.2</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>69.28</v>
+        <v>69.92</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>71.15000000000001</v>
+        <v>54.42</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>59.11</v>
+        <v>43.74</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -938,22 +898,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1346.5</v>
+        <v>1350.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>66.42</v>
+        <v>69.78</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>54.37</v>
+        <v>59.77</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>57.13</v>
+        <v>59.15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -962,22 +922,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>4209.4</v>
+        <v>8592</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>66.3</v>
+        <v>67.69</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>59.66</v>
+        <v>67.8</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>61.54</v>
+        <v>67.15000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -986,22 +946,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>7611</v>
+        <v>1377.2</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>64.61</v>
+        <v>66.97</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>58.44</v>
+        <v>60.92</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>66.56999999999999</v>
+        <v>61.29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1010,22 +970,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1357.9</v>
+        <v>409</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>64.58</v>
+        <v>66.66</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>59.11</v>
+        <v>56.37</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>60.49</v>
+        <v>53.71</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1034,22 +994,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1910.8</v>
+        <v>1440.1</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>64.09999999999999</v>
+        <v>66.36</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>51.65</v>
+        <v>59.35</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>60.39</v>
+        <v>53.45</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1058,22 +1018,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1035.1</v>
+        <v>1031.8</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>63.97</v>
+        <v>66.22</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>54.64</v>
+        <v>59.27</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>60.5</v>
+        <v>67.59</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1082,22 +1042,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>8489.5</v>
+        <v>4216.4</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>63.56</v>
+        <v>65.45</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>66.34999999999999</v>
+        <v>59.38</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>66.5</v>
+        <v>61.44</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1106,16 +1066,16 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4419.9</v>
+        <v>796.3</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>63.39</v>
+        <v>64.37</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>58.53</v>
+        <v>45.96</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>61.53</v>
+        <v>45.57</v>
       </c>
     </row>
     <row r="14">
@@ -1130,22 +1090,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>961.8</v>
+        <v>980.4</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>63.14</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>54.12</v>
+        <v>56.43</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>56.3</v>
+        <v>57.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1154,22 +1114,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>3149.5</v>
+        <v>1045.4</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>63.06</v>
+        <v>63.87</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>66.22</v>
+        <v>55.89</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>65.09</v>
+        <v>60.94</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1178,22 +1138,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>264.3</v>
+        <v>1862.8</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>62.24</v>
+        <v>62.56</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>52.27</v>
+        <v>59.6</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>55.59</v>
+        <v>60.89</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1202,22 +1162,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>2732.9</v>
+        <v>7598</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>62.03</v>
+        <v>62.52</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>62.37</v>
+        <v>58.22</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>53.51</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1226,22 +1186,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1001.9</v>
+        <v>3038</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>61.42</v>
+        <v>62.15</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>56.73</v>
+        <v>71.19</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>66.52</v>
+        <v>59.14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1250,22 +1210,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>779.8</v>
+        <v>13745</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>61.21</v>
+        <v>60.48</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>41.88</v>
+        <v>49.38</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>43.99</v>
+        <v>53.76</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1274,22 +1234,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1835.3</v>
+        <v>3182.2</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>61.18</v>
+        <v>59.15</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>72.37</v>
+        <v>48.61</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>67.7</v>
+        <v>57.01</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1298,22 +1258,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1838.3</v>
+        <v>3126.6</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>59.31</v>
+        <v>56.51</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>57.79</v>
+        <v>64.7</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>60.06</v>
+        <v>64.72</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1322,22 +1282,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>399.25</v>
+        <v>11489</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>59.3</v>
+        <v>54.99</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>52.27</v>
+        <v>47.88</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>51.88</v>
+        <v>52.48</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1346,22 +1306,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>426.9</v>
+        <v>4291.3</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>58.18</v>
+        <v>53.14</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>52.1</v>
+        <v>54.02</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>63.03</v>
+        <v>60.03</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1370,22 +1330,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>244.45</v>
+        <v>2174.2</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>57.68</v>
+        <v>52.82</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>44.44</v>
+        <v>46.17</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>43.94</v>
+        <v>45.63</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1394,22 +1354,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>292.5</v>
+        <v>255.15</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>55.15</v>
+        <v>52.74</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>40.45</v>
+        <v>48.84</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>38.12</v>
+        <v>53.73</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1418,22 +1378,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>591.85</v>
+        <v>1764.6</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>54.19</v>
+        <v>52.16</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>41.01</v>
+        <v>45.38</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>40.84</v>
+        <v>47.9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1442,22 +1402,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1769.4</v>
+        <v>1796</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>54.03</v>
+        <v>51.46</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>45.54</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>47.99</v>
+        <v>66.69</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1466,22 +1426,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>13395</v>
+        <v>290</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>53.08</v>
+        <v>50.76</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>45.43</v>
+        <v>39.39</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>52.21</v>
+        <v>37.52</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1490,22 +1450,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1414.8</v>
+        <v>239.43</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>52.96</v>
+        <v>50.75</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>61.94</v>
+        <v>41.6</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>61.28</v>
+        <v>42.67</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1514,22 +1474,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>2194.6</v>
+        <v>1402.6</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>52.3</v>
+        <v>50.19</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>45.79</v>
+        <v>61.1</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>45.48</v>
+        <v>60.93</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1538,22 +1498,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1287.7</v>
+        <v>1131.3</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>51.8</v>
+        <v>50.03</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>61.63</v>
+        <v>50.54</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>66.42</v>
+        <v>54.88</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1562,22 +1522,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>11367</v>
+        <v>2645.2</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>51.24</v>
+        <v>49.93</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>46.75</v>
+        <v>57.18</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>51.82</v>
+        <v>52.08</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1586,22 +1546,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>292.25</v>
+        <v>585.45</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>50.23</v>
+        <v>49.77</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>50.48</v>
+        <v>39.81</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>55.47</v>
+        <v>40.21</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1610,22 +1570,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1800.2</v>
+        <v>1318.1</v>
       </c>
       <c r="D34" s="4" t="n">
         <v>49.63</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>44.94</v>
+        <v>43.43</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>53.93</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1634,22 +1594,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>3074.8</v>
+        <v>1850.7</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>49.18</v>
+        <v>49.45</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>43.94</v>
+        <v>46.85</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>54.67</v>
+        <v>57.96</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1658,22 +1618,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1309.5</v>
+        <v>1437.1</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>46.8</v>
+        <v>47.82</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>42.48</v>
+        <v>48.43</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>47.02</v>
+        <v>50.57</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1682,22 +1642,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>10066</v>
+        <v>407.2</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>46.71</v>
+        <v>42.36</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>57.51</v>
+        <v>46.4</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>62.23</v>
+        <v>60.7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1706,22 +1666,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>365.8</v>
+        <v>353.2</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>45.87</v>
+        <v>41.23</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>48.81</v>
+        <v>43.3</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>58.1</v>
+        <v>37.17</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1730,22 +1690,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1351.8</v>
+        <v>9843</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>45.01</v>
+        <v>40.93</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>48.89</v>
+        <v>53.58</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>48.56</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1754,22 +1714,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>198.96</v>
+        <v>283.9</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>44.75</v>
+        <v>39.61</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>54.02</v>
+        <v>45.93</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>62.59</v>
+        <v>53.53</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1778,22 +1738,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1272.1</v>
+        <v>1744.9</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>44.74</v>
+        <v>39.4</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>49.47</v>
+        <v>41.52</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>53.74</v>
+        <v>50.99</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1802,22 +1762,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>451.3</v>
+        <v>2094.7</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>44.7</v>
+        <v>37.84</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>54.32</v>
+        <v>26.56</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>63.85</v>
+        <v>30.68</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1826,22 +1786,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>359.5</v>
+        <v>1231</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>43</v>
+        <v>36.52</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>44.77</v>
+        <v>51.4</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>37.51</v>
+        <v>61.87</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1850,22 +1810,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1409.6</v>
+        <v>1100.7</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>42.3</v>
+        <v>36.26</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>45.96</v>
+        <v>31.03</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>49.39</v>
+        <v>38.19</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1874,22 +1834,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1131.7</v>
+        <v>1041.2</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>41.69</v>
+        <v>36.1</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>32.86</v>
+        <v>30.75</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>39.17</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1898,22 +1858,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>1111.5</v>
+        <v>352.05</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>40.74</v>
+        <v>35.3</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>47.85</v>
+        <v>43.7</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>53.43</v>
+        <v>54.77</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1922,22 +1882,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1010</v>
+        <v>435.4</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>39.6</v>
+        <v>34.38</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>55.12</v>
+        <v>49.56</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>64.51000000000001</v>
+        <v>60.25</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1946,16 +1906,16 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>2125</v>
+        <v>188.71</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>37.21</v>
+        <v>31.65</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>27.45</v>
+        <v>46.74</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>31.05</v>
+        <v>58.47</v>
       </c>
     </row>
     <row r="49">
@@ -1970,22 +1930,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>180.8</v>
+        <v>175</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>35.92</v>
+        <v>31.2</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>33.09</v>
+        <v>30.91</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>37.73</v>
+        <v>36.64</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1994,16 +1954,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1051.4</v>
+        <v>953.2</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>33.21</v>
+        <v>30.56</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>31.21</v>
+        <v>47.93</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>33.65</v>
+        <v>60.38</v>
       </c>
     </row>
     <row r="51">
@@ -2018,16 +1978,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>246.25</v>
+        <v>233.1</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>28.76</v>
+        <v>20.87</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>41.82</v>
+        <v>37.49</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>52.21</v>
+        <v>49.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-07-04
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>8592</v>
+        <v>8893.5</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>67.69</v>
+        <v>75.92</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>67.8</v>
+        <v>71.98</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>67.15000000000001</v>
+        <v>69.11</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>46.06</v>
+        <v>26.8</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>7765.72</v>
+        <v>7836.95</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>7659.53</v>
+        <v>7719.96</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>422049</v>
+        <v>356931</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>123439</v>
+        <v>127875</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>3038</v>
+        <v>1904.8</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>62.15</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>71.19</v>
+        <v>62.79</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>59.14</v>
+        <v>62.41</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>28.73</v>
+        <v>35.19</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2470.78</v>
+        <v>1770.15</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>2446.11</v>
+        <v>1755.59</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>2368400</v>
+        <v>2289588</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>417125</v>
+        <v>457025</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,31 +624,31 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>3126.6</v>
+        <v>3212.1</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>56.51</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>64.7</v>
+        <v>74.62</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>64.72</v>
+        <v>61.28</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>58.1</v>
+        <v>35.36</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>2884.81</v>
+        <v>2518.93</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>2852.96</v>
+        <v>2484.12</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>849696</v>
+        <v>2254662</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>212261</v>
+        <v>440696</v>
       </c>
     </row>
     <row r="5">
@@ -663,70 +663,109 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1796</v>
+        <v>1874.2</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>51.46</v>
+        <v>62.62</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>67.29000000000001</v>
+        <v>72</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>66.69</v>
+        <v>68.59</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>41.46</v>
+        <v>39.33</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1590.36</v>
+        <v>1609</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>1551.95</v>
+        <v>1568.55</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>2220783</v>
+        <v>2151523</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>413561</v>
+        <v>431808</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>3180.9</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>62.61</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>66.72</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>65.38</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>2904.17</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>2870.54</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>645240</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>215720</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>NESTLEIND</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>1402.6</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>50.19</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>61.1</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>60.93</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>40.58</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>1324.83</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>1303.8</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>1989179</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>271854</v>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>1459.8</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>62.41</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>65.45999999999999</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>63.12</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>25.77</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>1332.65</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>1310.99</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>2010939</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>281495</v>
       </c>
     </row>
   </sheetData>
@@ -736,6 +775,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -793,7 +833,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -802,22 +842,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>5450</v>
+        <v>8893.5</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>78.63</v>
+        <v>75.92</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>64.78</v>
+        <v>71.98</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>59.34</v>
+        <v>69.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -826,22 +866,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1123.35</v>
+        <v>3340.6</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>72.33</v>
+        <v>75.47</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>59.85</v>
+        <v>57.45</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>57.25</v>
+        <v>44.88</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -850,22 +890,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1387.5</v>
+        <v>1031.4</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>71.20999999999999</v>
+        <v>75.15000000000001</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>58.92</v>
+        <v>62.32</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>59.57</v>
+        <v>59.99</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -874,22 +914,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>3216.2</v>
+        <v>1063.6</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>69.92</v>
+        <v>73.09</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>54.42</v>
+        <v>62.42</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>43.74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -898,22 +938,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1350.5</v>
+        <v>1411.4</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>69.78</v>
+        <v>72.87</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>59.77</v>
+        <v>61.43</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>59.15</v>
+        <v>61.01</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -922,22 +962,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>8592</v>
+        <v>5426.5</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>67.69</v>
+        <v>72.16</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>67.8</v>
+        <v>63.99</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>67.15000000000001</v>
+        <v>59.08</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -946,22 +986,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1377.2</v>
+        <v>281.65</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>66.97</v>
+        <v>71.33</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>60.92</v>
+        <v>57.46</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>61.29</v>
+        <v>58.92</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -970,22 +1010,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>409</v>
+        <v>1895.6</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>66.66</v>
+        <v>70.94</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>56.37</v>
+        <v>54.4</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>53.71</v>
+        <v>53.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -994,22 +1034,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1440.1</v>
+        <v>1153.4</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>66.36</v>
+        <v>70.31</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>59.35</v>
+        <v>62.69</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>53.45</v>
+        <v>58.66</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1018,22 +1058,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1031.8</v>
+        <v>1904.8</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>66.22</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>59.27</v>
+        <v>62.79</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>67.59</v>
+        <v>62.41</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1042,22 +1082,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>4216.4</v>
+        <v>3212.1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>65.45</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>59.38</v>
+        <v>74.62</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>61.44</v>
+        <v>61.28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1066,22 +1106,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>796.3</v>
+        <v>1458.2</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>64.37</v>
+        <v>67.61</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>45.96</v>
+        <v>60.64</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>45.57</v>
+        <v>54.27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1090,22 +1130,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>980.4</v>
+        <v>1374.1</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>64.18000000000001</v>
+        <v>67.12</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>56.43</v>
+        <v>62.39</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>57.3</v>
+        <v>60.56</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1114,22 +1154,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1045.4</v>
+        <v>14366</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>63.87</v>
+        <v>66.54000000000001</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>55.89</v>
+        <v>55.35</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>60.94</v>
+        <v>56.26</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1138,22 +1178,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1862.8</v>
+        <v>801.05</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>62.56</v>
+        <v>65.41</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>59.6</v>
+        <v>46.95</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>60.89</v>
+        <v>46.03</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1162,22 +1202,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>7598</v>
+        <v>4461.1</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>62.52</v>
+        <v>62.63</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>58.22</v>
+        <v>58.56</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>66.5</v>
+        <v>62.06</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1186,22 +1226,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>3038</v>
+        <v>1874.2</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>62.15</v>
+        <v>62.62</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>71.19</v>
+        <v>72</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>59.14</v>
+        <v>68.59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1210,22 +1250,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>13745</v>
+        <v>3180.9</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>60.48</v>
+        <v>62.61</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>49.38</v>
+        <v>66.72</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>53.76</v>
+        <v>65.38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1234,22 +1274,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>3182.2</v>
+        <v>1459.8</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>59.15</v>
+        <v>62.41</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>48.61</v>
+        <v>65.45999999999999</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>57.01</v>
+        <v>63.12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1258,22 +1298,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>3126.6</v>
+        <v>2737.8</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>56.51</v>
+        <v>62.35</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>64.7</v>
+        <v>62.11</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>64.72</v>
+        <v>54.13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1282,22 +1322,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>11489</v>
+        <v>1910.4</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>54.99</v>
+        <v>61.59</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>47.88</v>
+        <v>51.65</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>52.48</v>
+        <v>60.52</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1306,22 +1346,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>4291.3</v>
+        <v>11723</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>53.14</v>
+        <v>61.16</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>54.02</v>
+        <v>51.22</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>60.03</v>
+        <v>54.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1330,22 +1370,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>2174.2</v>
+        <v>1040</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>52.82</v>
+        <v>57.33</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>46.17</v>
+        <v>54.97</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>45.63</v>
+        <v>61.05</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1354,22 +1394,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>255.15</v>
+        <v>2201.2</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>52.74</v>
+        <v>56.23</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>48.84</v>
+        <v>48.22</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>53.73</v>
+        <v>46.63</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1378,22 +1418,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1764.6</v>
+        <v>3136.9</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>52.16</v>
+        <v>55.58</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>45.38</v>
+        <v>48.03</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>47.9</v>
+        <v>56.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1402,22 +1442,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1796</v>
+        <v>418.05</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>51.46</v>
+        <v>51.81</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>67.29000000000001</v>
+        <v>49.52</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>66.69</v>
+        <v>62.18</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1426,22 +1466,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>290</v>
+        <v>1139</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>50.76</v>
+        <v>51.74</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>39.39</v>
+        <v>35.15</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>37.52</v>
+        <v>40.36</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1450,22 +1490,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>239.43</v>
+        <v>1342.1</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>50.75</v>
+        <v>51.44</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>41.6</v>
+        <v>56.06</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>42.67</v>
+        <v>59.71</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1474,22 +1514,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1402.6</v>
+        <v>396.75</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>50.19</v>
+        <v>51.04</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>61.1</v>
+        <v>50.61</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>60.93</v>
+        <v>51.48</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1498,22 +1538,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1131.3</v>
+        <v>1410.1</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>50.03</v>
+        <v>50.94</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>50.54</v>
+        <v>49.16</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>54.88</v>
+        <v>50.9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1522,22 +1562,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>2645.2</v>
+        <v>239.35</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>49.93</v>
+        <v>50.94</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>57.18</v>
+        <v>41.78</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>52.08</v>
+        <v>42.95</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1546,22 +1586,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>585.45</v>
+        <v>289.95</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>49.77</v>
+        <v>50.72</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>39.81</v>
+        <v>39.19</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>40.21</v>
+        <v>35.91</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1570,22 +1610,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1318.1</v>
+        <v>1788.7</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>49.63</v>
+        <v>50.37</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>43.43</v>
+        <v>45.07</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>47.4</v>
+        <v>53.26</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1594,22 +1634,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1850.7</v>
+        <v>7339.5</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>49.45</v>
+        <v>49.88</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>46.85</v>
+        <v>53.07</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>57.96</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1618,22 +1658,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1437.1</v>
+        <v>1116.7</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>47.82</v>
+        <v>48.47</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>48.43</v>
+        <v>48.48</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>50.57</v>
+        <v>53.47</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1642,22 +1682,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>407.2</v>
+        <v>287.85</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>42.36</v>
+        <v>46.5</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>46.4</v>
+        <v>48.07</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>60.7</v>
+        <v>54.11</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1666,22 +1706,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>353.2</v>
+        <v>1304</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>41.23</v>
+        <v>46.28</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>43.3</v>
+        <v>41.92</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>37.17</v>
+        <v>46.82</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1690,22 +1730,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>9843</v>
+        <v>4026.6</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>40.93</v>
+        <v>43.89</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>53.58</v>
+        <v>52.77</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>60.3</v>
+        <v>57.83</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1714,22 +1754,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>283.9</v>
+        <v>2093.5</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>39.61</v>
+        <v>43.84</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>45.93</v>
+        <v>26.72</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>53.53</v>
+        <v>31.89</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1738,22 +1778,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1744.9</v>
+        <v>1047.2</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>39.4</v>
+        <v>42.92</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>41.52</v>
+        <v>31.24</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>50.99</v>
+        <v>34.63</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1762,22 +1802,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>2094.7</v>
+        <v>9785.5</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>37.84</v>
+        <v>42.34</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>26.56</v>
+        <v>52.27</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>30.68</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1786,22 +1826,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1231</v>
+        <v>438.7</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>36.52</v>
+        <v>41.38</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>51.4</v>
+        <v>50.43</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>61.87</v>
+        <v>61.32</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1810,22 +1850,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1100.7</v>
+        <v>356.45</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>36.26</v>
+        <v>41.18</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>31.03</v>
+        <v>45.55</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>38.19</v>
+        <v>55.45</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1834,22 +1874,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1041.2</v>
+        <v>567.7</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>36.1</v>
+        <v>40.31</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>30.75</v>
+        <v>37.36</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>33.4</v>
+        <v>38.75</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1858,22 +1898,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>352.05</v>
+        <v>176.08</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>35.3</v>
+        <v>39.92</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>43.7</v>
+        <v>32.25</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>54.77</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1882,16 +1922,16 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>435.4</v>
+        <v>1230.2</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>34.38</v>
+        <v>39.65</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>49.56</v>
+        <v>51.22</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>60.25</v>
+        <v>61.63</v>
       </c>
     </row>
     <row r="48">
@@ -1906,22 +1946,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>188.71</v>
+        <v>189.8</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>31.65</v>
+        <v>39.59</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>46.74</v>
+        <v>47.17</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>58.47</v>
+        <v>58.62</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1930,16 +1970,16 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>175</v>
+        <v>344.1</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>31.2</v>
+        <v>38.42</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>30.91</v>
+        <v>41.39</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>36.64</v>
+        <v>36.73</v>
       </c>
     </row>
     <row r="50">
@@ -1957,13 +1997,13 @@
         <v>953.2</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>30.56</v>
+        <v>34.96</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>47.93</v>
+        <v>48.06</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>60.38</v>
+        <v>60.43</v>
       </c>
     </row>
     <row r="51">
@@ -1978,16 +2018,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>233.1</v>
+        <v>237.84</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>20.87</v>
+        <v>30.89</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>37.49</v>
+        <v>39.77</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>49.09</v>
+        <v>49.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-07-11
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>8893.5</v>
+        <v>1935.5</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.92</v>
+        <v>71.2</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>71.98</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>69.11</v>
+        <v>63.61</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>26.8</v>
+        <v>24.44</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>7836.95</v>
+        <v>1775.24</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>7719.96</v>
+        <v>1759.42</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>356931</v>
+        <v>2128036</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>127875</v>
+        <v>466023</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1904.8</v>
+        <v>4584.4</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>70.23999999999999</v>
+        <v>67.97</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>62.79</v>
+        <v>61.84</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>62.41</v>
+        <v>63.62</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>35.19</v>
+        <v>23.77</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1770.15</v>
+        <v>4145.58</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>1755.59</v>
+        <v>4067.96</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>2289588</v>
+        <v>923392</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>457025</v>
+        <v>406284</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>3212.1</v>
+        <v>8845.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>69.23999999999999</v>
+        <v>67.47</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>74.62</v>
+        <v>70.3</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>61.28</v>
+        <v>68.77</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>35.36</v>
+        <v>20.76</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>2518.93</v>
+        <v>7888.8</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>2484.12</v>
+        <v>7764.74</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>2254662</v>
+        <v>340585</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>440696</v>
+        <v>127120</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1874.2</v>
+        <v>1020.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>62.62</v>
+        <v>63.72</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>72</v>
+        <v>60.6</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>68.59</v>
+        <v>59.47</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>39.33</v>
+        <v>26.85</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1609</v>
+        <v>940.76</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>1568.55</v>
+        <v>935.92</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>2151523</v>
+        <v>9316862</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>431808</v>
+        <v>634534</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,31 +702,31 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3180.9</v>
+        <v>3157.3</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>62.61</v>
+        <v>60.63</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>66.72</v>
+        <v>71.70999999999999</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>65.38</v>
+        <v>60.62</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>60.4</v>
+        <v>46.04</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2904.17</v>
+        <v>2557.58</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2870.54</v>
+        <v>2514.5</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>645240</v>
+        <v>2091425</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>215720</v>
+        <v>449275</v>
       </c>
     </row>
     <row r="7">
@@ -741,31 +741,70 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1459.8</v>
+        <v>1456.2</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>62.41</v>
+        <v>60.21</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>65.45999999999999</v>
+        <v>65.67</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>63.12</v>
+        <v>63.22</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>25.77</v>
+        <v>21.89</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1332.65</v>
+        <v>1333.14</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1310.99</v>
+        <v>1310.93</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>2010939</v>
+        <v>1720752</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>281495</v>
+        <v>282151</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>1828.1</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>53.06</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>66.48</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>67.47</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>42.83</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>1622.8</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>1580.83</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>2071318</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>421187</v>
       </c>
     </row>
   </sheetData>
@@ -776,6 +815,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -833,7 +873,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -842,22 +882,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>8893.5</v>
+        <v>1935.5</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.92</v>
+        <v>71.2</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>71.98</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>69.11</v>
+        <v>63.61</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -866,22 +906,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>3340.6</v>
+        <v>289.65</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>75.47</v>
+        <v>70.66</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>57.45</v>
+        <v>59.66</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>44.88</v>
+        <v>60.29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -890,22 +930,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1031.4</v>
+        <v>4584.4</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>75.15000000000001</v>
+        <v>67.97</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>62.32</v>
+        <v>61.84</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>59.99</v>
+        <v>63.62</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -914,22 +954,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1063.6</v>
+        <v>8845.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>73.09</v>
+        <v>67.47</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>62.42</v>
+        <v>70.3</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>69</v>
+        <v>68.77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -938,22 +978,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1411.4</v>
+        <v>824.95</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>72.87</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>61.43</v>
+        <v>52.27</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>61.01</v>
+        <v>48.32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -962,22 +1002,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>5426.5</v>
+        <v>1895</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>72.16</v>
+        <v>65.27</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>63.99</v>
+        <v>55.63</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>59.08</v>
+        <v>53.84</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -986,22 +1026,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>281.65</v>
+        <v>1020.5</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>71.33</v>
+        <v>63.72</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>57.46</v>
+        <v>60.6</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>58.92</v>
+        <v>59.47</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1010,22 +1050,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1895.6</v>
+        <v>1862.9</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>70.94</v>
+        <v>62.08</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>54.4</v>
+        <v>50.35</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>53.1</v>
+        <v>56.53</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1034,22 +1074,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1153.4</v>
+        <v>1931.1</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>70.31</v>
+        <v>61.48</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>62.69</v>
+        <v>52.42</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>58.66</v>
+        <v>60.91</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1058,16 +1098,16 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1904.8</v>
+        <v>3213.6</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>70.23999999999999</v>
+        <v>61.44</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>62.79</v>
+        <v>68.04000000000001</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>62.41</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12">
@@ -1082,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3212.1</v>
+        <v>3157.3</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>69.23999999999999</v>
+        <v>60.63</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>74.62</v>
+        <v>71.70999999999999</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>61.28</v>
+        <v>60.62</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1106,22 +1146,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1458.2</v>
+        <v>5312</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>67.61</v>
+        <v>60.58</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>60.64</v>
+        <v>60.89</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>54.27</v>
+        <v>57.86</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1130,22 +1170,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1374.1</v>
+        <v>1456.2</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>67.12</v>
+        <v>60.21</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>62.39</v>
+        <v>65.67</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>60.56</v>
+        <v>63.22</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1154,22 +1194,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>14366</v>
+        <v>1044.1</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>66.54000000000001</v>
+        <v>59.98</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>55.35</v>
+        <v>59.88</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>56.26</v>
+        <v>68.28</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1178,22 +1218,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>801.05</v>
+        <v>11711</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>65.41</v>
+        <v>57.96</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>46.95</v>
+        <v>51.06</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>46.03</v>
+        <v>54.12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1202,22 +1242,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>4461.1</v>
+        <v>1380.7</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>62.63</v>
+        <v>57.59</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>58.56</v>
+        <v>59.79</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>62.06</v>
+        <v>60.42</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1226,22 +1266,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1874.2</v>
+        <v>1441.3</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>62.62</v>
+        <v>57.07</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>72</v>
+        <v>57.94</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>68.59</v>
+        <v>53.12</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1250,22 +1290,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>3180.9</v>
+        <v>1454.8</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>62.61</v>
+        <v>57.02</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>66.72</v>
+        <v>52.77</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>65.38</v>
+        <v>52.62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1274,22 +1314,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1459.8</v>
+        <v>10155</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>62.41</v>
+        <v>55.76</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>65.45999999999999</v>
+        <v>57.8</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>63.12</v>
+        <v>61.18</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1298,22 +1338,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>2737.8</v>
+        <v>1036</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>62.35</v>
+        <v>54.79</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>62.11</v>
+        <v>54.29</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>54.13</v>
+        <v>60.86</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1322,22 +1362,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1910.4</v>
+        <v>1101.3</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>61.59</v>
+        <v>54.52</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>51.65</v>
+        <v>56.66</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>60.52</v>
+        <v>56.38</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1346,22 +1386,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>11723</v>
+        <v>241.96</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>61.16</v>
+        <v>54.05</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>51.22</v>
+        <v>43.77</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>54.2</v>
+        <v>43.59</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1370,22 +1410,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1040</v>
+        <v>1828.1</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>57.33</v>
+        <v>53.06</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>54.97</v>
+        <v>66.48</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>61.05</v>
+        <v>67.47</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1394,22 +1434,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>2201.2</v>
+        <v>1150.4</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>56.23</v>
+        <v>53.05</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>48.22</v>
+        <v>38.24</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>46.63</v>
+        <v>41.55</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1418,22 +1458,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>3136.9</v>
+        <v>13854</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>55.58</v>
+        <v>51.99</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>48.03</v>
+        <v>50.04</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>56.8</v>
+        <v>53.88</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1442,22 +1482,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>418.05</v>
+        <v>2677.8</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>51.81</v>
+        <v>50.66</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>49.52</v>
+        <v>57.78</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>62.18</v>
+        <v>52.87</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1466,22 +1506,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1139</v>
+        <v>7365.5</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>51.74</v>
+        <v>49.89</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>35.15</v>
+        <v>53.51</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>40.36</v>
+        <v>64.48999999999999</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1490,22 +1530,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1342.1</v>
+        <v>1307.8</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>51.44</v>
+        <v>49.65</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>56.06</v>
+        <v>42.5</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>59.71</v>
+        <v>47.05</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1514,22 +1554,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>396.75</v>
+        <v>3085.4</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>51.04</v>
+        <v>49.58</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>50.61</v>
+        <v>47.69</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>51.48</v>
+        <v>56.63</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1538,22 +1578,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1410.1</v>
+        <v>414.85</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>50.94</v>
+        <v>49.49</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>49.16</v>
+        <v>48.53</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>50.9</v>
+        <v>61.76</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1562,22 +1602,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>239.35</v>
+        <v>1068</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>50.94</v>
+        <v>47.85</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>41.78</v>
+        <v>33.98</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>42.95</v>
+        <v>35.81</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1586,22 +1626,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>289.95</v>
+        <v>1323.7</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>50.72</v>
+        <v>47.79</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>39.19</v>
+        <v>53.78</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>35.91</v>
+        <v>58.51</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1610,22 +1650,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1788.7</v>
+        <v>2150.6</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>50.37</v>
+        <v>47.27</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>45.07</v>
+        <v>44.38</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>53.26</v>
+        <v>44.83</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1634,22 +1674,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>7339.5</v>
+        <v>1106.7</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>49.88</v>
+        <v>46.68</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>53.07</v>
+        <v>47.82</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>64.3</v>
+        <v>53.19</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1658,22 +1698,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1116.7</v>
+        <v>567.7</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>48.47</v>
+        <v>45.53</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>48.48</v>
+        <v>37.36</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>53.47</v>
+        <v>38.75</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1682,22 +1722,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>287.85</v>
+        <v>191.19</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>46.5</v>
+        <v>45.11</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>48.07</v>
+        <v>48.35</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>54.11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1706,22 +1746,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>1304</v>
+        <v>244.96</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>46.28</v>
+        <v>44.98</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>41.92</v>
+        <v>43.35</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>46.82</v>
+        <v>51.7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1730,22 +1770,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>4026.6</v>
+        <v>2069</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>43.89</v>
+        <v>43.56</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>52.77</v>
+        <v>25.91</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>57.83</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1754,22 +1794,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>2093.5</v>
+        <v>1225.8</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>43.84</v>
+        <v>43.31</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>26.72</v>
+        <v>54.67</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>31.89</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1778,22 +1818,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1047.2</v>
+        <v>967.45</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>42.92</v>
+        <v>43.25</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>31.24</v>
+        <v>50.55</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>34.63</v>
+        <v>61.41</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1802,22 +1842,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>9785.5</v>
+        <v>175.46</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>42.34</v>
+        <v>42.11</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>52.27</v>
+        <v>31.99</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>59.1</v>
+        <v>37.3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1826,22 +1866,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>438.7</v>
+        <v>283.1</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>41.38</v>
+        <v>41.94</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>50.43</v>
+        <v>45.27</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>61.32</v>
+        <v>52.9</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1850,22 +1890,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>356.45</v>
+        <v>377.6</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>41.18</v>
+        <v>39.9</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>45.55</v>
+        <v>43.44</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>55.45</v>
+        <v>47.65</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1874,22 +1914,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>567.7</v>
+        <v>2902.8</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>40.31</v>
+        <v>39.89</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>37.36</v>
+        <v>46.03</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>38.75</v>
+        <v>41.68</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1898,22 +1938,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>176.08</v>
+        <v>337.95</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>39.92</v>
+        <v>38.78</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>32.25</v>
+        <v>40.05</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>37.5</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1922,22 +1962,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1230.2</v>
+        <v>1261.5</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>39.65</v>
+        <v>38.51</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>51.22</v>
+        <v>46.28</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>61.63</v>
+        <v>51.41</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1946,22 +1986,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>189.8</v>
+        <v>281.75</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>39.59</v>
+        <v>37.77</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>47.17</v>
+        <v>35.68</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>58.62</v>
+        <v>34.16</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1970,22 +2010,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>344.1</v>
+        <v>429.3</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>38.42</v>
+        <v>35.79</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>41.39</v>
+        <v>47.55</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>36.73</v>
+        <v>58.99</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1994,22 +2034,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>953.2</v>
+        <v>3886</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>34.96</v>
+        <v>33.23</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>48.06</v>
+        <v>50.08</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>60.43</v>
+        <v>56.12</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2018,16 +2058,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>237.84</v>
+        <v>344.55</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>30.89</v>
+        <v>31.29</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>39.77</v>
+        <v>41.26</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>49.98</v>
+        <v>52.55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-07-18
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1935.5</v>
+        <v>1950.1</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>71.2</v>
+        <v>70.42</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>65.23999999999999</v>
+        <v>64.87</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>63.61</v>
+        <v>63.52</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>24.44</v>
+        <v>22.18</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1775.24</v>
+        <v>1783.88</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1759.42</v>
+        <v>1766.57</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>2128036</v>
+        <v>2013540</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>466023</v>
+        <v>463695</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,31 +585,31 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>4584.4</v>
+        <v>1037.6</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>67.97</v>
+        <v>65.26000000000001</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>61.84</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>63.62</v>
+        <v>61.13</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>23.77</v>
+        <v>23.3</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4145.58</v>
+        <v>945</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>4067.96</v>
+        <v>939.34</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>923392</v>
+        <v>8601781</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>406284</v>
+        <v>656794</v>
       </c>
     </row>
     <row r="4">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>8845.5</v>
+        <v>8888</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>67.47</v>
+        <v>64.86</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>70.3</v>
+        <v>69.8</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>68.77</v>
+        <v>68.67</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>20.76</v>
+        <v>25.75</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>7888.8</v>
+        <v>7952.26</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7764.74</v>
+        <v>7819.62</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>340585</v>
+        <v>329671</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>127120</v>
+        <v>126904</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,31 +663,31 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1020.5</v>
+        <v>10443</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>63.72</v>
+        <v>62.07</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>60.6</v>
+        <v>61.52</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>59.47</v>
+        <v>62.65</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>26.85</v>
+        <v>47.99</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>940.76</v>
+        <v>9669.700000000001</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>935.92</v>
+        <v>9526.059999999999</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>9316862</v>
+        <v>379672</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>634534</v>
+        <v>291643</v>
       </c>
     </row>
     <row r="6">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3157.3</v>
+        <v>3160.7</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>60.63</v>
+        <v>59.45</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>71.70999999999999</v>
+        <v>71.78</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>60.62</v>
+        <v>60.66</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>46.04</v>
+        <v>45.35</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2557.58</v>
+        <v>2596.79</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2514.5</v>
+        <v>2546.24</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2091425</v>
+        <v>1903347</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>449275</v>
+        <v>449759</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,37 +741,37 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1456.2</v>
+        <v>1837.4</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>60.21</v>
+        <v>54.67</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>65.67</v>
+        <v>67.03</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>63.22</v>
+        <v>67.70999999999999</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>21.89</v>
+        <v>30.59</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1333.14</v>
+        <v>1635.86</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1310.93</v>
+        <v>1592.78</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>1720752</v>
+        <v>1976850</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>282151</v>
+        <v>423329</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -780,31 +780,31 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1828.1</v>
+        <v>1427.2</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>53.06</v>
+        <v>51.63</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>66.48</v>
+        <v>60.84</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>67.47</v>
+        <v>62.01</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>42.83</v>
+        <v>37.06</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1622.8</v>
+        <v>1340.65</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1580.83</v>
+        <v>1317.97</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2071318</v>
+        <v>1733604</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>421187</v>
+        <v>275209</v>
       </c>
     </row>
   </sheetData>
@@ -873,7 +873,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -882,22 +882,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1935.5</v>
+        <v>1444.3</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>71.2</v>
+        <v>70.84</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>65.23999999999999</v>
+        <v>64.14</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>63.61</v>
+        <v>62.79</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>289.65</v>
+        <v>1950.1</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>70.66</v>
+        <v>70.42</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>59.66</v>
+        <v>64.87</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>60.29</v>
+        <v>63.52</v>
       </c>
     </row>
     <row r="4">
@@ -930,22 +930,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>4584.4</v>
+        <v>4638.1</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>67.97</v>
+        <v>69.5</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>61.84</v>
+        <v>63.06</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>63.62</v>
+        <v>64.19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -954,22 +954,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>8845.5</v>
+        <v>1572.9</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>67.47</v>
+        <v>68.97</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>70.3</v>
+        <v>60.94</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>68.77</v>
+        <v>56.77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -978,22 +978,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>824.95</v>
+        <v>1037.6</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>66.56999999999999</v>
+        <v>65.26000000000001</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>52.27</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>48.32</v>
+        <v>61.13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1002,22 +1002,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1895</v>
+        <v>8888</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>65.27</v>
+        <v>64.86</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>55.63</v>
+        <v>69.8</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>53.84</v>
+        <v>68.67</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1020.5</v>
+        <v>2269</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>63.72</v>
+        <v>63.63</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>60.6</v>
+        <v>42.15</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>59.47</v>
+        <v>36.79</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1050,22 +1050,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1862.9</v>
+        <v>10443</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>62.08</v>
+        <v>62.07</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>50.35</v>
+        <v>61.52</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>56.53</v>
+        <v>62.65</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1074,22 +1074,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1931.1</v>
+        <v>286.6</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>61.48</v>
+        <v>61.39</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>52.42</v>
+        <v>58.42</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>60.91</v>
+        <v>59.78</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3213.6</v>
+        <v>1203.9</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>61.44</v>
+        <v>60.47</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>68.04000000000001</v>
+        <v>44.2</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>66</v>
+        <v>43.86</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1122,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3157.3</v>
+        <v>819.6</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>60.63</v>
+        <v>60.39</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>71.70999999999999</v>
+        <v>51.04</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>60.62</v>
+        <v>47.83</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1146,22 +1146,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>5312</v>
+        <v>3160.7</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>60.58</v>
+        <v>59.45</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>60.89</v>
+        <v>71.78</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>57.86</v>
+        <v>60.66</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,22 +1170,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1456.2</v>
+        <v>7563.5</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>60.21</v>
+        <v>58.59</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>65.67</v>
+        <v>56.84</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>63.22</v>
+        <v>65.88</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1194,22 +1194,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1044.1</v>
+        <v>11771</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>59.98</v>
+        <v>57.8</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>59.88</v>
+        <v>51.28</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>68.28</v>
+        <v>54.22</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1218,22 +1218,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>11711</v>
+        <v>3179.2</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>57.96</v>
+        <v>57.1</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>51.06</v>
+        <v>50.03</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>54.12</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1242,22 +1242,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1380.7</v>
+        <v>1044.3</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>57.59</v>
+        <v>56.99</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>59.79</v>
+        <v>55.52</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>60.42</v>
+        <v>61.26</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1266,22 +1266,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1441.3</v>
+        <v>5265.5</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>57.07</v>
+        <v>56.97</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>57.94</v>
+        <v>59.17</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>53.12</v>
+        <v>57.08</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1290,22 +1290,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1454.8</v>
+        <v>1327.2</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>57.02</v>
+        <v>56.34</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>52.77</v>
+        <v>45.52</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>52.62</v>
+        <v>48.23</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1314,22 +1314,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>10155</v>
+        <v>242.98</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>55.76</v>
+        <v>55.29</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>57.8</v>
+        <v>44.58</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>61.18</v>
+        <v>43.84</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1338,22 +1338,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1036</v>
+        <v>1854</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>54.79</v>
+        <v>55.03</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>54.29</v>
+        <v>51.11</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>60.86</v>
+        <v>51.53</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1362,22 +1362,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1101.3</v>
+        <v>1837.4</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>54.52</v>
+        <v>54.67</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>56.66</v>
+        <v>67.03</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>56.38</v>
+        <v>67.70999999999999</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>241.96</v>
+        <v>1908.8</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>54.05</v>
+        <v>54.06</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>43.77</v>
+        <v>51.4</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>43.59</v>
+        <v>60.45</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1410,22 +1410,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1828.1</v>
+        <v>1096.5</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>53.06</v>
+        <v>53</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>66.48</v>
+        <v>37.65</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>67.47</v>
+        <v>37.36</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1434,22 +1434,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1150.4</v>
+        <v>1098.2</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>53.05</v>
+        <v>52.94</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>38.24</v>
+        <v>54.39</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>41.55</v>
+        <v>55.34</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1458,22 +1458,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>13854</v>
+        <v>1024.4</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>51.99</v>
+        <v>52.76</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>50.04</v>
+        <v>58.66</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>53.88</v>
+        <v>67.88</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1482,22 +1482,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>2677.8</v>
+        <v>389.95</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>50.66</v>
+        <v>52.33</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>57.78</v>
+        <v>48.76</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>52.87</v>
+        <v>50.22</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1506,22 +1506,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>7365.5</v>
+        <v>1822.1</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>49.89</v>
+        <v>52.16</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>53.51</v>
+        <v>48.11</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>64.48999999999999</v>
+        <v>55.11</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1530,22 +1530,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1307.8</v>
+        <v>1427.2</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>49.65</v>
+        <v>51.63</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>42.5</v>
+        <v>60.84</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>47.05</v>
+        <v>62.01</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1554,22 +1554,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>3085.4</v>
+        <v>13783</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>49.58</v>
+        <v>51.19</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>47.69</v>
+        <v>49.53</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>56.63</v>
+        <v>53.63</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1578,22 +1578,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>414.85</v>
+        <v>2674.7</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>49.49</v>
+        <v>50.77</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>48.53</v>
+        <v>58.36</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>61.76</v>
+        <v>53.11</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1602,22 +1602,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1068</v>
+        <v>1328.5</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>47.85</v>
+        <v>50.47</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>33.98</v>
+        <v>54.33</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>35.81</v>
+        <v>58.83</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1626,22 +1626,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1323.7</v>
+        <v>1237.3</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>47.79</v>
+        <v>48.72</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>53.78</v>
+        <v>53.19</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>58.51</v>
+        <v>62.39</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1650,22 +1650,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>2150.6</v>
+        <v>247.29</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>47.27</v>
+        <v>48.64</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>44.38</v>
+        <v>44.51</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>44.83</v>
+        <v>52.24</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1674,22 +1674,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1106.7</v>
+        <v>2143.8</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>46.68</v>
+        <v>48.63</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>47.82</v>
+        <v>43.87</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>53.19</v>
+        <v>44.58</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1698,22 +1698,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>567.7</v>
+        <v>1418.7</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>45.53</v>
+        <v>48.25</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>37.36</v>
+        <v>55.03</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>38.75</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1722,22 +1722,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>191.19</v>
+        <v>3109.7</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>45.11</v>
+        <v>48.2</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>48.35</v>
+        <v>59.91</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>59</v>
+        <v>63.94</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1746,22 +1746,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>244.96</v>
+        <v>567.6</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>44.98</v>
+        <v>47.1</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>43.35</v>
+        <v>36.71</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>51.7</v>
+        <v>38.4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1770,22 +1770,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>2069</v>
+        <v>409.45</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>43.56</v>
+        <v>46.13</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>25.91</v>
+        <v>46.83</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>31.2</v>
+        <v>60.87</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1794,22 +1794,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1225.8</v>
+        <v>176</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>43.31</v>
+        <v>45.1</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>54.67</v>
+        <v>32.49</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>62.8</v>
+        <v>37.47</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1818,22 +1818,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>967.45</v>
+        <v>1088.6</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>43.25</v>
+        <v>42.46</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>50.55</v>
+        <v>44.65</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>61.41</v>
+        <v>51.77</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1842,22 +1842,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>175.46</v>
+        <v>959.3</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>42.11</v>
+        <v>41.97</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>31.99</v>
+        <v>47.57</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>37.3</v>
+        <v>60.14</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1866,22 +1866,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>283.1</v>
+        <v>280.7</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>41.94</v>
+        <v>41.87</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>45.27</v>
+        <v>35.24</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>52.9</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1890,22 +1890,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>377.6</v>
+        <v>335.6</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>39.9</v>
+        <v>40.22</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>43.44</v>
+        <v>39.53</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>47.65</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1914,22 +1914,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>2902.8</v>
+        <v>280.75</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>39.89</v>
+        <v>39.67</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>46.03</v>
+        <v>45.59</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>41.68</v>
+        <v>53.01</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1938,22 +1938,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>337.95</v>
+        <v>185.89</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>38.78</v>
+        <v>38.49</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>40.05</v>
+        <v>44.3</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>36.42</v>
+        <v>57.29</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1962,22 +1962,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1261.5</v>
+        <v>2842.4</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>38.51</v>
+        <v>36.21</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>46.28</v>
+        <v>44.71</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>51.41</v>
+        <v>41.29</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1986,22 +1986,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>281.75</v>
+        <v>427.65</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>37.77</v>
+        <v>35.33</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>35.68</v>
+        <v>47.04</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>34.16</v>
+        <v>58.6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2010,22 +2010,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>429.3</v>
+        <v>341.85</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>35.79</v>
+        <v>33.67</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>47.55</v>
+        <v>40.33</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>58.99</v>
+        <v>51.94</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2034,22 +2034,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>3886</v>
+        <v>1211.2</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>33.23</v>
+        <v>31.88</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>50.08</v>
+        <v>43.01</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>56.12</v>
+        <v>49.27</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2058,16 +2058,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>344.55</v>
+        <v>3775.6</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>31.29</v>
+        <v>29.53</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>41.26</v>
+        <v>45.97</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>52.55</v>
+        <v>53.56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-07-25
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1950.1</v>
+        <v>11283.5</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>70.42</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>64.87</v>
+        <v>68.65000000000001</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>63.52</v>
+        <v>65.76000000000001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>22.18</v>
+        <v>25.62</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1783.88</v>
+        <v>9728.32</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1766.57</v>
+        <v>9573.879999999999</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>2013540</v>
+        <v>472144</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>463695</v>
+        <v>305605</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1037.6</v>
+        <v>4697.3</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>65.26000000000001</v>
+        <v>71.54000000000001</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>64.09999999999999</v>
+        <v>63.96</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>61.13</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>23.3</v>
+        <v>36.73</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>945</v>
+        <v>4201.98</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>939.34</v>
+        <v>4118.98</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>8601781</v>
+        <v>824096</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>656794</v>
+        <v>414871</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>64.86</v>
+        <v>64.45</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>69.8</v>
+        <v>65.48999999999999</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>68.67</v>
+        <v>63.79</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>25.75</v>
+        <v>35.14</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>7952.26</v>
+        <v>1794.6</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7819.62</v>
+        <v>1775.67</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>329671</v>
+        <v>1900363</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>126904</v>
+        <v>465735</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,31 +663,31 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>10443</v>
+        <v>8862</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>62.07</v>
+        <v>58.93</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>61.52</v>
+        <v>69.08</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>62.65</v>
+        <v>68.54000000000001</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>47.99</v>
+        <v>30.03</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>9669.700000000001</v>
+        <v>8012.73</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>9526.059999999999</v>
+        <v>7871.26</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>379672</v>
+        <v>282293</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>291643</v>
+        <v>126610</v>
       </c>
     </row>
     <row r="6">
@@ -702,109 +702,31 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3160.7</v>
+        <v>3026.4</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>59.45</v>
+        <v>45.39</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>71.78</v>
+        <v>64.62</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>60.66</v>
+        <v>58.9</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>45.35</v>
+        <v>23.47</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2596.79</v>
+        <v>2629.66</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2546.24</v>
+        <v>2572.89</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1903347</v>
+        <v>1812985</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>449759</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>ADANIPORTS</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>1837.4</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>54.67</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>67.03</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>67.70999999999999</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>30.59</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>1635.86</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>1592.78</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>1976850</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>423329</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>NESTLEIND</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>1427.2</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>51.63</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>60.84</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>62.01</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>37.06</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>1340.65</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>1317.97</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>1733604</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>275209</v>
+        <v>430649</v>
       </c>
     </row>
   </sheetData>
@@ -814,8 +736,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -873,7 +793,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -882,22 +802,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1444.3</v>
+        <v>11283.5</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>70.84</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>64.14</v>
+        <v>68.65000000000001</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>62.79</v>
+        <v>65.76000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -906,22 +826,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1950.1</v>
+        <v>4697.3</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>70.42</v>
+        <v>71.54000000000001</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>64.87</v>
+        <v>63.96</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>63.52</v>
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -930,16 +850,16 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>4638.1</v>
+        <v>1244.7</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>69.5</v>
+        <v>65.36</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>63.06</v>
+        <v>50.84</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>64.19</v>
+        <v>46.62</v>
       </c>
     </row>
     <row r="5">
@@ -954,22 +874,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1572.9</v>
+        <v>1555.8</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>68.97</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>60.94</v>
+        <v>59.68</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>56.77</v>
+        <v>56.34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -978,22 +898,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1037.6</v>
+        <v>1954</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>65.26000000000001</v>
+        <v>64.45</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>64.09999999999999</v>
+        <v>65.48999999999999</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>61.13</v>
+        <v>63.79</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1002,22 +922,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>8888</v>
+        <v>7721.5</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>64.86</v>
+        <v>63.15</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>69.8</v>
+        <v>57.9</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>68.67</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1026,22 +946,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>2269</v>
+        <v>1434.6</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>63.63</v>
+        <v>62.23</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>42.15</v>
+        <v>62.22</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>36.79</v>
+        <v>62.19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1050,22 +970,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>10443</v>
+        <v>2254.3</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>62.07</v>
+        <v>60.21</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>61.52</v>
+        <v>41.47</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>62.65</v>
+        <v>36.43</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1074,22 +994,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>286.6</v>
+        <v>3229.7</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>61.39</v>
+        <v>60.11</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>58.42</v>
+        <v>49.18</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>59.78</v>
+        <v>57.32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1098,22 +1018,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1203.9</v>
+        <v>1039.8</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>60.47</v>
+        <v>59.37</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>44.2</v>
+        <v>57.43</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>43.86</v>
+        <v>59.09</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1122,22 +1042,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>819.6</v>
+        <v>8862</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>60.39</v>
+        <v>58.93</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>51.04</v>
+        <v>69.08</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>47.83</v>
+        <v>68.54000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1146,22 +1066,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>3160.7</v>
+        <v>1889.4</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>59.45</v>
+        <v>58.77</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>71.78</v>
+        <v>52.63</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>60.66</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,22 +1090,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>7563.5</v>
+        <v>11908</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>58.59</v>
+        <v>58.28</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>56.84</v>
+        <v>52.96</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>65.88</v>
+        <v>54.97</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1194,22 +1114,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>11771</v>
+        <v>1853.5</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>57.8</v>
+        <v>57.04</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>51.28</v>
+        <v>50.19</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>54.22</v>
+        <v>56.35</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1218,22 +1138,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>3179.2</v>
+        <v>1907</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>57.1</v>
+        <v>56.29</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>50.03</v>
+        <v>52.54</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>57.7</v>
+        <v>60.98</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1242,22 +1162,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1044.3</v>
+        <v>1443.5</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>56.99</v>
+        <v>52.7</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>55.52</v>
+        <v>62.57</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>61.26</v>
+        <v>62.72</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1266,22 +1186,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>5265.5</v>
+        <v>280</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>56.97</v>
+        <v>52.5</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>59.17</v>
+        <v>55.72</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>57.08</v>
+        <v>58.62</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1290,22 +1210,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1327.2</v>
+        <v>2161.8</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>56.34</v>
+        <v>52.4</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>45.52</v>
+        <v>43.99</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>48.23</v>
+        <v>44.63</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1314,22 +1234,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>242.98</v>
+        <v>288.2</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>55.29</v>
+        <v>52.22</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>44.58</v>
+        <v>48.95</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>43.84</v>
+        <v>54.19</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1338,22 +1258,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1854</v>
+        <v>1246.8</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>55.03</v>
+        <v>50.32</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>51.11</v>
+        <v>53.77</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>51.53</v>
+        <v>62.57</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1362,22 +1282,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1837.4</v>
+        <v>248.76</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>54.67</v>
+        <v>49.93</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>67.03</v>
+        <v>45.27</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>67.70999999999999</v>
+        <v>52.58</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1386,22 +1306,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1908.8</v>
+        <v>384.75</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>54.06</v>
+        <v>49.1</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>51.4</v>
+        <v>46.86</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>60.45</v>
+        <v>49.16</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1410,22 +1330,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1096.5</v>
+        <v>283.45</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>53</v>
+        <v>48.79</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>37.65</v>
+        <v>37.4</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>37.36</v>
+        <v>34.43</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1434,22 +1354,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1098.2</v>
+        <v>177.12</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>52.94</v>
+        <v>48.74</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>54.39</v>
+        <v>33.59</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>55.34</v>
+        <v>37.83</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1458,22 +1378,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1024.4</v>
+        <v>1084.2</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>52.76</v>
+        <v>48.63</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>58.66</v>
+        <v>53.2</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>67.88</v>
+        <v>54.81</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1482,22 +1402,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>389.95</v>
+        <v>2668.8</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>52.33</v>
+        <v>48.58</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>48.76</v>
+        <v>54.65</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>50.22</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1506,22 +1426,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1822.1</v>
+        <v>234.71</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>52.16</v>
+        <v>46.2</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>48.11</v>
+        <v>39.64</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>55.11</v>
+        <v>41.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1530,22 +1450,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1427.2</v>
+        <v>1005.1</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>51.63</v>
+        <v>45.77</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>60.84</v>
+        <v>54.79</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>62.01</v>
+        <v>65.56</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1554,22 +1474,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>13783</v>
+        <v>1015</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>51.19</v>
+        <v>45.42</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>49.53</v>
+        <v>50.37</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>53.63</v>
+        <v>59.52</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1578,22 +1498,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>2674.7</v>
+        <v>3026.4</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>50.77</v>
+        <v>45.39</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>58.36</v>
+        <v>64.62</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>53.11</v>
+        <v>58.9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1602,22 +1522,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1328.5</v>
+        <v>3089.4</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>50.47</v>
+        <v>45.19</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>54.33</v>
+        <v>58.44</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>58.83</v>
+        <v>63.34</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1626,22 +1546,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1237.3</v>
+        <v>13442</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>48.72</v>
+        <v>44.61</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>53.19</v>
+        <v>45.97</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>62.39</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1650,22 +1570,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>247.29</v>
+        <v>1088</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>48.64</v>
+        <v>44.35</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>44.51</v>
+        <v>44.56</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>52.24</v>
+        <v>51.73</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1674,22 +1594,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>2143.8</v>
+        <v>4985</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>48.63</v>
+        <v>43.61</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>43.87</v>
+        <v>52.56</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>44.58</v>
+        <v>54.06</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1698,22 +1618,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1418.7</v>
+        <v>405</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>48.25</v>
+        <v>42.55</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>55.03</v>
+        <v>45.42</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>51.9</v>
+        <v>59.96</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1722,22 +1642,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>3109.7</v>
+        <v>1278</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>48.2</v>
+        <v>42.36</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>59.91</v>
+        <v>39.82</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>63.94</v>
+        <v>45.32</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1746,22 +1666,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>567.6</v>
+        <v>347.2</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>47.1</v>
+        <v>42.34</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>36.71</v>
+        <v>43.07</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>38.4</v>
+        <v>53.17</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1770,22 +1690,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>409.45</v>
+        <v>555.05</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>46.13</v>
+        <v>42.25</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>46.83</v>
+        <v>35.31</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>60.87</v>
+        <v>37.67</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1794,22 +1714,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>176</v>
+        <v>1778.5</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>45.1</v>
+        <v>42.18</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>32.49</v>
+        <v>59.26</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>37.47</v>
+        <v>64.89</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1818,22 +1738,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1088.6</v>
+        <v>1040.9</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>42.46</v>
+        <v>41.82</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>44.65</v>
+        <v>33.71</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>51.77</v>
+        <v>34.27</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1842,22 +1762,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>959.3</v>
+        <v>2874.8</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>41.97</v>
+        <v>41.01</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>47.57</v>
+        <v>46.04</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>60.14</v>
+        <v>41.6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1866,22 +1786,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>280.7</v>
+        <v>1393</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>41.87</v>
+        <v>40.9</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>35.24</v>
+        <v>53.89</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>34</v>
+        <v>51.44</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1890,22 +1810,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>335.6</v>
+        <v>942.8</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>40.22</v>
+        <v>39.04</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>39.53</v>
+        <v>47.39</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>36.3</v>
+        <v>60.04</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1914,16 +1834,16 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>280.75</v>
+        <v>427.4</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>39.67</v>
+        <v>37.45</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>45.59</v>
+        <v>46.96</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>53.01</v>
+        <v>58.54</v>
       </c>
     </row>
     <row r="46">
@@ -1938,22 +1858,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>185.89</v>
+        <v>182.67</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>38.49</v>
+        <v>34.09</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>44.3</v>
+        <v>42</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>57.29</v>
+        <v>56.09</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1962,22 +1882,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>2842.4</v>
+        <v>3785.6</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>36.21</v>
+        <v>33.81</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>44.71</v>
+        <v>45.09</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>41.29</v>
+        <v>53.02</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1986,22 +1906,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>427.65</v>
+        <v>742.8</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>35.33</v>
+        <v>33.7</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>47.04</v>
+        <v>37.38</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>58.6</v>
+        <v>41.44</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2010,22 +1930,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>341.85</v>
+        <v>323.8</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>33.67</v>
+        <v>33.24</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>40.33</v>
+        <v>36.91</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>51.94</v>
+        <v>35.72</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2034,22 +1954,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1211.2</v>
+        <v>1223</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>31.88</v>
+        <v>29.46</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>43.01</v>
+        <v>42.7</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>49.27</v>
+        <v>52.66</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2058,16 +1978,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>3775.6</v>
+        <v>1151.7</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>29.53</v>
+        <v>25.36</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>45.97</v>
+        <v>37.83</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>53.56</v>
+        <v>45.84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-08-01
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>11283.5</v>
+        <v>4875.2</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.45999999999999</v>
+        <v>78.91</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.65000000000001</v>
+        <v>68.22</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>65.76000000000001</v>
+        <v>66.52</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>25.62</v>
+        <v>41.22</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>9728.32</v>
+        <v>4248.59</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>9573.879999999999</v>
+        <v>4158.99</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>472144</v>
+        <v>839280</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>305605</v>
+        <v>432452</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>4697.3</v>
+        <v>1141.2</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>71.54000000000001</v>
+        <v>74.12</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>63.96</v>
+        <v>68.01000000000001</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>64.56</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>36.73</v>
+        <v>32.26</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4201.98</v>
+        <v>960.5599999999999</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>4118.98</v>
+        <v>951.64</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>824096</v>
+        <v>9735997</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>414871</v>
+        <v>709931</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1954</v>
+        <v>11432</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>64.45</v>
+        <v>73.47</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>65.48999999999999</v>
+        <v>71.84</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>63.79</v>
+        <v>67.3</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>35.14</v>
+        <v>37.4</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1794.6</v>
+        <v>9829.75</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1775.67</v>
+        <v>9660.309999999999</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>1900363</v>
+        <v>463071</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>465735</v>
+        <v>316327</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>8862</v>
+        <v>1990.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>58.93</v>
+        <v>66.91</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>69.08</v>
+        <v>68.95</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>68.54000000000001</v>
+        <v>65.31999999999999</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>30.03</v>
+        <v>36.67</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>8012.73</v>
+        <v>1808.91</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>7871.26</v>
+        <v>1788.15</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>282293</v>
+        <v>2244994</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>126610</v>
+        <v>477588</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,31 +702,109 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3026.4</v>
+        <v>8988</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>45.39</v>
+        <v>64.63</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>64.62</v>
+        <v>71.44</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>58.9</v>
+        <v>69.5</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>23.47</v>
+        <v>26.29</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2629.66</v>
+        <v>8069.95</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2572.89</v>
+        <v>7922.5</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1812985</v>
+        <v>267425</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>430649</v>
+        <v>128788</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>1509.6</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>63.91</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>68.61</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>65.37</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>24.75</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>1357.48</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>1332.48</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>2233770</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>291098</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>1435.4</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>59.44</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>62.49</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>62.33</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>28.45</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>1350.98</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>1349.48</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>12531100</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>1029652</v>
       </c>
     </row>
   </sheetData>
@@ -736,6 +814,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -793,7 +873,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -802,22 +882,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>11283.5</v>
+        <v>4875.2</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.45999999999999</v>
+        <v>78.91</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.65000000000001</v>
+        <v>68.22</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>65.76000000000001</v>
+        <v>66.52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -826,22 +906,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>4697.3</v>
+        <v>1346.9</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>71.54000000000001</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>63.96</v>
+        <v>57.07</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>64.59999999999999</v>
+        <v>49.42</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -850,22 +930,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1244.7</v>
+        <v>1141.2</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>65.36</v>
+        <v>74.12</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>50.84</v>
+        <v>68.01000000000001</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>46.62</v>
+        <v>64.56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -874,22 +954,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1555.8</v>
+        <v>11432</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>64.68000000000001</v>
+        <v>73.47</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>59.68</v>
+        <v>71.84</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>56.34</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -898,22 +978,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1954</v>
+        <v>2029.1</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>64.45</v>
+        <v>72.03</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>65.48999999999999</v>
+        <v>61.31</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>63.79</v>
+        <v>57.53</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -922,22 +1002,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>7721.5</v>
+        <v>1651.3</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>63.15</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>57.9</v>
+        <v>65.02</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>66.3</v>
+        <v>59.14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -946,22 +1026,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1434.6</v>
+        <v>1972</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>62.23</v>
+        <v>67.19</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>62.22</v>
+        <v>58.44</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>62.19</v>
+        <v>63.72</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -970,22 +1050,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2254.3</v>
+        <v>3398.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>60.21</v>
+        <v>67.01000000000001</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>41.47</v>
+        <v>59.1</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>36.43</v>
+        <v>61.86</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -994,22 +1074,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3229.7</v>
+        <v>1990.5</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>60.11</v>
+        <v>66.91</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>49.18</v>
+        <v>68.95</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>57.32</v>
+        <v>65.31999999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1018,22 +1098,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1039.8</v>
+        <v>7833.5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>59.37</v>
+        <v>66.15000000000001</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>57.43</v>
+        <v>62.34</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>59.09</v>
+        <v>68.08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1042,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>8862</v>
+        <v>256.46</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>58.93</v>
+        <v>66.09</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>69.08</v>
+        <v>54.04</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>68.54000000000001</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1066,22 +1146,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1889.4</v>
+        <v>8988</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>58.77</v>
+        <v>64.63</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>52.63</v>
+        <v>71.44</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>52.4</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1090,22 +1170,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>11908</v>
+        <v>1509.6</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>58.28</v>
+        <v>63.91</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>52.96</v>
+        <v>68.61</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>54.97</v>
+        <v>65.37</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1114,22 +1194,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1853.5</v>
+        <v>2365.6</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>57.04</v>
+        <v>62.71</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>50.19</v>
+        <v>48.29</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>56.35</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1138,22 +1218,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1907</v>
+        <v>11847</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>56.29</v>
+        <v>62.67</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>52.54</v>
+        <v>56.98</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>60.98</v>
+        <v>56.76</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1162,22 +1242,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1443.5</v>
+        <v>302.45</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>52.7</v>
+        <v>62.36</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>62.57</v>
+        <v>62.13</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>62.72</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1186,22 +1266,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>280</v>
+        <v>1473.2</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>52.5</v>
+        <v>61.52</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>55.72</v>
+        <v>60.67</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>58.62</v>
+        <v>55.14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1210,22 +1290,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>2161.8</v>
+        <v>14188</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>52.4</v>
+        <v>60.88</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>43.99</v>
+        <v>53.82</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>44.63</v>
+        <v>55.71</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1234,22 +1314,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>288.2</v>
+        <v>183.65</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>52.22</v>
+        <v>60.76</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>48.95</v>
+        <v>41.45</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>54.19</v>
+        <v>40.48</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1258,22 +1338,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1246.8</v>
+        <v>2746.2</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>50.32</v>
+        <v>59.94</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>53.77</v>
+        <v>60.45</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>62.57</v>
+        <v>54.32</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1282,22 +1362,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>248.76</v>
+        <v>1435.4</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>49.93</v>
+        <v>59.44</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>45.27</v>
+        <v>62.49</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>52.58</v>
+        <v>62.33</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1306,22 +1386,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>384.75</v>
+        <v>1877.5</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>49.1</v>
+        <v>59.06</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>46.86</v>
+        <v>51.86</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>49.16</v>
+        <v>57.3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1330,22 +1410,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>283.45</v>
+        <v>1130.1</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>48.79</v>
+        <v>57.7</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>37.4</v>
+        <v>43.86</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>34.43</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1354,22 +1434,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>177.12</v>
+        <v>1270</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>48.74</v>
+        <v>56.98</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>33.59</v>
+        <v>58.41</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>37.83</v>
+        <v>64.02</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1378,22 +1458,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1084.2</v>
+        <v>1046.7</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>48.63</v>
+        <v>54.92</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>53.2</v>
+        <v>58.87</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>54.81</v>
+        <v>68.38</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1402,22 +1482,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>2668.8</v>
+        <v>2999.2</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>48.58</v>
+        <v>53.94</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>54.65</v>
+        <v>49.19</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>52</v>
+        <v>42.37</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1426,22 +1506,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>234.71</v>
+        <v>1307.8</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>46.2</v>
+        <v>53.42</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>39.64</v>
+        <v>44.36</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>41.9</v>
+        <v>47.05</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1450,22 +1530,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1005.1</v>
+        <v>389.4</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>45.77</v>
+        <v>53.08</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>54.79</v>
+        <v>49.13</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>65.56</v>
+        <v>50.29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1474,22 +1554,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1015</v>
+        <v>3938.9</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>45.42</v>
+        <v>52.84</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>50.37</v>
+        <v>50.49</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>59.52</v>
+        <v>55.98</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1498,22 +1578,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>3026.4</v>
+        <v>189.69</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>45.39</v>
+        <v>52.49</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>64.62</v>
+        <v>48.3</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>58.9</v>
+        <v>58.59</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1522,22 +1602,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>3089.4</v>
+        <v>970.4</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>45.19</v>
+        <v>51.49</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>58.44</v>
+        <v>51.86</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>63.34</v>
+        <v>61.73</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1546,22 +1626,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>13442</v>
+        <v>1098.5</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>44.61</v>
+        <v>50.97</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>45.97</v>
+        <v>55.22</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>51.9</v>
+        <v>55.82</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1570,22 +1650,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1088</v>
+        <v>339.75</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>44.35</v>
+        <v>50.91</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>44.56</v>
+        <v>42.46</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>51.73</v>
+        <v>36.51</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1594,22 +1674,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>4985</v>
+        <v>1027.4</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>43.61</v>
+        <v>50.86</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>52.56</v>
+        <v>52.38</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>54.06</v>
+        <v>60.44</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1618,22 +1698,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>405</v>
+        <v>5171</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>42.55</v>
+        <v>50.76</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>45.42</v>
+        <v>56.28</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>59.96</v>
+        <v>56.16</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1642,22 +1722,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1278</v>
+        <v>3104.8</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>42.36</v>
+        <v>47.15</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>39.82</v>
+        <v>59.05</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>45.32</v>
+        <v>63.75</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1666,22 +1746,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>347.2</v>
+        <v>284.25</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>42.34</v>
+        <v>46.19</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>43.07</v>
+        <v>46.33</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>53.17</v>
+        <v>53.2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1690,22 +1770,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>555.05</v>
+        <v>2101.3</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>42.25</v>
+        <v>45.39</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>35.31</v>
+        <v>40.56</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>37.67</v>
+        <v>43.12</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1714,22 +1794,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1778.5</v>
+        <v>347.25</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>42.18</v>
+        <v>45.31</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>59.26</v>
+        <v>43.09</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>64.89</v>
+        <v>53.19</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1738,22 +1818,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1040.9</v>
+        <v>3009.5</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>41.82</v>
+        <v>44.73</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>33.71</v>
+        <v>63.76</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>34.27</v>
+        <v>58.58</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1762,22 +1842,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>2874.8</v>
+        <v>1083.1</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>41.01</v>
+        <v>44.38</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>46.04</v>
+        <v>43.86</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>41.6</v>
+        <v>51.42</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1786,22 +1866,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1393</v>
+        <v>242.53</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>40.9</v>
+        <v>43.91</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>53.89</v>
+        <v>42.6</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>51.44</v>
+        <v>51.13</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1810,22 +1890,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>942.8</v>
+        <v>281</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>39.04</v>
+        <v>43.66</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>47.39</v>
+        <v>36.24</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>60.04</v>
+        <v>34.04</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1834,22 +1914,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>427.4</v>
+        <v>548.5</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>37.45</v>
+        <v>40.6</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>46.96</v>
+        <v>34.24</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>58.54</v>
+        <v>37.13</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1858,22 +1938,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>182.67</v>
+        <v>748.15</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>34.09</v>
+        <v>39.34</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>42</v>
+        <v>38.61</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>56.09</v>
+        <v>41.81</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1882,22 +1962,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>3785.6</v>
+        <v>414.15</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>33.81</v>
+        <v>38.56</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>45.09</v>
+        <v>44.4</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>53.02</v>
+        <v>56.79</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1906,22 +1986,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>742.8</v>
+        <v>1696.5</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>33.7</v>
+        <v>34.75</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>37.38</v>
+        <v>52.46</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>41.44</v>
+        <v>61.54</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1930,22 +2010,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>323.8</v>
+        <v>1229.5</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>33.24</v>
+        <v>33.88</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>36.91</v>
+        <v>42.98</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>35.72</v>
+        <v>52.78</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1954,16 +2034,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1223</v>
+        <v>387.85</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>29.46</v>
+        <v>33.3</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>42.7</v>
+        <v>40.38</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>52.66</v>
+        <v>56.69</v>
       </c>
     </row>
     <row r="51">
@@ -1978,16 +2058,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1151.7</v>
+        <v>1148.1</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>25.36</v>
+        <v>28.36</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>37.83</v>
+        <v>37.54</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>45.84</v>
+        <v>45.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-08-08
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>4875.2</v>
+        <v>1059.6</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>78.91</v>
+        <v>69.86</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.22</v>
+        <v>61.38</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>66.52</v>
+        <v>65.43000000000001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>41.22</v>
+        <v>22.02</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>4248.59</v>
+        <v>958.91</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>4158.99</v>
+        <v>932.38</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>839280</v>
+        <v>5077369</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>432452</v>
+        <v>235214</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1141.2</v>
+        <v>4941</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>74.12</v>
+        <v>68.63</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>68.01000000000001</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>64.56</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>32.26</v>
+        <v>48.99</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>960.5599999999999</v>
+        <v>4294.12</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>951.64</v>
+        <v>4197.04</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>9735997</v>
+        <v>915968</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>709931</v>
+        <v>438289</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>11432</v>
+        <v>1540</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>73.47</v>
+        <v>67.61</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>71.84</v>
+        <v>70.94</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>67.3</v>
+        <v>66.54000000000001</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>37.4</v>
+        <v>22.71</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>9829.75</v>
+        <v>1368.59</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>9660.309999999999</v>
+        <v>1342.28</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>463071</v>
+        <v>2387949</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>316327</v>
+        <v>296960</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1990.5</v>
+        <v>8020</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>66.91</v>
+        <v>67.45</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>68.95</v>
+        <v>64.95</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>65.31999999999999</v>
+        <v>69.23</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>36.67</v>
+        <v>24.91</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1808.91</v>
+        <v>7211.6</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>1788.15</v>
+        <v>7068.97</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>2244994</v>
+        <v>694922</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>477588</v>
+        <v>220166</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>8988</v>
+        <v>315</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>64.63</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>71.44</v>
+        <v>65.17</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>69.5</v>
+        <v>64.22</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>26.29</v>
+        <v>39.01</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>8069.95</v>
+        <v>271.81</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7922.5</v>
+        <v>271.75</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>267425</v>
+        <v>36867490</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>128788</v>
+        <v>289970</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,70 +741,265 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1509.6</v>
+        <v>11620</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>63.91</v>
+        <v>66.8</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>68.61</v>
+        <v>72.95999999999999</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>65.37</v>
+        <v>67.87</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>24.75</v>
+        <v>46.55</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>1357.48</v>
+        <v>9927.889999999999</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1332.48</v>
+        <v>9741.33</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>2233770</v>
+        <v>431456</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>291098</v>
+        <v>320213</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>1635</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>66.51000000000001</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>63.42</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>58.43</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>30.88</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>1470.04</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>1467.42</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>2929444</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>144836</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>1307.9</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>62.37</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>65.47</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>1222.88</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>1202.81</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>1678639</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>317205</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>8974.5</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>57.44</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>70.26000000000001</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>69.31999999999999</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>21.76</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>8115.22</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>7963.05</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>266371</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>128615</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1078</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>53.22</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>60.09</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>60.29</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>34.06</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>971.87</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>960.55</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>10198426</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>670614</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>ICICIBANK</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>1435.4</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>59.44</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>62.49</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>62.33</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>28.45</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>1350.98</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>1349.48</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>12531100</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>1029652</v>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1421</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>52.22</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>62.03</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>26.56</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>1346.65</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>1343.3</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>12861962</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>1019323</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>1945</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>62.72</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>32.09</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>1818.2</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>1796.27</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>2386479</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>466671</v>
       </c>
     </row>
   </sheetData>
@@ -816,6 +1011,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -873,7 +1073,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -882,22 +1082,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>4875.2</v>
+        <v>1097.2</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>78.91</v>
+        <v>70.8</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.22</v>
+        <v>61.79</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>66.52</v>
+        <v>63.86</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -906,22 +1106,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1346.9</v>
+        <v>1059.6</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>74.95999999999999</v>
+        <v>69.86</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>57.07</v>
+        <v>61.38</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>49.42</v>
+        <v>65.43000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -930,22 +1130,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1141.2</v>
+        <v>3502</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>74.12</v>
+        <v>69.39</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>68.01000000000001</v>
+        <v>62.54</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>64.56</v>
+        <v>63.67</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -954,22 +1154,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>11432</v>
+        <v>1356.6</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>73.47</v>
+        <v>68.70999999999999</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>71.84</v>
+        <v>57.8</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>67.3</v>
+        <v>49.79</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -978,22 +1178,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>2029.1</v>
+        <v>4941</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>72.03</v>
+        <v>68.63</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>61.31</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>57.53</v>
+        <v>67.15000000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1002,22 +1202,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1651.3</v>
+        <v>1540</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>71.84999999999999</v>
+        <v>67.61</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>65.02</v>
+        <v>70.94</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>59.14</v>
+        <v>66.54000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1026,22 +1226,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1972</v>
+        <v>8020</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>67.19</v>
+        <v>67.45</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>58.44</v>
+        <v>64.95</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>63.72</v>
+        <v>69.23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1050,22 +1250,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>3398.5</v>
+        <v>315</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>67.01000000000001</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>59.1</v>
+        <v>65.17</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>61.86</v>
+        <v>64.22</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1074,22 +1274,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1990.5</v>
+        <v>11620</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>66.91</v>
+        <v>66.8</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>68.95</v>
+        <v>72.95999999999999</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>65.31999999999999</v>
+        <v>67.87</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1098,22 +1298,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>7833.5</v>
+        <v>1635</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>66.15000000000001</v>
+        <v>66.51000000000001</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>62.34</v>
+        <v>63.42</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>68.08</v>
+        <v>58.43</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1122,22 +1322,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>256.46</v>
+        <v>12105</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>66.09</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>54.04</v>
+        <v>59.58</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>46.9</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1146,22 +1346,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>8988</v>
+        <v>3323</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>64.63</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>71.44</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>69.5</v>
+        <v>68.39</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,22 +1370,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1509.6</v>
+        <v>2452.7</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>63.91</v>
+        <v>63.37</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>68.61</v>
+        <v>52.91</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>65.37</v>
+        <v>41.11</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1194,22 +1394,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>2365.6</v>
+        <v>1115</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>62.71</v>
+        <v>62.95</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>48.29</v>
+        <v>64.54000000000001</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>39.06</v>
+        <v>70.89</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1218,22 +1418,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>11847</v>
+        <v>187.53</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>62.67</v>
+        <v>62.91</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>56.98</v>
+        <v>44.66</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>56.76</v>
+        <v>41.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1242,22 +1442,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>302.45</v>
+        <v>1307.9</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>62.36</v>
+        <v>62.37</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>62.13</v>
+        <v>62.5</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>62.3</v>
+        <v>65.47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1266,22 +1466,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1473.2</v>
+        <v>1175.1</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>61.52</v>
+        <v>62.22</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>60.67</v>
+        <v>48.17</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>55.14</v>
+        <v>41.43</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1290,22 +1490,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>14188</v>
+        <v>4056</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>60.88</v>
+        <v>61.72</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>53.82</v>
+        <v>54.19</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>55.71</v>
+        <v>57.91</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1314,22 +1514,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>183.65</v>
+        <v>1477</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>60.76</v>
+        <v>60.98</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>41.45</v>
+        <v>59.26</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>40.48</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1338,22 +1538,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>2746.2</v>
+        <v>1959.9</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>59.94</v>
+        <v>60.6</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>60.45</v>
+        <v>57.18</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>54.32</v>
+        <v>62.94</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1362,22 +1562,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1435.4</v>
+        <v>256.8</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>59.44</v>
+        <v>59.87</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>62.49</v>
+        <v>54.23</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>62.33</v>
+        <v>46.98</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1386,22 +1586,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1877.5</v>
+        <v>2008.9</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>59.06</v>
+        <v>59.56</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>51.86</v>
+        <v>59.75</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>57.3</v>
+        <v>56.66</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1410,22 +1610,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1130.1</v>
+        <v>1334.8</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>57.7</v>
+        <v>58.67</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>43.86</v>
+        <v>48.18</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>39.1</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1434,22 +1634,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1270</v>
+        <v>8974.5</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>56.98</v>
+        <v>57.44</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>58.41</v>
+        <v>70.26000000000001</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>64.02</v>
+        <v>69.31999999999999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1458,22 +1658,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1046.7</v>
+        <v>13940</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>54.92</v>
+        <v>57.06</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>58.87</v>
+        <v>53.32</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>68.38</v>
+        <v>55.4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1482,22 +1682,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>2999.2</v>
+        <v>5333</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>53.94</v>
+        <v>55.62</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>49.19</v>
+        <v>59.27</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>42.37</v>
+        <v>57.69</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1506,22 +1706,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1307.8</v>
+        <v>347</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>53.42</v>
+        <v>55.23</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>44.36</v>
+        <v>44.83</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>47.05</v>
+        <v>37.18</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1530,22 +1730,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>389.4</v>
+        <v>2735</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>53.08</v>
+        <v>53.68</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>49.13</v>
+        <v>59.56</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>50.29</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1554,22 +1754,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>3938.9</v>
+        <v>1078</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>52.84</v>
+        <v>53.22</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>50.49</v>
+        <v>60.09</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>55.98</v>
+        <v>60.29</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1578,22 +1778,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>189.69</v>
+        <v>1861.5</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>52.49</v>
+        <v>52.62</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>48.3</v>
+        <v>49.85</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>58.59</v>
+        <v>55.82</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1602,22 +1802,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>970.4</v>
+        <v>1421</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>51.49</v>
+        <v>52.22</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>51.86</v>
+        <v>62.03</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>61.73</v>
+        <v>62.1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1626,22 +1826,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1098.5</v>
+        <v>286.1</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>50.97</v>
+        <v>52.16</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>55.22</v>
+        <v>40.38</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>55.82</v>
+        <v>35.67</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1650,22 +1850,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>339.75</v>
+        <v>1945</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>50.91</v>
+        <v>52.1</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>42.46</v>
+        <v>62.72</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>36.51</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1674,22 +1874,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1027.4</v>
+        <v>390.75</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>50.86</v>
+        <v>51.5</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>52.38</v>
+        <v>49.35</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>60.44</v>
+        <v>50.39</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1698,22 +1898,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>5171</v>
+        <v>2997</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>50.76</v>
+        <v>49.94</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>56.28</v>
+        <v>48.96</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>56.16</v>
+        <v>42.3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1722,22 +1922,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>3104.8</v>
+        <v>401</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>47.15</v>
+        <v>48.97</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>59.05</v>
+        <v>45.39</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>63.75</v>
+        <v>58.56</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1746,22 +1946,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>284.25</v>
+        <v>187.55</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>46.19</v>
+        <v>46.85</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>46.33</v>
+        <v>46.64</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>53.2</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1770,22 +1970,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>2101.3</v>
+        <v>3026</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>45.39</v>
+        <v>46.49</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>40.56</v>
+        <v>64.08</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>43.12</v>
+        <v>58.73</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1794,22 +1994,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>347.25</v>
+        <v>2096</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>45.31</v>
+        <v>45.93</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>43.09</v>
+        <v>40.15</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>53.19</v>
+        <v>42.96</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1818,22 +2018,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>3009.5</v>
+        <v>1082.3</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>44.73</v>
+        <v>44.84</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>63.76</v>
+        <v>43.73</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>58.58</v>
+        <v>51.36</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1842,22 +2042,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1083.1</v>
+        <v>1072.4</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>44.38</v>
+        <v>44.08</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>43.86</v>
+        <v>51.45</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>51.42</v>
+        <v>54.12</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1866,22 +2066,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>242.53</v>
+        <v>342.5</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>43.91</v>
+        <v>42.41</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>42.6</v>
+        <v>41.15</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>51.13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1890,22 +2090,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>281</v>
+        <v>415.25</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>43.66</v>
+        <v>40.91</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>36.24</v>
+        <v>44.86</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>34.04</v>
+        <v>56.99</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1914,22 +2114,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>548.5</v>
+        <v>1238</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>40.6</v>
+        <v>40.05</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>34.24</v>
+        <v>44.14</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>37.13</v>
+        <v>53.22</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1938,22 +2138,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>748.15</v>
+        <v>540</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>39.34</v>
+        <v>39.6</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>38.61</v>
+        <v>32.84</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>41.81</v>
+        <v>36.41</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1962,22 +2162,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>414.15</v>
+        <v>238.85</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>38.56</v>
+        <v>39.32</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>44.4</v>
+        <v>41.06</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>56.79</v>
+        <v>50.15</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1986,22 +2186,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1696.5</v>
+        <v>1172</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>34.75</v>
+        <v>38.91</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>52.46</v>
+        <v>40.83</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>61.54</v>
+        <v>47.23</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2010,22 +2210,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>1229.5</v>
+        <v>1693.5</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>33.88</v>
+        <v>35.19</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>42.98</v>
+        <v>52.19</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>52.78</v>
+        <v>61.4</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2034,22 +2234,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>387.85</v>
+        <v>731</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>33.3</v>
+        <v>34.5</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>40.38</v>
+        <v>36.16</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>56.69</v>
+        <v>40.53</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2058,16 +2258,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1148.1</v>
+        <v>271.6</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>28.36</v>
+        <v>32.84</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>37.54</v>
+        <v>39.12</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>45.65</v>
+        <v>49.81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-08-15
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Screener Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="RSI Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screener Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSI Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,31 +546,31 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1059.6</v>
+        <v>8100</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>69.86</v>
+        <v>68.88</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>61.38</v>
+        <v>65.59</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>65.43000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>22.02</v>
+        <v>30.8</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>958.91</v>
+        <v>7254.36</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>932.38</v>
+        <v>7107.57</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>5077369</v>
+        <v>537863</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>235214</v>
+        <v>221443</v>
       </c>
     </row>
     <row r="3">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>4941</v>
+        <v>5056.2</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>68.63</v>
+        <v>68.55</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>69.51000000000001</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>67.15000000000001</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>48.99</v>
+        <v>52.48</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4294.12</v>
+        <v>4345.35</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>4197.04</v>
+        <v>4240.96</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>915968</v>
+        <v>1023022</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>438289</v>
+        <v>448643</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1540</v>
+        <v>11700</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>67.61</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>70.94</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>66.54000000000001</v>
+        <v>68.02</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>22.71</v>
+        <v>55.74</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1368.59</v>
+        <v>10082.73</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1342.28</v>
+        <v>9871.610000000001</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>2387949</v>
+        <v>417529</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>296960</v>
+        <v>321520</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>8020</v>
+        <v>318.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>67.45</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>64.95</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>69.23</v>
+        <v>64.72</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>24.91</v>
+        <v>37.58</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>7211.6</v>
+        <v>274.64</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>7068.97</v>
+        <v>273.86</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>694922</v>
+        <v>33568779</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>220166</v>
+        <v>293192</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>315</v>
+        <v>1632.8</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>67.04000000000001</v>
+        <v>62.46</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>65.17</v>
+        <v>63.19</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>64.22</v>
+        <v>58.33</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>39.01</v>
+        <v>30.07</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>271.81</v>
+        <v>1480.79</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>271.75</v>
+        <v>1475.96</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>36867490</v>
+        <v>2956849</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>289970</v>
+        <v>144641</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,37 +741,37 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>11620</v>
+        <v>1122</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>66.8</v>
+        <v>60.44</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>72.95999999999999</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>67.87</v>
+        <v>71.13</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>46.55</v>
+        <v>21.63</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>9927.889999999999</v>
+        <v>977.7</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>9741.33</v>
+        <v>945.61</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>431456</v>
+        <v>5456958</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>320213</v>
+        <v>264005</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -780,37 +780,37 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1635</v>
+        <v>3248.7</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>66.51000000000001</v>
+        <v>54.91</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>63.42</v>
+        <v>63.66</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>58.43</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>30.88</v>
+        <v>24.7</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1470.04</v>
+        <v>2987.94</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1467.42</v>
+        <v>2941.65</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2929444</v>
+        <v>685853</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>144836</v>
+        <v>220344</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -819,37 +819,37 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1307.9</v>
+        <v>8920.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>62.37</v>
+        <v>54.75</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>62.5</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>65.47</v>
+        <v>69.11</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>24.85</v>
+        <v>22.11</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>1222.88</v>
+        <v>8167.47</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>1202.81</v>
+        <v>8009.77</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>1678639</v>
+        <v>354479</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>317205</v>
+        <v>128263</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -858,37 +858,37 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>8974.5</v>
+        <v>1087</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>57.44</v>
+        <v>53.8</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>70.26000000000001</v>
+        <v>60.79</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>69.31999999999999</v>
+        <v>60.86</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>21.76</v>
+        <v>24.92</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>8115.22</v>
+        <v>979.6900000000001</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>7963.05</v>
+        <v>966.91</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>266371</v>
+        <v>9224734</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>128615</v>
+        <v>676213</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1078</v>
+        <v>1930</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>53.22</v>
+        <v>47.16</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>60.09</v>
+        <v>60.77</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>60.29</v>
+        <v>61.88</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>34.06</v>
+        <v>25.16</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>971.87</v>
+        <v>1825.96</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>960.55</v>
+        <v>1803.25</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>10198426</v>
+        <v>2339607</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>670614</v>
+        <v>463072</v>
       </c>
     </row>
     <row r="12">
@@ -936,70 +936,31 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1421</v>
+        <v>1406.8</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>52.22</v>
+        <v>46.92</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>62.03</v>
+        <v>61.24</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>62.1</v>
+        <v>61.72</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>26.56</v>
+        <v>20.54</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>1346.65</v>
+        <v>1350.71</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1343.3</v>
+        <v>1346.5</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>12861962</v>
+        <v>12083442</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1019323</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>SUNPHARMA</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>1945</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>52.1</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>62.72</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>62.7</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>32.09</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>1818.2</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>1796.27</v>
-      </c>
-      <c r="J13" s="4" t="n">
-        <v>2386479</v>
-      </c>
-      <c r="K13" s="4" t="n">
-        <v>466671</v>
+        <v>1016453</v>
       </c>
     </row>
   </sheetData>
@@ -1015,7 +976,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1073,7 +1033,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1082,22 +1042,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1097.2</v>
+        <v>1370</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>70.8</v>
+        <v>70.53</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>61.79</v>
+        <v>58.07</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>63.86</v>
+        <v>49.91</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1106,22 +1066,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1059.6</v>
+        <v>8100</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>69.86</v>
+        <v>68.88</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>61.38</v>
+        <v>65.59</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>65.43000000000001</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1130,22 +1090,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>3502</v>
+        <v>5056.2</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>69.39</v>
+        <v>68.55</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>62.54</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>63.67</v>
+        <v>68.20999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1154,22 +1114,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1356.6</v>
+        <v>11700</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>68.70999999999999</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>57.8</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>49.79</v>
+        <v>68.02</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1178,22 +1138,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4941</v>
+        <v>318.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>68.63</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>69.51000000000001</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>67.15000000000001</v>
+        <v>64.72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1202,22 +1162,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1540</v>
+        <v>1992.1</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>67.61</v>
+        <v>63.13</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>70.94</v>
+        <v>59.67</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>66.54000000000001</v>
+        <v>64.45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1226,22 +1186,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>8020</v>
+        <v>1632.8</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>67.45</v>
+        <v>62.46</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>64.95</v>
+        <v>63.19</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>69.23</v>
+        <v>58.33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1250,22 +1210,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>315</v>
+        <v>2025</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>67.04000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>65.17</v>
+        <v>59.7</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>64.22</v>
+        <v>56.63</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1274,22 +1234,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>11620</v>
+        <v>1122</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>66.8</v>
+        <v>60.44</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>72.95999999999999</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>67.87</v>
+        <v>71.13</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1298,22 +1258,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1635</v>
+        <v>3428.2</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>66.51000000000001</v>
+        <v>60.05</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>63.42</v>
+        <v>58.75</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>58.43</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1322,22 +1282,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>12105</v>
+        <v>410.8</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>65.79000000000001</v>
+        <v>58.74</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>59.58</v>
+        <v>49.02</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>58</v>
+        <v>59.92</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1346,22 +1306,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>3323</v>
+        <v>1169.2</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>64.56999999999999</v>
+        <v>58.65</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>68.98999999999999</v>
+        <v>47.65</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>68.39</v>
+        <v>41.14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1370,22 +1330,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>2452.7</v>
+        <v>4057</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>63.37</v>
+        <v>58.64</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>52.91</v>
+        <v>54.22</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>41.11</v>
+        <v>57.93</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1394,22 +1354,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1115</v>
+        <v>1067.7</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>62.95</v>
+        <v>56.21</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>64.54000000000001</v>
+        <v>56.69</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>70.89</v>
+        <v>62.49</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1418,22 +1378,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>187.53</v>
+        <v>1506.9</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>62.91</v>
+        <v>56.07</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>44.66</v>
+        <v>64.06</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>41.7</v>
+        <v>64.58</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1442,22 +1402,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1307.9</v>
+        <v>1029.5</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>62.37</v>
+        <v>55.84</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>62.5</v>
+        <v>57.07</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>65.47</v>
+        <v>64.20999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1466,22 +1426,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1175.1</v>
+        <v>184</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>62.22</v>
+        <v>54.92</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>48.17</v>
+        <v>42.38</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>41.43</v>
+        <v>40.59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1490,22 +1450,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>4056</v>
+        <v>3248.7</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>61.72</v>
+        <v>54.91</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>54.19</v>
+        <v>63.66</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>57.91</v>
+        <v>67.04000000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1514,22 +1474,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1477</v>
+        <v>8920.5</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>60.98</v>
+        <v>54.75</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>59.26</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>54.5</v>
+        <v>69.11</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1538,22 +1498,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1959.9</v>
+        <v>1087</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>60.6</v>
+        <v>53.8</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>57.18</v>
+        <v>60.79</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>62.94</v>
+        <v>60.86</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1562,22 +1522,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>256.8</v>
+        <v>5310</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>59.87</v>
+        <v>53.35</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>54.23</v>
+        <v>58.65</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>46.98</v>
+        <v>57.48</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1586,22 +1546,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>2008.9</v>
+        <v>2361</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>59.56</v>
+        <v>53.16</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>59.75</v>
+        <v>48.04</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>56.66</v>
+        <v>38.99</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1610,22 +1570,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1334.8</v>
+        <v>1206</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>58.67</v>
+        <v>51.22</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>48.18</v>
+        <v>44.52</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>48.8</v>
+        <v>48.97</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1634,16 +1594,16 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>8974.5</v>
+        <v>391.15</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>57.44</v>
+        <v>51.15</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>70.26000000000001</v>
+        <v>49.5</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>69.31999999999999</v>
+        <v>50.48</v>
       </c>
     </row>
     <row r="26">
@@ -1658,22 +1618,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>13940</v>
+        <v>13834</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>57.06</v>
+        <v>51.05</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>53.32</v>
+        <v>51.03</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>55.4</v>
+        <v>54.28</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1682,22 +1642,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>5333</v>
+        <v>1310</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>55.62</v>
+        <v>50.79</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>59.27</v>
+        <v>45.12</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>57.69</v>
+        <v>47.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1706,22 +1666,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>347</v>
+        <v>1450</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>55.23</v>
+        <v>50.72</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>44.83</v>
+        <v>57.16</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>37.18</v>
+        <v>53.59</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1730,22 +1690,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>2735</v>
+        <v>249.05</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>53.68</v>
+        <v>50.56</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>59.56</v>
+        <v>49.71</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>54</v>
+        <v>45.55</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1754,22 +1714,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1078</v>
+        <v>3035.1</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>53.22</v>
+        <v>49.78</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>60.09</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>60.29</v>
+        <v>58.94</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1778,22 +1738,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1861.5</v>
+        <v>1270</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>52.62</v>
+        <v>49.55</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>49.85</v>
+        <v>56.51</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>55.82</v>
+        <v>64.02</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1802,22 +1762,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1421</v>
+        <v>11706</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>52.22</v>
+        <v>48.8</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>62.03</v>
+        <v>51.59</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>62.1</v>
+        <v>54.51</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1826,16 +1786,16 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>286.1</v>
+        <v>2978</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>52.16</v>
+        <v>47.59</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>40.38</v>
+        <v>48.41</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>35.67</v>
+        <v>42.17</v>
       </c>
     </row>
     <row r="34">
@@ -1850,22 +1810,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1945</v>
+        <v>1930</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>52.1</v>
+        <v>47.16</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>62.72</v>
+        <v>60.77</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>62.7</v>
+        <v>61.88</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1874,22 +1834,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>390.75</v>
+        <v>1406.8</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>51.5</v>
+        <v>46.92</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>49.35</v>
+        <v>61.24</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>50.39</v>
+        <v>61.72</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1898,22 +1858,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>2997</v>
+        <v>1079.5</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>49.94</v>
+        <v>46.4</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>48.96</v>
+        <v>43.28</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>42.3</v>
+        <v>51.16</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1922,22 +1882,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>401</v>
+        <v>2696.3</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>48.97</v>
+        <v>45.7</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>45.39</v>
+        <v>56.6</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>58.56</v>
+        <v>53.03</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1946,22 +1906,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>187.55</v>
+        <v>2077</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>46.85</v>
+        <v>44.75</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>46.64</v>
+        <v>38.64</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>57.7</v>
+        <v>42.38</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1970,22 +1930,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>3026</v>
+        <v>334.5</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>46.49</v>
+        <v>43.44</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>64.08</v>
+        <v>41.64</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>58.73</v>
+        <v>36.23</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1994,22 +1954,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>2096</v>
+        <v>1700</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>45.93</v>
+        <v>42.52</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>40.15</v>
+        <v>52.76</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>42.96</v>
+        <v>61.64</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -2018,22 +1978,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1082.3</v>
+        <v>184.85</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>44.84</v>
+        <v>42.28</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>43.73</v>
+        <v>43.58</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>51.36</v>
+        <v>56.09</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -2042,22 +2002,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1072.4</v>
+        <v>340</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>44.08</v>
+        <v>42.27</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>51.45</v>
+        <v>40.13</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>54.12</v>
+        <v>51.4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -2066,22 +2026,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>342.5</v>
+        <v>278.2</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>42.41</v>
+        <v>41.06</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>41.15</v>
+        <v>36.44</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>52</v>
+        <v>33.58</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -2090,22 +2050,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>415.25</v>
+        <v>1795</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>40.91</v>
+        <v>38.37</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>44.86</v>
+        <v>45.43</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>56.99</v>
+        <v>52.72</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -2114,22 +2074,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1238</v>
+        <v>535.85</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>40.05</v>
+        <v>38.06</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>44.14</v>
+        <v>32.16</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>53.22</v>
+        <v>36.07</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -2138,22 +2098,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>540</v>
+        <v>236.4</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>39.6</v>
+        <v>36.41</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>32.84</v>
+        <v>40.02</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>36.41</v>
+        <v>49.52</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -2162,22 +2122,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>238.85</v>
+        <v>1217.4</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>39.32</v>
+        <v>36.1</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>41.06</v>
+        <v>41.92</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>50.15</v>
+        <v>52.07</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -2186,22 +2146,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1172</v>
+        <v>407.1</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>38.91</v>
+        <v>34.34</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>40.83</v>
+        <v>42.04</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>47.23</v>
+        <v>55.14</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2210,22 +2170,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>1693.5</v>
+        <v>727</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>35.19</v>
+        <v>33.96</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>52.19</v>
+        <v>35.59</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>61.4</v>
+        <v>40.25</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2234,16 +2194,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>731</v>
+        <v>1008.6</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>34.5</v>
+        <v>31.17</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>36.16</v>
+        <v>44.43</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>40.53</v>
+        <v>50.78</v>
       </c>
     </row>
     <row r="51">
@@ -2258,16 +2218,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>271.6</v>
+        <v>266.6</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>32.84</v>
+        <v>30.05</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>39.12</v>
+        <v>36.44</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>49.81</v>
+        <v>48.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-08-22
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,31 +546,31 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>8100</v>
+        <v>328</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>68.88</v>
+        <v>69.53</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>65.59</v>
+        <v>68.17</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>69.5</v>
+        <v>66.01000000000001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>30.8</v>
+        <v>38.8</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>7254.36</v>
+        <v>277.7</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>7107.57</v>
+        <v>276.21</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>537863</v>
+        <v>31386238</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>221443</v>
+        <v>301937</v>
       </c>
     </row>
     <row r="3">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>5056.2</v>
+        <v>5086.1</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>68.55</v>
+        <v>69.13</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>71.68000000000001</v>
+        <v>72.23</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>68.20999999999999</v>
+        <v>68.48</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>52.48</v>
+        <v>52.06</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4345.35</v>
+        <v>4392.15</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>4240.96</v>
+        <v>4282.33</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>1023022</v>
+        <v>851335</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>448643</v>
+        <v>451296</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>11700</v>
+        <v>8042</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>66.65000000000001</v>
+        <v>63.22</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>73.20999999999999</v>
+        <v>64.06</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>68.02</v>
+        <v>69.17</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>55.74</v>
+        <v>34.96</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>10082.73</v>
+        <v>7304.81</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>9871.610000000001</v>
+        <v>7153.89</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>417529</v>
+        <v>495308</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>321520</v>
+        <v>219892</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>318.5</v>
+        <v>11700</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>65.04000000000001</v>
+        <v>62.91</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>65.98999999999999</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>64.72</v>
+        <v>68.02</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>37.58</v>
+        <v>54.07</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>274.64</v>
+        <v>10186.02</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>273.86</v>
+        <v>9960.559999999999</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>33568779</v>
+        <v>410254</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>293192</v>
+        <v>321256</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1632.8</v>
+        <v>1130</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>62.46</v>
+        <v>60.96</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>63.19</v>
+        <v>65.7</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>58.33</v>
+        <v>71.39</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>30.07</v>
+        <v>21.38</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1480.79</v>
+        <v>986.88</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1475.96</v>
+        <v>954.4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2956849</v>
+        <v>5018614</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>144641</v>
+        <v>265883</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,37 +741,37 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1122</v>
+        <v>3308</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>60.44</v>
+        <v>59.7</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>65.06999999999999</v>
+        <v>65.93000000000001</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>71.13</v>
+        <v>68.13</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>21.63</v>
+        <v>25.83</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>977.7</v>
+        <v>3007.1</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>945.61</v>
+        <v>2959.36</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>5456958</v>
+        <v>804541</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>264005</v>
+        <v>224366</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -780,187 +780,31 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3248.7</v>
+        <v>8693</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>54.91</v>
+        <v>45.18</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>63.66</v>
+        <v>61.69</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>67.04000000000001</v>
+        <v>65.86</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>24.7</v>
+        <v>21.97</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2987.94</v>
+        <v>8206.190000000001</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2941.65</v>
+        <v>8048.12</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>685853</v>
+        <v>356988</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>220344</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>APOLLOHOSP</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>8920.5</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>54.75</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>70.40000000000001</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>69.11</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>22.11</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>8167.47</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>8009.77</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>354479</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>128263</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>BAJFINANCE</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>1087</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>60.79</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>60.86</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>24.92</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>979.6900000000001</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>966.91</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>9224734</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>676213</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>SUNPHARMA</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>1930</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>47.16</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>60.77</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>61.88</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>25.16</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>1825.96</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>1803.25</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>2339607</v>
-      </c>
-      <c r="K11" s="4" t="n">
-        <v>463072</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>ICICIBANK</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>1406.8</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>46.92</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>61.24</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>61.72</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>20.54</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>1350.71</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>1346.5</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>12083442</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>1016453</v>
+        <v>124992</v>
       </c>
     </row>
   </sheetData>
@@ -972,10 +816,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1033,7 +873,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1042,22 +882,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1370</v>
+        <v>328</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>70.53</v>
+        <v>69.53</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>58.07</v>
+        <v>68.17</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>49.91</v>
+        <v>66.01000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1066,22 +906,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>8100</v>
+        <v>5086.1</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>68.88</v>
+        <v>69.13</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>65.59</v>
+        <v>72.23</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>69.5</v>
+        <v>68.48</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1090,16 +930,16 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>5056.2</v>
+        <v>8042</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>68.55</v>
+        <v>63.22</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>71.68000000000001</v>
+        <v>64.06</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>68.20999999999999</v>
+        <v>69.17</v>
       </c>
     </row>
     <row r="5">
@@ -1117,7 +957,7 @@
         <v>11700</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>66.65000000000001</v>
+        <v>62.91</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>73.20999999999999</v>
@@ -1129,7 +969,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1138,22 +978,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>318.5</v>
+        <v>402.8</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>65.04000000000001</v>
+        <v>62.21</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>65.98999999999999</v>
+        <v>54.56</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>64.72</v>
+        <v>52.93</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1162,22 +1002,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1992.1</v>
+        <v>2032.5</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>63.13</v>
+        <v>61.18</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>59.67</v>
+        <v>61.08</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>64.45</v>
+        <v>57.64</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1186,22 +1026,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1632.8</v>
+        <v>1130</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>62.46</v>
+        <v>60.96</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>63.19</v>
+        <v>65.7</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>58.33</v>
+        <v>71.39</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1210,22 +1050,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2025</v>
+        <v>414</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>60.5</v>
+        <v>60.83</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>59.7</v>
+        <v>50.12</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>56.63</v>
+        <v>60.32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1234,22 +1074,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1122</v>
+        <v>4093</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>60.44</v>
+        <v>60.35</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>65.06999999999999</v>
+        <v>55.41</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>71.13</v>
+        <v>58.49</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1258,22 +1098,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3428.2</v>
+        <v>3308</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>60.05</v>
+        <v>59.7</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>58.75</v>
+        <v>65.93000000000001</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>62.4</v>
+        <v>68.13</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1282,22 +1122,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>410.8</v>
+        <v>3412.2</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>58.74</v>
+        <v>57.13</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>49.02</v>
+        <v>57.93</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>59.92</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1306,22 +1146,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1169.2</v>
+        <v>1293.7</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>58.65</v>
+        <v>55.95</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>47.65</v>
+        <v>59.84</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>41.14</v>
+        <v>65.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1330,22 +1170,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>4057</v>
+        <v>1095</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>58.64</v>
+        <v>55.13</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>54.22</v>
+        <v>61.44</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>57.93</v>
+        <v>61.38</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1354,22 +1194,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1067.7</v>
+        <v>554.8</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>56.21</v>
+        <v>54.59</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>56.69</v>
+        <v>38.49</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>62.49</v>
+        <v>38.05</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1378,22 +1218,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1506.9</v>
+        <v>1029.85</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>56.07</v>
+        <v>54.16</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>64.06</v>
+        <v>57.55</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>64.58</v>
+        <v>64.39</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1402,22 +1242,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1029.5</v>
+        <v>1946</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>55.84</v>
+        <v>52.77</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>57.07</v>
+        <v>54.77</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>64.20999999999999</v>
+        <v>62.07</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1426,22 +1266,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>184</v>
+        <v>1316</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>54.92</v>
+        <v>52.27</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>42.38</v>
+        <v>46.01</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>40.59</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1450,22 +1290,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>3248.7</v>
+        <v>1420</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>54.91</v>
+        <v>51.78</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>63.66</v>
+        <v>61.63</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>67.04000000000001</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1474,22 +1314,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>8920.5</v>
+        <v>1302.5</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>54.75</v>
+        <v>50.37</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>70.40000000000001</v>
+        <v>51.99</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>69.11</v>
+        <v>47.84</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1498,22 +1338,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1087</v>
+        <v>1048.7</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>53.8</v>
+        <v>49.43</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>60.79</v>
+        <v>53.62</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>60.86</v>
+        <v>61.55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1522,22 +1362,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>5310</v>
+        <v>1477.1</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>53.35</v>
+        <v>49.22</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>58.65</v>
+        <v>60.66</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>57.48</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1546,22 +1386,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>2361</v>
+        <v>180.79</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>53.16</v>
+        <v>48.78</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>48.04</v>
+        <v>40.37</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>38.99</v>
+        <v>39.87</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1570,22 +1410,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1206</v>
+        <v>1584</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>51.22</v>
+        <v>48.62</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>44.52</v>
+        <v>58.21</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>48.97</v>
+        <v>56.29</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1594,22 +1434,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>391.15</v>
+        <v>2302</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>51.15</v>
+        <v>48.3</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>49.5</v>
+        <v>45.16</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>50.48</v>
+        <v>38.09</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1618,22 +1458,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>13834</v>
+        <v>1245.8</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>51.05</v>
+        <v>47.65</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>51.03</v>
+        <v>45.96</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>54.28</v>
+        <v>53.62</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1642,22 +1482,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1310</v>
+        <v>1121</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>50.79</v>
+        <v>47.14</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>45.12</v>
+        <v>43.54</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>47.2</v>
+        <v>38.78</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1666,22 +1506,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1450</v>
+        <v>11570</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>50.72</v>
+        <v>45.96</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>57.16</v>
+        <v>50.85</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>53.59</v>
+        <v>54.14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1690,22 +1530,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>249.05</v>
+        <v>1432.2</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>50.56</v>
+        <v>45.91</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>49.71</v>
+        <v>54.48</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>45.55</v>
+        <v>52.46</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1714,22 +1554,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>3035.1</v>
+        <v>272.4</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>49.78</v>
+        <v>45.89</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>64.56999999999999</v>
+        <v>41.39</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>58.94</v>
+        <v>50.01</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1738,22 +1578,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1270</v>
+        <v>244</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>49.55</v>
+        <v>45.49</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>56.51</v>
+        <v>46.75</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>64.02</v>
+        <v>44.59</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1762,22 +1602,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>11706</v>
+        <v>8693</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>48.8</v>
+        <v>45.18</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>51.59</v>
+        <v>61.69</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>54.51</v>
+        <v>65.86</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1786,22 +1626,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>2978</v>
+        <v>2994.9</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>47.59</v>
+        <v>45.15</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>48.41</v>
+        <v>62.28</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>42.17</v>
+        <v>58.33</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1810,22 +1650,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1930</v>
+        <v>5165</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>47.16</v>
+        <v>45.01</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>60.77</v>
+        <v>53.47</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>61.88</v>
+        <v>55.4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1834,22 +1674,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1406.8</v>
+        <v>1700</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>46.92</v>
+        <v>44.54</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>61.24</v>
+        <v>52.76</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>61.72</v>
+        <v>61.64</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1858,22 +1698,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1079.5</v>
+        <v>340</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>46.4</v>
+        <v>44.53</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>43.28</v>
+        <v>40.13</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>51.16</v>
+        <v>51.4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1882,22 +1722,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2696.3</v>
+        <v>1904</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>45.7</v>
+        <v>43.5</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>56.6</v>
+        <v>57.24</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>53.03</v>
+        <v>60.43</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1906,22 +1746,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>2077</v>
+        <v>1174.7</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>44.75</v>
+        <v>43.2</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>38.64</v>
+        <v>41.97</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>42.38</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1930,22 +1770,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>334.5</v>
+        <v>13565</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>43.44</v>
+        <v>42.76</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>41.64</v>
+        <v>48.18</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>36.23</v>
+        <v>52.87</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1954,22 +1794,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1700</v>
+        <v>2924</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>42.52</v>
+        <v>42.33</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>52.76</v>
+        <v>46.84</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>61.64</v>
+        <v>41.78</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1978,22 +1818,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>184.85</v>
+        <v>1792.9</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>42.28</v>
+        <v>40.46</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>43.58</v>
+        <v>45.29</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>56.09</v>
+        <v>52.62</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -2002,22 +1842,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>340</v>
+        <v>183</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>42.27</v>
+        <v>40.3</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>40.13</v>
+        <v>43.2</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>51.4</v>
+        <v>55.9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -2026,22 +1866,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>278.2</v>
+        <v>1049</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>41.06</v>
+        <v>39.91</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>36.44</v>
+        <v>38.57</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>33.58</v>
+        <v>49.05</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -2050,22 +1890,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1795</v>
+        <v>2640</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>38.37</v>
+        <v>39.6</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>45.43</v>
+        <v>52.56</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>52.72</v>
+        <v>51.68</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -2074,22 +1914,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>535.85</v>
+        <v>236.4</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>38.06</v>
+        <v>38.85</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>32.16</v>
+        <v>40.02</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>36.07</v>
+        <v>49.52</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -2098,22 +1938,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>236.4</v>
+        <v>2028</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>36.41</v>
+        <v>38.76</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>40.02</v>
+        <v>34.13</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>49.52</v>
+        <v>40.59</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -2122,22 +1962,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1217.4</v>
+        <v>405.2</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>36.1</v>
+        <v>38.17</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>41.92</v>
+        <v>41.38</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>52.07</v>
+        <v>54.71</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -2146,22 +1986,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>407.1</v>
+        <v>726.95</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>34.34</v>
+        <v>37.81</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>42.04</v>
+        <v>35.58</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>55.14</v>
+        <v>40.24</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2170,22 +2010,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>727</v>
+        <v>269.4</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>33.96</v>
+        <v>35.37</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>35.59</v>
+        <v>32.62</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>40.25</v>
+        <v>32.19</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2194,22 +2034,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1008.6</v>
+        <v>317.9</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>31.17</v>
+        <v>33.17</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>44.43</v>
+        <v>37.79</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>50.78</v>
+        <v>35.36</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2218,16 +2058,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>266.6</v>
+        <v>1000</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>30.05</v>
+        <v>32.56</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>36.44</v>
+        <v>43.53</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>48.45</v>
+        <v>50.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>